<commit_message>
wip mobilisasi lanjutan, malnutrisi lanjutan, depresi lanjutan
</commit_message>
<xml_diff>
--- a/dataset/lansia.xlsx
+++ b/dataset/lansia.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/macbokprom12021/PycharmProjects/CKG-Helper/dataset/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{696D3EC9-8FA8-2440-9CCC-A5FA84CDC6CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F8705F7F-7607-0C46-A1D9-828030FBE96D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4480" yWindow="-21000" windowWidth="36000" windowHeight="19540" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -403,7 +403,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="DJ1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00001A000000}">
+    <comment ref="DV1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00001A000000}">
       <text>
         <r>
           <rPr>
@@ -418,7 +418,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="DM1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00001B000000}">
+    <comment ref="DY1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00001B000000}">
       <text>
         <r>
           <rPr>
@@ -433,7 +433,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="DR1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00001C000000}">
+    <comment ref="ED1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00001C000000}">
       <text>
         <r>
           <rPr>
@@ -448,7 +448,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="DU1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00001D000000}">
+    <comment ref="EG1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00001D000000}">
       <text>
         <r>
           <rPr>
@@ -463,7 +463,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="EB1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00001E000000}">
+    <comment ref="EN1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00001E000000}">
       <text>
         <r>
           <rPr>
@@ -478,7 +478,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="ED1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00001F000000}">
+    <comment ref="EP1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00001F000000}">
       <text>
         <r>
           <rPr>
@@ -493,7 +493,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="EE1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000020000000}">
+    <comment ref="EQ1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000020000000}">
       <text>
         <r>
           <rPr>
@@ -508,7 +508,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="EF1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000021000000}">
+    <comment ref="ER1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000021000000}">
       <text>
         <r>
           <rPr>
@@ -523,7 +523,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="EG1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000022000000}">
+    <comment ref="ES1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000022000000}">
       <text>
         <r>
           <rPr>
@@ -538,7 +538,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="EQ1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000023000000}">
+    <comment ref="FC1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000023000000}">
       <text>
         <r>
           <rPr>
@@ -553,7 +553,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="FI1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000024000000}">
+    <comment ref="FU1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000024000000}">
       <text>
         <r>
           <rPr>
@@ -568,7 +568,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="FS1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000025000000}">
+    <comment ref="GE1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000025000000}">
       <text>
         <r>
           <rPr>
@@ -583,7 +583,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="FT1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000026000000}">
+    <comment ref="GF1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000026000000}">
       <text>
         <r>
           <rPr>
@@ -598,7 +598,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="FV1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000027000000}">
+    <comment ref="GH1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000027000000}">
       <text>
         <r>
           <rPr>
@@ -613,7 +613,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="FW1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000028000000}">
+    <comment ref="GI1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000028000000}">
       <text>
         <r>
           <rPr>
@@ -628,7 +628,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="FX1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000029000000}">
+    <comment ref="GJ1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000029000000}">
       <text>
         <r>
           <rPr>
@@ -643,7 +643,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="FY1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00002A000000}">
+    <comment ref="GK1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00002A000000}">
       <text>
         <r>
           <rPr>
@@ -658,7 +658,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="GU1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00002B000000}">
+    <comment ref="HG1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00002B000000}">
       <text>
         <r>
           <rPr>
@@ -673,7 +673,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="GV1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00002C000000}">
+    <comment ref="HH1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00002C000000}">
       <text>
         <r>
           <rPr>
@@ -688,7 +688,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="GW1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00002D000000}">
+    <comment ref="HI1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00002D000000}">
       <text>
         <r>
           <rPr>
@@ -708,7 +708,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="393" uniqueCount="287">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="417" uniqueCount="308">
   <si>
     <t>batas_awal</t>
   </si>
@@ -1569,6 +1569,69 @@
   </si>
   <si>
     <t>Tidak Berubah</t>
+  </si>
+  <si>
+    <t>sppb_1</t>
+  </si>
+  <si>
+    <t>sppb_2</t>
+  </si>
+  <si>
+    <t>sppb_3</t>
+  </si>
+  <si>
+    <t>sppb_4</t>
+  </si>
+  <si>
+    <t>sppb_5</t>
+  </si>
+  <si>
+    <t>Bertahan 10 detik</t>
+  </si>
+  <si>
+    <t>4.83 - 6.20 detik</t>
+  </si>
+  <si>
+    <t>&lt;11.19 detik</t>
+  </si>
+  <si>
+    <t>mna_sf_1</t>
+  </si>
+  <si>
+    <t>mna_sf_2</t>
+  </si>
+  <si>
+    <t>mna_sf_3</t>
+  </si>
+  <si>
+    <t>mna_sf_4</t>
+  </si>
+  <si>
+    <t>mna_sf_5</t>
+  </si>
+  <si>
+    <t>mna_sf_6</t>
+  </si>
+  <si>
+    <t>mna_sf_7</t>
+  </si>
+  <si>
+    <t>Nafsu Makan Yang Sangat Berkurang</t>
+  </si>
+  <si>
+    <t>Penurunan BB &gt; 3 Kg</t>
+  </si>
+  <si>
+    <t>Harus berbaring di tempat tidur atau menggunakan kursi roda</t>
+  </si>
+  <si>
+    <t>Dementia atau depresi berat</t>
+  </si>
+  <si>
+    <t>IMT &lt;19</t>
+  </si>
+  <si>
+    <t>&lt;31 cm</t>
   </si>
 </sst>
 </file>
@@ -1971,7 +2034,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:HM2"/>
+  <dimension ref="A1:HY2"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="17.5" style="1" bestFit="1" customWidth="1"/>
@@ -2066,108 +2129,108 @@
     <col min="97" max="97" width="10.5" style="1" bestFit="1" customWidth="1"/>
     <col min="98" max="98" width="15.83203125" style="1" bestFit="1" customWidth="1"/>
     <col min="99" max="102" width="15.83203125" style="1" customWidth="1"/>
-    <col min="103" max="106" width="10.5" style="1" customWidth="1"/>
-    <col min="107" max="107" width="16" style="1" bestFit="1" customWidth="1"/>
-    <col min="108" max="108" width="25" style="1" bestFit="1" customWidth="1"/>
-    <col min="109" max="109" width="8.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="110" max="110" width="19.6640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="111" max="111" width="17.1640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="112" max="112" width="23.5" style="1" bestFit="1" customWidth="1"/>
-    <col min="113" max="113" width="14.83203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="114" max="114" width="14.83203125" style="1" customWidth="1"/>
-    <col min="115" max="115" width="10.5" style="1" bestFit="1" customWidth="1"/>
-    <col min="116" max="116" width="21.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="117" max="117" width="11.6640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="118" max="118" width="22.83203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="119" max="119" width="22.83203125" style="1" customWidth="1"/>
-    <col min="120" max="120" width="16.1640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="121" max="121" width="16.1640625" style="1" customWidth="1"/>
-    <col min="122" max="122" width="19.83203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="123" max="123" width="12.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="124" max="125" width="12.33203125" style="1" customWidth="1"/>
-    <col min="126" max="126" width="14.1640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="127" max="127" width="14.1640625" style="1" customWidth="1"/>
-    <col min="128" max="128" width="18.83203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="129" max="129" width="23.6640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="130" max="130" width="23.6640625" style="1" customWidth="1"/>
-    <col min="131" max="131" width="26" style="1" bestFit="1" customWidth="1"/>
-    <col min="132" max="132" width="26" style="1" customWidth="1"/>
-    <col min="133" max="133" width="36.1640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="134" max="134" width="41.5" style="1" bestFit="1" customWidth="1"/>
-    <col min="135" max="135" width="29" style="1" bestFit="1" customWidth="1"/>
-    <col min="136" max="136" width="20.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="137" max="137" width="9.83203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="138" max="139" width="12.83203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="140" max="141" width="12.83203125" style="1" customWidth="1"/>
-    <col min="142" max="142" width="17.5" style="1" bestFit="1" customWidth="1"/>
-    <col min="143" max="143" width="18.5" style="1" bestFit="1" customWidth="1"/>
-    <col min="144" max="144" width="17.5" style="1" customWidth="1"/>
-    <col min="145" max="145" width="11.83203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="146" max="146" width="13" style="1" bestFit="1" customWidth="1"/>
-    <col min="147" max="147" width="19.5" style="1" bestFit="1" customWidth="1"/>
-    <col min="148" max="148" width="12.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="149" max="151" width="19.5" style="1" customWidth="1"/>
-    <col min="152" max="152" width="9.83203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="153" max="153" width="9.83203125" style="1" customWidth="1"/>
-    <col min="154" max="154" width="11.5" style="1" bestFit="1" customWidth="1"/>
-    <col min="155" max="158" width="11.5" style="1" customWidth="1"/>
-    <col min="159" max="159" width="13.83203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="160" max="160" width="4.5" style="1" bestFit="1" customWidth="1"/>
-    <col min="161" max="161" width="9" style="1" bestFit="1" customWidth="1"/>
-    <col min="162" max="162" width="15.1640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="163" max="163" width="16.1640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="164" max="164" width="18.1640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="165" max="165" width="18.1640625" style="1" customWidth="1"/>
-    <col min="166" max="166" width="18.1640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="167" max="167" width="8.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="168" max="170" width="8.33203125" style="1" customWidth="1"/>
-    <col min="171" max="171" width="22" style="1" bestFit="1" customWidth="1"/>
-    <col min="172" max="172" width="7.6640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="173" max="173" width="12.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="174" max="174" width="20.5" style="1" bestFit="1" customWidth="1"/>
-    <col min="175" max="175" width="12.1640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="176" max="176" width="17.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="177" max="177" width="20.5" style="1" customWidth="1"/>
-    <col min="178" max="180" width="6.83203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="181" max="181" width="17.1640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="182" max="183" width="17.1640625" style="1" customWidth="1"/>
-    <col min="184" max="184" width="14" style="1" bestFit="1" customWidth="1"/>
-    <col min="185" max="185" width="14" style="1" customWidth="1"/>
-    <col min="186" max="186" width="15.5" style="1" bestFit="1" customWidth="1"/>
-    <col min="187" max="187" width="18.1640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="188" max="188" width="18.1640625" style="1" customWidth="1"/>
-    <col min="189" max="189" width="17.6640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="190" max="190" width="11.83203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="191" max="191" width="18.1640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="192" max="194" width="18.1640625" style="1" customWidth="1"/>
-    <col min="195" max="195" width="46.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="196" max="196" width="35" style="1" bestFit="1" customWidth="1"/>
-    <col min="197" max="197" width="43.1640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="198" max="198" width="18.1640625" style="1" customWidth="1"/>
-    <col min="199" max="199" width="9.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="200" max="200" width="10.6640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="201" max="201" width="10.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="202" max="203" width="10.33203125" style="1" customWidth="1"/>
-    <col min="204" max="204" width="11.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="205" max="205" width="10.33203125" style="1" customWidth="1"/>
-    <col min="206" max="206" width="12.1640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="207" max="207" width="14.5" style="1" bestFit="1" customWidth="1"/>
-    <col min="208" max="208" width="16" style="1" bestFit="1" customWidth="1"/>
-    <col min="209" max="209" width="21" style="1" bestFit="1" customWidth="1"/>
-    <col min="210" max="210" width="23.6640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="211" max="211" width="13.6640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="212" max="212" width="20.5" style="1" bestFit="1" customWidth="1"/>
-    <col min="213" max="213" width="18" style="1" bestFit="1" customWidth="1"/>
-    <col min="214" max="214" width="15.5" style="1" bestFit="1" customWidth="1"/>
-    <col min="215" max="215" width="21.83203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="216" max="216" width="21.1640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="217" max="218" width="10.83203125" style="1"/>
-    <col min="219" max="219" width="24.83203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="220" max="220" width="29.1640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="221" max="16384" width="10.83203125" style="1"/>
+    <col min="103" max="118" width="10.5" style="1" customWidth="1"/>
+    <col min="119" max="119" width="16" style="1" bestFit="1" customWidth="1"/>
+    <col min="120" max="120" width="25" style="1" bestFit="1" customWidth="1"/>
+    <col min="121" max="121" width="8.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="122" max="122" width="19.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="123" max="123" width="17.1640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="124" max="124" width="23.5" style="1" bestFit="1" customWidth="1"/>
+    <col min="125" max="125" width="14.83203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="126" max="126" width="14.83203125" style="1" customWidth="1"/>
+    <col min="127" max="127" width="10.5" style="1" bestFit="1" customWidth="1"/>
+    <col min="128" max="128" width="21.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="129" max="129" width="11.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="130" max="130" width="22.83203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="131" max="131" width="22.83203125" style="1" customWidth="1"/>
+    <col min="132" max="132" width="16.1640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="133" max="133" width="16.1640625" style="1" customWidth="1"/>
+    <col min="134" max="134" width="19.83203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="135" max="135" width="12.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="136" max="137" width="12.33203125" style="1" customWidth="1"/>
+    <col min="138" max="138" width="14.1640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="139" max="139" width="14.1640625" style="1" customWidth="1"/>
+    <col min="140" max="140" width="18.83203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="141" max="141" width="23.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="142" max="142" width="23.6640625" style="1" customWidth="1"/>
+    <col min="143" max="143" width="26" style="1" bestFit="1" customWidth="1"/>
+    <col min="144" max="144" width="26" style="1" customWidth="1"/>
+    <col min="145" max="145" width="36.1640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="146" max="146" width="41.5" style="1" bestFit="1" customWidth="1"/>
+    <col min="147" max="147" width="29" style="1" bestFit="1" customWidth="1"/>
+    <col min="148" max="148" width="20.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="149" max="149" width="9.83203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="150" max="151" width="12.83203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="152" max="153" width="12.83203125" style="1" customWidth="1"/>
+    <col min="154" max="154" width="17.5" style="1" bestFit="1" customWidth="1"/>
+    <col min="155" max="155" width="18.5" style="1" bestFit="1" customWidth="1"/>
+    <col min="156" max="156" width="17.5" style="1" customWidth="1"/>
+    <col min="157" max="157" width="11.83203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="158" max="158" width="13" style="1" bestFit="1" customWidth="1"/>
+    <col min="159" max="159" width="19.5" style="1" bestFit="1" customWidth="1"/>
+    <col min="160" max="160" width="12.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="161" max="163" width="19.5" style="1" customWidth="1"/>
+    <col min="164" max="164" width="9.83203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="165" max="165" width="9.83203125" style="1" customWidth="1"/>
+    <col min="166" max="166" width="11.5" style="1" bestFit="1" customWidth="1"/>
+    <col min="167" max="170" width="11.5" style="1" customWidth="1"/>
+    <col min="171" max="171" width="13.83203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="172" max="172" width="4.5" style="1" bestFit="1" customWidth="1"/>
+    <col min="173" max="173" width="9" style="1" bestFit="1" customWidth="1"/>
+    <col min="174" max="174" width="15.1640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="175" max="175" width="16.1640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="176" max="176" width="18.1640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="177" max="177" width="18.1640625" style="1" customWidth="1"/>
+    <col min="178" max="178" width="18.1640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="179" max="179" width="8.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="180" max="182" width="8.33203125" style="1" customWidth="1"/>
+    <col min="183" max="183" width="22" style="1" bestFit="1" customWidth="1"/>
+    <col min="184" max="184" width="7.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="185" max="185" width="12.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="186" max="186" width="20.5" style="1" bestFit="1" customWidth="1"/>
+    <col min="187" max="187" width="12.1640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="188" max="188" width="17.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="189" max="189" width="20.5" style="1" customWidth="1"/>
+    <col min="190" max="192" width="6.83203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="193" max="193" width="17.1640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="194" max="195" width="17.1640625" style="1" customWidth="1"/>
+    <col min="196" max="196" width="14" style="1" bestFit="1" customWidth="1"/>
+    <col min="197" max="197" width="14" style="1" customWidth="1"/>
+    <col min="198" max="198" width="15.5" style="1" bestFit="1" customWidth="1"/>
+    <col min="199" max="199" width="18.1640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="200" max="200" width="18.1640625" style="1" customWidth="1"/>
+    <col min="201" max="201" width="17.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="202" max="202" width="11.83203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="203" max="203" width="18.1640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="204" max="206" width="18.1640625" style="1" customWidth="1"/>
+    <col min="207" max="207" width="46.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="208" max="208" width="35" style="1" bestFit="1" customWidth="1"/>
+    <col min="209" max="209" width="43.1640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="210" max="210" width="18.1640625" style="1" customWidth="1"/>
+    <col min="211" max="211" width="9.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="212" max="212" width="10.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="213" max="213" width="10.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="214" max="215" width="10.33203125" style="1" customWidth="1"/>
+    <col min="216" max="216" width="11.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="217" max="217" width="10.33203125" style="1" customWidth="1"/>
+    <col min="218" max="218" width="12.1640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="219" max="219" width="14.5" style="1" bestFit="1" customWidth="1"/>
+    <col min="220" max="220" width="16" style="1" bestFit="1" customWidth="1"/>
+    <col min="221" max="221" width="21" style="1" bestFit="1" customWidth="1"/>
+    <col min="222" max="222" width="23.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="223" max="223" width="13.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="224" max="224" width="20.5" style="1" bestFit="1" customWidth="1"/>
+    <col min="225" max="225" width="18" style="1" bestFit="1" customWidth="1"/>
+    <col min="226" max="226" width="15.5" style="1" bestFit="1" customWidth="1"/>
+    <col min="227" max="227" width="21.83203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="228" max="228" width="21.1640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="229" max="230" width="10.83203125" style="1"/>
+    <col min="231" max="231" width="24.83203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="232" max="232" width="29.1640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="233" max="16384" width="10.83203125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:221" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:233" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2484,313 +2547,349 @@
         <v>283</v>
       </c>
       <c r="DC1" s="1" t="s">
+        <v>287</v>
+      </c>
+      <c r="DD1" s="1" t="s">
+        <v>288</v>
+      </c>
+      <c r="DE1" s="1" t="s">
+        <v>289</v>
+      </c>
+      <c r="DF1" s="1" t="s">
+        <v>290</v>
+      </c>
+      <c r="DG1" s="1" t="s">
+        <v>291</v>
+      </c>
+      <c r="DH1" s="1" t="s">
+        <v>295</v>
+      </c>
+      <c r="DI1" s="1" t="s">
+        <v>296</v>
+      </c>
+      <c r="DJ1" s="1" t="s">
+        <v>297</v>
+      </c>
+      <c r="DK1" s="1" t="s">
+        <v>298</v>
+      </c>
+      <c r="DL1" s="1" t="s">
+        <v>299</v>
+      </c>
+      <c r="DM1" s="1" t="s">
+        <v>300</v>
+      </c>
+      <c r="DN1" s="1" t="s">
+        <v>301</v>
+      </c>
+      <c r="DO1" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="DD1" s="1" t="s">
+      <c r="DP1" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="DE1" s="1" t="s">
+      <c r="DQ1" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="DF1" s="1" t="s">
+      <c r="DR1" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="DG1" s="1" t="s">
+      <c r="DS1" s="1" t="s">
         <v>79</v>
       </c>
-      <c r="DH1" s="1" t="s">
+      <c r="DT1" s="1" t="s">
         <v>80</v>
       </c>
-      <c r="DI1" s="1" t="s">
+      <c r="DU1" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="DJ1" s="1" t="s">
+      <c r="DV1" s="1" t="s">
         <v>82</v>
       </c>
-      <c r="DK1" s="1" t="s">
+      <c r="DW1" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="DL1" s="1" t="s">
+      <c r="DX1" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="DM1" s="1" t="s">
+      <c r="DY1" s="1" t="s">
         <v>85</v>
       </c>
-      <c r="DN1" s="1" t="s">
+      <c r="DZ1" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="DO1" s="1" t="s">
+      <c r="EA1" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="DP1" s="1" t="s">
+      <c r="EB1" s="1" t="s">
         <v>88</v>
       </c>
-      <c r="DQ1" s="1" t="s">
+      <c r="EC1" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="DR1" s="1" t="s">
+      <c r="ED1" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="DS1" s="1" t="s">
+      <c r="EE1" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="DT1" s="1" t="s">
+      <c r="EF1" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="DU1" s="1" t="s">
+      <c r="EG1" s="1" t="s">
         <v>93</v>
       </c>
-      <c r="DV1" s="1" t="s">
+      <c r="EH1" s="1" t="s">
         <v>94</v>
       </c>
-      <c r="DW1" s="1" t="s">
+      <c r="EI1" s="1" t="s">
         <v>95</v>
       </c>
-      <c r="DX1" s="1" t="s">
+      <c r="EJ1" s="1" t="s">
         <v>96</v>
       </c>
-      <c r="DY1" s="1" t="s">
+      <c r="EK1" s="1" t="s">
         <v>97</v>
       </c>
-      <c r="DZ1" s="1" t="s">
+      <c r="EL1" s="1" t="s">
         <v>98</v>
       </c>
-      <c r="EA1" s="1" t="s">
+      <c r="EM1" s="1" t="s">
         <v>99</v>
       </c>
-      <c r="EB1" s="1" t="s">
+      <c r="EN1" s="1" t="s">
         <v>100</v>
       </c>
-      <c r="EC1" s="1" t="s">
+      <c r="EO1" s="1" t="s">
         <v>101</v>
       </c>
-      <c r="ED1" s="1" t="s">
+      <c r="EP1" s="1" t="s">
         <v>102</v>
       </c>
-      <c r="EE1" s="1" t="s">
+      <c r="EQ1" s="1" t="s">
         <v>103</v>
       </c>
-      <c r="EF1" s="1" t="s">
+      <c r="ER1" s="1" t="s">
         <v>104</v>
       </c>
-      <c r="EG1" s="1" t="s">
+      <c r="ES1" s="1" t="s">
         <v>105</v>
       </c>
-      <c r="EH1" s="1" t="s">
+      <c r="ET1" s="1" t="s">
         <v>106</v>
       </c>
-      <c r="EI1" s="1" t="s">
+      <c r="EU1" s="1" t="s">
         <v>107</v>
       </c>
-      <c r="EJ1" s="1" t="s">
+      <c r="EV1" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="EK1" s="1" t="s">
+      <c r="EW1" s="1" t="s">
         <v>109</v>
       </c>
-      <c r="EL1" s="1" t="s">
+      <c r="EX1" s="1" t="s">
         <v>110</v>
       </c>
-      <c r="EM1" s="1" t="s">
+      <c r="EY1" s="1" t="s">
         <v>111</v>
       </c>
-      <c r="EN1" s="1" t="s">
+      <c r="EZ1" s="1" t="s">
         <v>112</v>
       </c>
-      <c r="EO1" s="1" t="s">
+      <c r="FA1" s="1" t="s">
         <v>113</v>
       </c>
-      <c r="EP1" s="1" t="s">
+      <c r="FB1" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="EQ1" s="1" t="s">
+      <c r="FC1" s="1" t="s">
         <v>115</v>
       </c>
-      <c r="ER1" s="1" t="s">
+      <c r="FD1" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="ES1" s="1" t="s">
+      <c r="FE1" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="ET1" s="1" t="s">
+      <c r="FF1" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="EU1" s="1" t="s">
+      <c r="FG1" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="EV1" s="1" t="s">
+      <c r="FH1" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="EW1" s="1" t="s">
+      <c r="FI1" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="EX1" s="1" t="s">
+      <c r="FJ1" s="1" t="s">
         <v>122</v>
       </c>
-      <c r="EY1" s="1" t="s">
+      <c r="FK1" s="1" t="s">
         <v>123</v>
       </c>
-      <c r="EZ1" s="1" t="s">
+      <c r="FL1" s="1" t="s">
         <v>124</v>
       </c>
-      <c r="FA1" s="1" t="s">
+      <c r="FM1" s="1" t="s">
         <v>125</v>
       </c>
-      <c r="FB1" s="1" t="s">
+      <c r="FN1" s="1" t="s">
         <v>126</v>
       </c>
-      <c r="FC1" s="1" t="s">
+      <c r="FO1" s="1" t="s">
         <v>127</v>
       </c>
-      <c r="FD1" s="1" t="s">
+      <c r="FP1" s="1" t="s">
         <v>128</v>
       </c>
-      <c r="FE1" s="1" t="s">
+      <c r="FQ1" s="1" t="s">
         <v>129</v>
       </c>
-      <c r="FF1" s="1" t="s">
+      <c r="FR1" s="1" t="s">
         <v>130</v>
       </c>
-      <c r="FG1" s="1" t="s">
+      <c r="FS1" s="1" t="s">
         <v>131</v>
       </c>
-      <c r="FH1" s="1" t="s">
+      <c r="FT1" s="1" t="s">
         <v>132</v>
       </c>
-      <c r="FI1" s="1" t="s">
+      <c r="FU1" s="1" t="s">
         <v>133</v>
       </c>
-      <c r="FJ1" s="1" t="s">
+      <c r="FV1" s="1" t="s">
         <v>134</v>
       </c>
-      <c r="FK1" s="1" t="s">
+      <c r="FW1" s="1" t="s">
         <v>135</v>
       </c>
-      <c r="FL1" s="1" t="s">
+      <c r="FX1" s="1" t="s">
         <v>136</v>
       </c>
-      <c r="FM1" s="1" t="s">
+      <c r="FY1" s="1" t="s">
         <v>137</v>
       </c>
-      <c r="FN1" s="1" t="s">
+      <c r="FZ1" s="1" t="s">
         <v>138</v>
       </c>
-      <c r="FO1" s="1" t="s">
+      <c r="GA1" s="1" t="s">
         <v>139</v>
       </c>
-      <c r="FP1" s="1" t="s">
+      <c r="GB1" s="1" t="s">
         <v>140</v>
       </c>
-      <c r="FQ1" s="1" t="s">
+      <c r="GC1" s="1" t="s">
         <v>141</v>
       </c>
-      <c r="FR1" s="1" t="s">
+      <c r="GD1" s="1" t="s">
         <v>142</v>
       </c>
-      <c r="FS1" s="1" t="s">
+      <c r="GE1" s="1" t="s">
         <v>143</v>
       </c>
-      <c r="FT1" s="1" t="s">
+      <c r="GF1" s="1" t="s">
         <v>144</v>
       </c>
-      <c r="FU1" s="1" t="s">
+      <c r="GG1" s="1" t="s">
         <v>145</v>
       </c>
-      <c r="FV1" s="1" t="s">
+      <c r="GH1" s="1" t="s">
         <v>146</v>
       </c>
-      <c r="FW1" s="1" t="s">
+      <c r="GI1" s="1" t="s">
         <v>147</v>
       </c>
-      <c r="FX1" s="1" t="s">
+      <c r="GJ1" s="1" t="s">
         <v>148</v>
       </c>
-      <c r="FY1" s="1" t="s">
+      <c r="GK1" s="1" t="s">
         <v>149</v>
       </c>
-      <c r="FZ1" s="1" t="s">
+      <c r="GL1" s="1" t="s">
         <v>150</v>
       </c>
-      <c r="GA1" s="1" t="s">
+      <c r="GM1" s="1" t="s">
         <v>151</v>
       </c>
-      <c r="GB1" s="1" t="s">
+      <c r="GN1" s="1" t="s">
         <v>152</v>
       </c>
-      <c r="GC1" s="1" t="s">
+      <c r="GO1" s="1" t="s">
         <v>153</v>
       </c>
-      <c r="GD1" s="1" t="s">
+      <c r="GP1" s="1" t="s">
         <v>154</v>
       </c>
-      <c r="GE1" s="1" t="s">
+      <c r="GQ1" s="1" t="s">
         <v>155</v>
       </c>
-      <c r="GF1" s="1" t="s">
+      <c r="GR1" s="1" t="s">
         <v>156</v>
       </c>
-      <c r="GG1" s="1" t="s">
+      <c r="GS1" s="1" t="s">
         <v>157</v>
       </c>
-      <c r="GH1" s="1" t="s">
+      <c r="GT1" s="1" t="s">
         <v>158</v>
       </c>
-      <c r="GI1" s="1" t="s">
+      <c r="GU1" s="1" t="s">
         <v>159</v>
       </c>
-      <c r="GJ1" s="1" t="s">
+      <c r="GV1" s="1" t="s">
         <v>160</v>
       </c>
-      <c r="GK1" s="1" t="s">
+      <c r="GW1" s="1" t="s">
         <v>161</v>
       </c>
-      <c r="GL1" s="1" t="s">
+      <c r="GX1" s="1" t="s">
         <v>162</v>
       </c>
-      <c r="GM1" s="1" t="s">
+      <c r="GY1" s="1" t="s">
         <v>163</v>
       </c>
-      <c r="GN1" s="1" t="s">
+      <c r="GZ1" s="1" t="s">
         <v>164</v>
       </c>
-      <c r="GO1" s="1" t="s">
+      <c r="HA1" s="1" t="s">
         <v>165</v>
       </c>
-      <c r="GP1" s="1" t="s">
+      <c r="HB1" s="1" t="s">
         <v>166</v>
       </c>
-      <c r="GQ1" s="1" t="s">
+      <c r="HC1" s="1" t="s">
         <v>167</v>
       </c>
-      <c r="GR1" s="1" t="s">
+      <c r="HD1" s="1" t="s">
         <v>168</v>
       </c>
-      <c r="GS1" s="1" t="s">
+      <c r="HE1" s="1" t="s">
         <v>169</v>
       </c>
-      <c r="GT1" s="1" t="s">
+      <c r="HF1" s="1" t="s">
         <v>170</v>
       </c>
-      <c r="GU1" s="1" t="s">
+      <c r="HG1" s="1" t="s">
         <v>171</v>
       </c>
-      <c r="GV1" s="1" t="s">
+      <c r="HH1" s="1" t="s">
         <v>172</v>
       </c>
-      <c r="GW1" s="1" t="s">
+      <c r="HI1" s="1" t="s">
         <v>173</v>
       </c>
-      <c r="GX1" s="1" t="s">
+      <c r="HJ1" s="1" t="s">
         <v>174</v>
       </c>
-      <c r="GY1" s="1" t="s">
+      <c r="HK1" s="1" t="s">
         <v>175</v>
       </c>
-      <c r="HM1" s="1" t="s">
+      <c r="HY1" s="1" t="s">
         <v>189</v>
       </c>
     </row>
-    <row r="2" spans="1:221" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:233" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>190</v>
       </c>
@@ -3092,448 +3191,484 @@
         <v>285</v>
       </c>
       <c r="DC2" s="1" t="s">
+        <v>292</v>
+      </c>
+      <c r="DD2" s="1" t="s">
+        <v>292</v>
+      </c>
+      <c r="DE2" s="1" t="s">
+        <v>292</v>
+      </c>
+      <c r="DF2" s="1" t="s">
+        <v>293</v>
+      </c>
+      <c r="DG2" s="1" t="s">
+        <v>294</v>
+      </c>
+      <c r="DH2" s="1" t="s">
+        <v>302</v>
+      </c>
+      <c r="DI2" s="1" t="s">
+        <v>303</v>
+      </c>
+      <c r="DJ2" s="1" t="s">
+        <v>304</v>
+      </c>
+      <c r="DK2" s="1" t="s">
+        <v>195</v>
+      </c>
+      <c r="DL2" s="1" t="s">
+        <v>305</v>
+      </c>
+      <c r="DM2" s="1" t="s">
+        <v>306</v>
+      </c>
+      <c r="DN2" s="1" t="s">
+        <v>307</v>
+      </c>
+      <c r="DO2" s="1" t="s">
         <v>200</v>
       </c>
-      <c r="DD2" s="1" t="s">
+      <c r="DP2" s="1" t="s">
         <v>207</v>
       </c>
-      <c r="DE2" s="1" t="s">
+      <c r="DQ2" s="1" t="s">
         <v>195</v>
       </c>
-      <c r="DF2" s="1" t="s">
+      <c r="DR2" s="1" t="s">
         <v>195</v>
       </c>
-      <c r="DG2" s="1" t="s">
+      <c r="DS2" s="1" t="s">
         <v>195</v>
       </c>
-      <c r="DH2" s="1" t="s">
+      <c r="DT2" s="1" t="s">
         <v>195</v>
       </c>
-      <c r="DI2" s="1" t="s">
+      <c r="DU2" s="1" t="s">
         <v>195</v>
       </c>
-      <c r="DJ2" s="1" t="s">
+      <c r="DV2" s="1" t="s">
         <v>208</v>
       </c>
-      <c r="DK2" s="1" t="s">
+      <c r="DW2" s="1" t="s">
         <v>200</v>
       </c>
-      <c r="DL2" s="1" t="s">
+      <c r="DX2" s="1" t="s">
         <v>209</v>
       </c>
-      <c r="DM2" s="1" t="s">
+      <c r="DY2" s="1" t="s">
         <v>210</v>
       </c>
-      <c r="DN2" s="1" t="s">
+      <c r="DZ2" s="1" t="s">
         <v>211</v>
       </c>
-      <c r="DO2" s="1" t="s">
+      <c r="EA2" s="1" t="s">
         <v>212</v>
       </c>
-      <c r="DP2" s="1" t="s">
+      <c r="EB2" s="1" t="s">
         <v>200</v>
       </c>
-      <c r="DQ2" s="1" t="s">
+      <c r="EC2" s="1" t="s">
         <v>213</v>
       </c>
-      <c r="DR2" s="1" t="s">
+      <c r="ED2" s="1" t="s">
         <v>214</v>
       </c>
-      <c r="DS2" s="1" t="s">
+      <c r="EE2" s="1" t="s">
         <v>200</v>
       </c>
-      <c r="DT2" s="1" t="s">
+      <c r="EF2" s="1" t="s">
         <v>215</v>
       </c>
-      <c r="DU2" s="1" t="s">
+      <c r="EG2" s="1" t="s">
         <v>216</v>
       </c>
-      <c r="DV2" s="1" t="s">
+      <c r="EH2" s="1" t="s">
         <v>200</v>
       </c>
-      <c r="DW2" s="1" t="s">
+      <c r="EI2" s="1" t="s">
         <v>217</v>
       </c>
-      <c r="DX2" s="1" t="s">
+      <c r="EJ2" s="1" t="s">
         <v>200</v>
       </c>
-      <c r="DY2" s="1" t="s">
+      <c r="EK2" s="1" t="s">
         <v>218</v>
       </c>
-      <c r="DZ2" s="1" t="s">
+      <c r="EL2" s="1" t="s">
         <v>219</v>
       </c>
-      <c r="EA2" s="1" t="s">
+      <c r="EM2" s="1" t="s">
         <v>220</v>
       </c>
-      <c r="EB2" s="1" t="s">
+      <c r="EN2" s="1" t="s">
         <v>221</v>
       </c>
-      <c r="EC2" s="1" t="s">
+      <c r="EO2" s="1" t="s">
         <v>222</v>
       </c>
-      <c r="ED2" s="1" t="s">
+      <c r="EP2" s="1" t="s">
         <v>223</v>
       </c>
-      <c r="EE2" s="1" t="s">
+      <c r="EQ2" s="1" t="s">
         <v>224</v>
       </c>
-      <c r="EF2" s="1" t="s">
+      <c r="ER2" s="1" t="s">
         <v>225</v>
       </c>
-      <c r="EG2" s="1" t="s">
+      <c r="ES2" s="1" t="s">
         <v>208</v>
       </c>
-      <c r="EH2" s="1" t="s">
+      <c r="ET2" s="1" t="s">
         <v>226</v>
       </c>
-      <c r="EI2" s="1" t="s">
+      <c r="EU2" s="1" t="s">
         <v>200</v>
       </c>
-      <c r="EJ2" s="1" t="s">
+      <c r="EV2" s="1" t="s">
         <v>195</v>
       </c>
-      <c r="EK2" s="1" t="s">
+      <c r="EW2" s="1" t="s">
         <v>193</v>
-      </c>
-      <c r="EL2" s="1" t="s">
-        <v>200</v>
-      </c>
-      <c r="EM2" s="1" t="s">
-        <v>195</v>
-      </c>
-      <c r="EN2" s="1" t="s">
-        <v>195</v>
-      </c>
-      <c r="EO2" s="1" t="s">
-        <v>200</v>
-      </c>
-      <c r="EP2" s="1" t="s">
-        <v>227</v>
-      </c>
-      <c r="EQ2" s="1" t="s">
-        <v>228</v>
-      </c>
-      <c r="ER2" s="1" t="s">
-        <v>195</v>
-      </c>
-      <c r="ES2" s="1" t="s">
-        <v>195</v>
-      </c>
-      <c r="ET2" s="1" t="s">
-        <v>195</v>
-      </c>
-      <c r="EU2" s="1" t="s">
-        <v>195</v>
-      </c>
-      <c r="EV2" s="1" t="s">
-        <v>200</v>
-      </c>
-      <c r="EW2" s="1" t="s">
-        <v>203</v>
       </c>
       <c r="EX2" s="1" t="s">
         <v>200</v>
       </c>
       <c r="EY2" s="1" t="s">
-        <v>229</v>
+        <v>195</v>
       </c>
       <c r="EZ2" s="1" t="s">
-        <v>229</v>
+        <v>195</v>
       </c>
       <c r="FA2" s="1" t="s">
-        <v>230</v>
+        <v>200</v>
       </c>
       <c r="FB2" s="1" t="s">
-        <v>231</v>
+        <v>227</v>
       </c>
       <c r="FC2" s="1" t="s">
+        <v>228</v>
+      </c>
+      <c r="FD2" s="1" t="s">
+        <v>195</v>
+      </c>
+      <c r="FE2" s="1" t="s">
+        <v>195</v>
+      </c>
+      <c r="FF2" s="1" t="s">
+        <v>195</v>
+      </c>
+      <c r="FG2" s="1" t="s">
+        <v>195</v>
+      </c>
+      <c r="FH2" s="1" t="s">
         <v>200</v>
       </c>
-      <c r="FD2" s="1" t="s">
-        <v>232</v>
-      </c>
-      <c r="FE2" s="1" t="s">
-        <v>233</v>
-      </c>
-      <c r="FF2" s="1" t="s">
-        <v>200</v>
-      </c>
-      <c r="FG2" s="1" t="s">
-        <v>234</v>
-      </c>
-      <c r="FH2" s="1" t="s">
-        <v>235</v>
-      </c>
       <c r="FI2" s="1" t="s">
-        <v>236</v>
+        <v>203</v>
       </c>
       <c r="FJ2" s="1" t="s">
         <v>200</v>
       </c>
       <c r="FK2" s="1" t="s">
-        <v>237</v>
+        <v>229</v>
       </c>
       <c r="FL2" s="1" t="s">
         <v>229</v>
       </c>
       <c r="FM2" s="1" t="s">
-        <v>203</v>
+        <v>230</v>
       </c>
       <c r="FN2" s="1" t="s">
-        <v>238</v>
+        <v>231</v>
       </c>
       <c r="FO2" s="1" t="s">
         <v>200</v>
       </c>
       <c r="FP2" s="1" t="s">
+        <v>232</v>
+      </c>
+      <c r="FQ2" s="1" t="s">
+        <v>233</v>
+      </c>
+      <c r="FR2" s="1" t="s">
+        <v>200</v>
+      </c>
+      <c r="FS2" s="1" t="s">
+        <v>234</v>
+      </c>
+      <c r="FT2" s="1" t="s">
+        <v>235</v>
+      </c>
+      <c r="FU2" s="1" t="s">
+        <v>236</v>
+      </c>
+      <c r="FV2" s="1" t="s">
+        <v>200</v>
+      </c>
+      <c r="FW2" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="FX2" s="1" t="s">
+        <v>229</v>
+      </c>
+      <c r="FY2" s="1" t="s">
+        <v>203</v>
+      </c>
+      <c r="FZ2" s="1" t="s">
         <v>238</v>
       </c>
-      <c r="FQ2" s="1" t="s">
+      <c r="GA2" s="1" t="s">
+        <v>200</v>
+      </c>
+      <c r="GB2" s="1" t="s">
+        <v>238</v>
+      </c>
+      <c r="GC2" s="1" t="s">
         <v>239</v>
       </c>
-      <c r="FR2" s="1" t="s">
+      <c r="GD2" s="1" t="s">
         <v>240</v>
       </c>
-      <c r="FS2" s="1" t="s">
+      <c r="GE2" s="1" t="s">
         <v>208</v>
       </c>
-      <c r="FT2" s="1" t="s">
+      <c r="GF2" s="1" t="s">
         <v>241</v>
       </c>
-      <c r="FU2" s="1" t="s">
+      <c r="GG2" s="1" t="s">
         <v>242</v>
       </c>
-      <c r="FV2" s="1" t="s">
+      <c r="GH2" s="1" t="s">
         <v>193</v>
       </c>
-      <c r="FW2" s="1" t="s">
+      <c r="GI2" s="1" t="s">
         <v>193</v>
       </c>
-      <c r="FX2" s="1" t="s">
+      <c r="GJ2" s="1" t="s">
         <v>193</v>
       </c>
-      <c r="FY2" s="1" t="s">
+      <c r="GK2" s="1" t="s">
         <v>195</v>
       </c>
-      <c r="FZ2" s="1" t="s">
+      <c r="GL2" s="1" t="s">
         <v>208</v>
       </c>
-      <c r="GA2" s="1" t="s">
+      <c r="GM2" s="1" t="s">
         <v>243</v>
       </c>
-      <c r="GB2" s="1" t="s">
+      <c r="GN2" s="1" t="s">
         <v>200</v>
       </c>
-      <c r="GC2" s="1" t="s">
+      <c r="GO2" s="1" t="s">
         <v>208</v>
       </c>
-      <c r="GD2" s="1" t="s">
+      <c r="GP2" s="1" t="s">
         <v>244</v>
       </c>
-      <c r="GE2" s="1" t="s">
+      <c r="GQ2" s="1" t="s">
         <v>200</v>
       </c>
-      <c r="GF2" s="1" t="s">
+      <c r="GR2" s="1" t="s">
         <v>245</v>
       </c>
-      <c r="GG2" s="1" t="s">
+      <c r="GS2" s="1" t="s">
         <v>246</v>
       </c>
-      <c r="GH2" s="1" t="s">
+      <c r="GT2" s="1" t="s">
         <v>243</v>
       </c>
-      <c r="GI2" s="1" t="s">
+      <c r="GU2" s="1" t="s">
         <v>200</v>
       </c>
-      <c r="GJ2" s="1" t="s">
+      <c r="GV2" s="1" t="s">
         <v>247</v>
       </c>
-      <c r="GK2" s="1" t="s">
+      <c r="GW2" s="1" t="s">
         <v>248</v>
       </c>
-      <c r="GL2" s="1" t="s">
+      <c r="GX2" s="1" t="s">
         <v>249</v>
       </c>
-      <c r="GM2" s="1" t="s">
+      <c r="GY2" s="1" t="s">
         <v>250</v>
       </c>
-      <c r="GN2" s="1" t="s">
+      <c r="GZ2" s="1" t="s">
         <v>251</v>
       </c>
-      <c r="GO2" s="1" t="s">
+      <c r="HA2" s="1" t="s">
         <v>252</v>
       </c>
-      <c r="GP2" s="1" t="s">
+      <c r="HB2" s="1" t="s">
         <v>253</v>
       </c>
-      <c r="GQ2" s="1" t="s">
+      <c r="HC2" s="1" t="s">
         <v>208</v>
       </c>
-      <c r="GR2" s="1" t="s">
+      <c r="HD2" s="1" t="s">
         <v>254</v>
       </c>
-      <c r="GS2" s="1" t="s">
+      <c r="HE2" s="1" t="s">
         <v>200</v>
       </c>
-      <c r="GT2" s="1" t="s">
+      <c r="HF2" s="1" t="s">
         <v>214</v>
       </c>
-      <c r="GU2" s="1" t="s">
+      <c r="HG2" s="1" t="s">
         <v>255</v>
       </c>
-      <c r="GV2" s="1" t="s">
+      <c r="HH2" s="1" t="s">
         <v>255</v>
       </c>
-      <c r="GW2" s="1" t="s">
+      <c r="HI2" s="1" t="s">
         <v>214</v>
       </c>
-      <c r="GX2" s="1" t="s">
+      <c r="HJ2" s="1" t="s">
         <v>200</v>
       </c>
-      <c r="GY2" s="1" t="s">
+      <c r="HK2" s="1" t="s">
         <v>214</v>
       </c>
     </row>
   </sheetData>
-  <dataValidations count="63">
+  <dataValidations count="73">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E2" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"Belum Menikah,Menikah,Cerai Mati,Cerai Hidup"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I2:J2 F2:G2 CA2:CG2 BY2 FV2:FY2 ER2:EU2 EM2:EN2 EJ2:EK2 DE2:DI2 BS2 BL2 BC2 AZ2 AW2 AT2 AQ2 AM2:AN2 AJ2 Z2:AF2 L2:U2" xr:uid="{00000000-0002-0000-0000-000001000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I2:J2 F2:G2 CA2:CG2 BY2 GH2:GK2 FD2:FG2 EY2:EZ2 EV2:EW2 DQ2:DU2 BS2 BL2 BC2 AZ2 AW2 AT2 AQ2 AM2:AN2 AJ2 Z2:AF2 L2:U2 DK2" xr:uid="{00000000-0002-0000-0000-000001000000}">
       <formula1>"Ya,Tidak"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H2" xr:uid="{00000000-0002-0000-0000-000002000000}">
       <formula1>"Non disabilitas,Penyandang disabilitas"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AG2 K2 GP2 GM2 DO2 DD2" xr:uid="{00000000-0002-0000-0000-000003000000}"/>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AG2 K2 HB2 GY2 EA2 DP2" xr:uid="{00000000-0002-0000-0000-000003000000}"/>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="V2:Y2" xr:uid="{00000000-0002-0000-0000-000004000000}">
       <formula1>"Tidak sama sekali,Kurang dari 1 minggu,Lebih dari 1 minggu,Hampir setiap hari"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AL2" xr:uid="{00000000-0002-0000-0000-000005000000}">
       <formula1>"1 s.d &lt;10 tahun lalu,10 s.d &lt;15 tahun lalu,15 tahun lalu atau lebih"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BK2 BG2 GX2 GS2 GI2 GE2 GB2 FO2 FJ2 FF2 FC2 EX2 EV2 EO2 EL2 EI2 DX2 DV2 DS2 DP2 DK2 DC2 BQ2:BR2" xr:uid="{00000000-0002-0000-0000-000006000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BK2 BG2 HJ2 HE2 GU2 GQ2 GN2 GA2 FV2 FR2 FO2 FJ2 FH2 FA2 EX2 EU2 EJ2 EH2 EE2 EB2 DW2 DO2 BQ2:BR2" xr:uid="{00000000-0002-0000-0000-000006000000}">
       <formula1>"True,False"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DJ2" xr:uid="{00000000-0002-0000-0000-000007000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DV2" xr:uid="{00000000-0002-0000-0000-000007000000}">
       <formula1>"Normal,Abnormal TBC,Abnormal non TBC"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DL2" xr:uid="{00000000-0002-0000-0000-000008000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DX2" xr:uid="{00000000-0002-0000-0000-000008000000}">
       <formula1>"Riwayat kontak serumah,Riwayat kontak erat,Tidak ada,Tidak diketahui"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DM2" xr:uid="{00000000-0002-0000-0000-000009000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DY2" xr:uid="{00000000-0002-0000-0000-000009000000}">
       <formula1>"Bakteriologis,Klinis"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DN2" xr:uid="{00000000-0002-0000-0000-00000A000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DZ2" xr:uid="{00000000-0002-0000-0000-00000A000000}">
       <formula1>"TCM,BTA,NPOC,Tidak dilakukan"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DQ2" xr:uid="{00000000-0002-0000-0000-00000B000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="EC2" xr:uid="{00000000-0002-0000-0000-00000B000000}">
       <formula1>"Suspek frambusia,Bukan frambusia,Tidak Ada"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="GT2:GW2 DR2 GY2" xr:uid="{00000000-0002-0000-0000-00000C000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="HF2:HI2 ED2 HK2" xr:uid="{00000000-0002-0000-0000-00000C000000}">
       <formula1>"Reaktif,Non Reaktif"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DT2" xr:uid="{00000000-0002-0000-0000-00000D000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="EF2" xr:uid="{00000000-0002-0000-0000-00000D000000}">
       <formula1>"Kusta,Bukan kusta,Meragukan,Tidak Ada"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DU2" xr:uid="{00000000-0002-0000-0000-00000E000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="EG2" xr:uid="{00000000-0002-0000-0000-00000E000000}">
       <formula1>"Kusta,Bukan kusta,Meragukan"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DW2" xr:uid="{00000000-0002-0000-0000-00000F000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="EI2" xr:uid="{00000000-0002-0000-0000-00000F000000}">
       <formula1>"Skabies,Bukan Skabies,Meragukan,Tidak Ada"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DY2" xr:uid="{00000000-0002-0000-0000-000010000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="EK2" xr:uid="{00000000-0002-0000-0000-000010000000}">
       <formula1>"Tidak ada serumen impaksi,Ada serumen impaksi"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DZ2" xr:uid="{00000000-0002-0000-0000-000011000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="EL2" xr:uid="{00000000-0002-0000-0000-000011000000}">
       <formula1>"Tidak ada infeksi telinga,Ada infeksi telinga"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="EA2" xr:uid="{00000000-0002-0000-0000-000012000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="EM2" xr:uid="{00000000-0002-0000-0000-000012000000}">
       <formula1>"Normal,Curiga gangguan pendengaran"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="EB2" xr:uid="{00000000-0002-0000-0000-000013000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="EN2" xr:uid="{00000000-0002-0000-0000-000013000000}">
       <formula1>"Normal,Gangguan Pendengaran"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="EC2" xr:uid="{00000000-0002-0000-0000-000014000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="EO2" xr:uid="{00000000-0002-0000-0000-000014000000}">
       <formula1>"Normal (visus 6/6 - 6/12),Curiga gangguan penglihatan (visus &lt;6/12)"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="ED2" xr:uid="{00000000-0002-0000-0000-000015000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="EP2" xr:uid="{00000000-0002-0000-0000-000015000000}">
       <formula1>"Normal (visus 6/6 - 6/12),Gangguan penglihatan ringan (visus &lt;6/12 - 6/18),Gangguan penglihatan sedang (&lt;6/18 - 6/60),Gangguan penglihatan berat (&lt;6/60 - 3/60),Buta (&lt;3/60)"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="EE2" xr:uid="{00000000-0002-0000-0000-000016000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="EQ2" xr:uid="{00000000-0002-0000-0000-000016000000}">
       <formula1>"Visus membaik,Visus tidak membaik (visus tetap)"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="EF2" xr:uid="{00000000-0002-0000-0000-000017000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="ER2" xr:uid="{00000000-0002-0000-0000-000017000000}">
       <formula1>"Kelainan refraksi ringan (0.50 - 3.00 Dioptri),Kelainan refraksi sedang (3.00 - 6.00 Dioptri),Kelainan refraksi berat (&gt;6.00 Dioptri)"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="EG2" xr:uid="{00000000-0002-0000-0000-000018000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="ES2" xr:uid="{00000000-0002-0000-0000-000018000000}">
       <formula1>"Normal,Curiga kelainan mata"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="EH2" xr:uid="{00000000-0002-0000-0000-000019000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="ET2" xr:uid="{00000000-0002-0000-0000-000019000000}">
       <formula1>"Curiga katarak,Normal"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="EP2" xr:uid="{00000000-0002-0000-0000-00001A000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="FB2" xr:uid="{00000000-0002-0000-0000-00001A000000}">
       <formula1>"Iya,Tidak"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="EQ2" xr:uid="{00000000-0002-0000-0000-00001B000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="FC2" xr:uid="{00000000-0002-0000-0000-00001B000000}">
       <formula1>"&lt;20 bungkus per tahun,20-30 bungkus per tahun,&gt;30 bungkus per tahun"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="FG2" xr:uid="{00000000-0002-0000-0000-00001C000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="FS2" xr:uid="{00000000-0002-0000-0000-00001C000000}">
       <formula1>"HBsAg Non Reaktif,HBsAg Reaktif"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="FH2" xr:uid="{00000000-0002-0000-0000-00001D000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="FT2" xr:uid="{00000000-0002-0000-0000-00001D000000}">
       <formula1>"Anti HCV Non Reaktif,Anti HCV Reaktif"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="FI2" xr:uid="{00000000-0002-0000-0000-00001E000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="FU2" xr:uid="{00000000-0002-0000-0000-00001E000000}">
       <formula1>"VL HCV RNA Negatif,VL HCV RNA Positif"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="GC2" xr:uid="{00000000-0002-0000-0000-00001F000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="GO2" xr:uid="{00000000-0002-0000-0000-00001F000000}">
       <formula1>"Normal,Abnormal"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="GD2" xr:uid="{00000000-0002-0000-0000-000020000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="GP2" xr:uid="{00000000-0002-0000-0000-000020000000}">
       <formula1>"Normal,Abnormal ST Depresi,Abnormal T Inversi,Abnormal Hipertrofi Ventrikel Kiri,Abnormal Atrial Fibrilasi,Abnormal Q-Patologis,Abnormal ST Elevasi,Abnormal Gambaran Abnormal Lainnya"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="GF2" xr:uid="{00000000-0002-0000-0000-000021000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="GR2" xr:uid="{00000000-0002-0000-0000-000021000000}">
       <formula1>"Bersedia,Menolak,Tidak tahu"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="GG2" xr:uid="{00000000-0002-0000-0000-000022000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="GS2" xr:uid="{00000000-0002-0000-0000-000022000000}">
       <formula1>"Ditemukan benjolan,Tidak ditemukan benjolan"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="GH2 GA2" xr:uid="{00000000-0002-0000-0000-000023000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="GT2 GM2" xr:uid="{00000000-0002-0000-0000-000023000000}">
       <formula1>"Negatif,Positif"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="GJ2" xr:uid="{00000000-0002-0000-0000-000024000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="GV2" xr:uid="{00000000-0002-0000-0000-000024000000}">
       <formula1>"Memiliki diagnosis kanker &gt;5 tahun yang lalu,Memiliki diagnosis kanker &lt;5 tahun yang lalu,Tidak pernah didiagnosis menderita kanker"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="GK2" xr:uid="{00000000-0002-0000-0000-000025000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="GW2" xr:uid="{00000000-0002-0000-0000-000025000000}">
       <formula1>"Memiliki keluarga yang terdiagnosis kanker paru,Memiliki keluarga yang terdiagnosis kanker lain,Tidak ada keluarga yang terdiagnosis kanker"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="GL2" xr:uid="{00000000-0002-0000-0000-000026000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="GX2" xr:uid="{00000000-0002-0000-0000-000026000000}">
       <formula1>"Perokok aktif (dalam 1 tahun ini masih merokok),Perokok/bekas perokok berhenti &lt;10 tahun lalu,Perokok pasif dari lingkungan rumah/tempat kerja,Tidak pernah merokok"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="GN2" xr:uid="{00000000-0002-0000-0000-000027000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="GZ2" xr:uid="{00000000-0002-0000-0000-000027000000}">
       <formula1>"Memiliki tempat tinggal berpotensi tinggi,Tidak yakin memiliki tempat tinggal berpotensi tinggi,Tidak memiliki tempat tinggal berpotensi tinggi"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="GO2" xr:uid="{00000000-0002-0000-0000-000028000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="HA2" xr:uid="{00000000-0002-0000-0000-000028000000}">
       <formula1>"Memiliki lingkungan dalam rumah yang tidak sehat,Tidak yakin memiliki lingkungan dalam rumah yang tidak sehat,Memiliki lingkungan dalam rumah yang sehat"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="GQ2" xr:uid="{00000000-0002-0000-0000-000029000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="HC2" xr:uid="{00000000-0002-0000-0000-000029000000}">
       <formula1>"Normal,Tidak Normal"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="FR2" xr:uid="{00000000-0002-0000-0000-00002A000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="GD2" xr:uid="{00000000-0002-0000-0000-00002A000000}">
       <formula1>"SADANIS,USG Payudara"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="FS2" xr:uid="{00000000-0002-0000-0000-00002B000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="GE2" xr:uid="{00000000-0002-0000-0000-00002B000000}">
       <formula1>"Normal,Ditemukan benjolan,Curiga kanker"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="FT2" xr:uid="{00000000-0002-0000-0000-00002C000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="GF2" xr:uid="{00000000-0002-0000-0000-00002C000000}">
       <formula1>" Normal,Simple cyst,Non simple cyst"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="FU2" xr:uid="{00000000-0002-0000-0000-00002D000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="GG2" xr:uid="{00000000-0002-0000-0000-00002D000000}">
       <formula1>"HPV Negatif,HPV Positif"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="FZ2" xr:uid="{00000000-0002-0000-0000-00002E000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="GL2" xr:uid="{00000000-0002-0000-0000-00002E000000}">
       <formula1>"Normal,Curiga kanker"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BZ2" xr:uid="{00000000-0002-0000-0000-00002F000000}">
@@ -3598,6 +3733,57 @@
         </mc:Fallback>
       </mc:AlternateContent>
     </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DC2:DD2" xr:uid="{8624A411-ABFC-AD42-9F33-B885D13D9656}">
+      <formula1>"Bertahan 10 detik,Tidak bertahan 10 detik,Tidak dilakukan"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DE2" xr:uid="{27C5DDB0-8CF7-684B-A261-24A7DB1D3F89}">
+      <formula1>"Bertahan 10 detik,Bertahan 3 - 9.99 detik,Bertahan &lt; 3 detik"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DF2" xr:uid="{F158B156-CDAF-B64E-9412-DC98B28AAB2D}">
+      <mc:AlternateContent xmlns:x12ac="http://schemas.microsoft.com/office/spreadsheetml/2011/1/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+        <mc:Choice Requires="x12ac">
+          <x12ac:list>"4,82 detik",4.83 - 6.20 detik,6.21 - 8.70 detik,"&gt;8,70 detik",Tidak dapat menyelesaikan</x12ac:list>
+        </mc:Choice>
+        <mc:Fallback>
+          <formula1>"4,82 detik,4.83 - 6.20 detik,6.21 - 8.70 detik,&gt;8,70 detik,Tidak dapat menyelesaikan"</formula1>
+        </mc:Fallback>
+      </mc:AlternateContent>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DG2" xr:uid="{FA3B3CBF-2776-6F44-B496-E4AACD7B8DE5}">
+      <mc:AlternateContent xmlns:x12ac="http://schemas.microsoft.com/office/spreadsheetml/2011/1/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+        <mc:Choice Requires="x12ac">
+          <x12ac:list>&lt;11.19 detik,"11.2 - 13,69 detik",13.7 - 16.69 detik,16.7 - 59.9 detik,&gt;60 detik atau tidak menyelesaikan</x12ac:list>
+        </mc:Choice>
+        <mc:Fallback>
+          <formula1>"&lt;11.19 detik,11.2 - 13,69 detik,13.7 - 16.69 detik,16.7 - 59.9 detik,&gt;60 detik atau tidak menyelesaikan"</formula1>
+        </mc:Fallback>
+      </mc:AlternateContent>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DH2" xr:uid="{E7F1499F-D1E2-2A45-B604-5C8D9095D6FE}">
+      <formula1>"Nafsu Makan Yang Sangat Berkurang,Nafsu Makan Sedikit Berkurang,Nafsu Makan Biasa saja"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DI2" xr:uid="{7BA75764-D8E9-1244-889F-533206C29E1E}">
+      <formula1>"Penurunan BB &gt; 3 Kg,Tidak Tahu,Penurunan BB antara 1 - 3 Kg"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DJ2" xr:uid="{B6F2B7AB-5238-904C-898F-2DD19DAB3A37}">
+      <mc:AlternateContent xmlns:x12ac="http://schemas.microsoft.com/office/spreadsheetml/2011/1/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+        <mc:Choice Requires="x12ac">
+          <x12ac:list>Harus berbaring di tempat tidur atau menggunakan kursi roda,"Bisa bangun dari tempat tidur atau kursi roda, tetapi tidak bisa keluar rumah",Bisa bepergian keluar rumah</x12ac:list>
+        </mc:Choice>
+        <mc:Fallback>
+          <formula1>"Harus berbaring di tempat tidur atau menggunakan kursi roda,Bisa bangun dari tempat tidur atau kursi roda, tetapi tidak bisa keluar rumah,Bisa bepergian keluar rumah"</formula1>
+        </mc:Fallback>
+      </mc:AlternateContent>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DL2" xr:uid="{2747DE2C-9959-3048-987D-CB575AA915B8}">
+      <formula1>"Dementia atau depresi berat,Demensia/kepikunan ringan,Tidak ada masalah psikologis"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DM2" xr:uid="{5F47AFFC-E088-F741-819D-BC4A4B3B866E}">
+      <formula1>"IMT &lt;19,IMT 19 - &lt;21,IMT 21 - &lt;23,IMT &gt;= 23"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DN2" xr:uid="{DC939003-7519-6246-A4A2-66B3FBE91AAA}">
+      <formula1>"&lt;31 cm,&gt;= 31 cm"</formula1>
+    </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>

</xml_diff>

<commit_message>
i believe lansia perempuan is done
</commit_message>
<xml_diff>
--- a/dataset/lansia.xlsx
+++ b/dataset/lansia.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/macbokprom12021/PycharmProjects/CKG-Helper/dataset/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FE886EB6-AEFC-5E40-8968-AA2991247EE8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C0A82DB6-4387-9D44-843F-88583303A11F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4480" yWindow="-21000" windowWidth="36000" windowHeight="19540" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -573,7 +573,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="389" uniqueCount="289">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="390" uniqueCount="290">
   <si>
     <t>batas_awal</t>
   </si>
@@ -800,6 +800,144 @@
     <t>diastolik_2</t>
   </si>
   <si>
+    <t>mengingat_3_kata</t>
+  </si>
+  <si>
+    <t>tanggal_berapa_dimana</t>
+  </si>
+  <si>
+    <t>ulangi_3_kata_sebelumnya</t>
+  </si>
+  <si>
+    <t>berdiri_di_kursi</t>
+  </si>
+  <si>
+    <t>berat_badan_berkurang</t>
+  </si>
+  <si>
+    <t>hilang_nafsu_makan</t>
+  </si>
+  <si>
+    <t>lila_kurang_21cm</t>
+  </si>
+  <si>
+    <t>2_minggu_terakhir_sedih</t>
+  </si>
+  <si>
+    <t>2_minggu_sedikit_minat</t>
+  </si>
+  <si>
+    <t>kendali_bab</t>
+  </si>
+  <si>
+    <t>kendali_bak</t>
+  </si>
+  <si>
+    <t>membersihkan_diri</t>
+  </si>
+  <si>
+    <t>penggunaan_jamban</t>
+  </si>
+  <si>
+    <t>makan_minum</t>
+  </si>
+  <si>
+    <t>berubah_sikap</t>
+  </si>
+  <si>
+    <t>berpindah</t>
+  </si>
+  <si>
+    <t>memakai_baju</t>
+  </si>
+  <si>
+    <t>naik_turun_tangga</t>
+  </si>
+  <si>
+    <t>mandi</t>
+  </si>
+  <si>
+    <t>mini_cog_1</t>
+  </si>
+  <si>
+    <t>mini_cog_2</t>
+  </si>
+  <si>
+    <t>mini_cog_3</t>
+  </si>
+  <si>
+    <t>ina_1</t>
+  </si>
+  <si>
+    <t>ina_2</t>
+  </si>
+  <si>
+    <t>ina_3</t>
+  </si>
+  <si>
+    <t>ina_4</t>
+  </si>
+  <si>
+    <t>ina_5</t>
+  </si>
+  <si>
+    <t>ina_6</t>
+  </si>
+  <si>
+    <t>ina_7</t>
+  </si>
+  <si>
+    <t>ina_8</t>
+  </si>
+  <si>
+    <t>sppb_1</t>
+  </si>
+  <si>
+    <t>sppb_2</t>
+  </si>
+  <si>
+    <t>sppb_3</t>
+  </si>
+  <si>
+    <t>sppb_4</t>
+  </si>
+  <si>
+    <t>sppb_5</t>
+  </si>
+  <si>
+    <t>mna_sf_1</t>
+  </si>
+  <si>
+    <t>mna_sf_2</t>
+  </si>
+  <si>
+    <t>mna_sf_3</t>
+  </si>
+  <si>
+    <t>mna_sf_4</t>
+  </si>
+  <si>
+    <t>mna_sf_5</t>
+  </si>
+  <si>
+    <t>mna_sf_6</t>
+  </si>
+  <si>
+    <t>mna_sf_7</t>
+  </si>
+  <si>
+    <t>depresi_lanjutan_1</t>
+  </si>
+  <si>
+    <t>depresi_lanjutan_2</t>
+  </si>
+  <si>
+    <t>depresi_lanjutan_3</t>
+  </si>
+  <si>
+    <t>depresi_lanjutan_4</t>
+  </si>
+  <si>
     <t>periksa_risiko_tbc</t>
   </si>
   <si>
@@ -1049,45 +1187,6 @@
     <t>foto_torax</t>
   </si>
   <si>
-    <t>mengingat_3_kata</t>
-  </si>
-  <si>
-    <t>tanggal_berapa_dimana</t>
-  </si>
-  <si>
-    <t>ulangi_3_kata_sebelumnya</t>
-  </si>
-  <si>
-    <t>berdiri_di_kursi</t>
-  </si>
-  <si>
-    <t>berat_badan_berkurang</t>
-  </si>
-  <si>
-    <t>hilang_nafsu_makan</t>
-  </si>
-  <si>
-    <t>lila_kurang_21cm</t>
-  </si>
-  <si>
-    <t>2_minggu_terakhir_sedih</t>
-  </si>
-  <si>
-    <t>2_minggu_sedikit_minat</t>
-  </si>
-  <si>
-    <t>kendali_bab</t>
-  </si>
-  <si>
-    <t>kendali_bak</t>
-  </si>
-  <si>
-    <t>membersihkan_diri</t>
-  </si>
-  <si>
-    <t>penggunaan_jamban</t>
-  </si>
-  <si>
     <t>status</t>
   </si>
   <si>
@@ -1097,6 +1196,9 @@
     <t>2026-05-17</t>
   </si>
   <si>
+    <t>SANIYA</t>
+  </si>
+  <si>
     <t>Belum Menikah</t>
   </si>
   <si>
@@ -1142,6 +1244,72 @@
     <t>120</t>
   </si>
   <si>
+    <t>Benar semua</t>
+  </si>
+  <si>
+    <t>Tidak terkendali/tak teratur (perlu pencahar)</t>
+  </si>
+  <si>
+    <t>Kadang-kadang tak terkendali (hanya 1 x / 24 jam)</t>
+  </si>
+  <si>
+    <t>Mandiri</t>
+  </si>
+  <si>
+    <t>Bisa (pindah) dengan kursi roda</t>
+  </si>
+  <si>
+    <t>Sebagian dibantu (misalnya: mengancing baju)</t>
+  </si>
+  <si>
+    <t>Butuh pertolongan</t>
+  </si>
+  <si>
+    <t>SUDAH DITANYAKAN</t>
+  </si>
+  <si>
+    <t>Benar</t>
+  </si>
+  <si>
+    <t>Benar semua kata</t>
+  </si>
+  <si>
+    <t>Tidak, Berubah</t>
+  </si>
+  <si>
+    <t>Tidak Berubah</t>
+  </si>
+  <si>
+    <t>Tidak Tahu</t>
+  </si>
+  <si>
+    <t>Bertahan 10 detik</t>
+  </si>
+  <si>
+    <t>4.83 - 6.20 detik</t>
+  </si>
+  <si>
+    <t>&lt;11.19 detik</t>
+  </si>
+  <si>
+    <t>Nafsu Makan Yang Sangat Berkurang</t>
+  </si>
+  <si>
+    <t>Penurunan BB &gt; 3 Kg</t>
+  </si>
+  <si>
+    <t>Harus berbaring di tempat tidur atau menggunakan kursi roda</t>
+  </si>
+  <si>
+    <t>Dementia atau depresi berat</t>
+  </si>
+  <si>
+    <t>IMT &lt;19</t>
+  </si>
+  <si>
+    <t>&lt;31 cm</t>
+  </si>
+  <si>
     <t>Tidak batuk</t>
   </si>
   <si>
@@ -1241,18 +1409,18 @@
     <t>9</t>
   </si>
   <si>
+    <t>Abnormal T Inversi</t>
+  </si>
+  <si>
+    <t>Bersedia</t>
+  </si>
+  <si>
+    <t>Ditemukan benjolan</t>
+  </si>
+  <si>
     <t>Negatif</t>
   </si>
   <si>
-    <t>Abnormal T Inversi</t>
-  </si>
-  <si>
-    <t>Bersedia</t>
-  </si>
-  <si>
-    <t>Ditemukan benjolan</t>
-  </si>
-  <si>
     <t>Memiliki diagnosis kanker &gt;5 tahun yang lalu</t>
   </si>
   <si>
@@ -1274,172 +1442,7 @@
     <t>Pernah didiagnosis tuberkulosis (TBC)</t>
   </si>
   <si>
-    <t>SANIYA</t>
-  </si>
-  <si>
-    <t>Benar semua</t>
-  </si>
-  <si>
-    <t>Tidak terkendali/tak teratur (perlu pencahar)</t>
-  </si>
-  <si>
-    <t>Kadang-kadang tak terkendali (hanya 1 x / 24 jam)</t>
-  </si>
-  <si>
-    <t>Mandiri</t>
-  </si>
-  <si>
-    <t>makan_minum</t>
-  </si>
-  <si>
-    <t>berubah_sikap</t>
-  </si>
-  <si>
-    <t>berpindah</t>
-  </si>
-  <si>
-    <t>Bisa (pindah) dengan kursi roda</t>
-  </si>
-  <si>
-    <t>memakai_baju</t>
-  </si>
-  <si>
-    <t>Sebagian dibantu (misalnya: mengancing baju)</t>
-  </si>
-  <si>
-    <t>naik_turun_tangga</t>
-  </si>
-  <si>
-    <t>Butuh pertolongan</t>
-  </si>
-  <si>
-    <t>mandi</t>
-  </si>
-  <si>
-    <t>mini_cog_1</t>
-  </si>
-  <si>
-    <t>SUDAH DITANYAKAN</t>
-  </si>
-  <si>
-    <t>mini_cog_2</t>
-  </si>
-  <si>
-    <t>Benar</t>
-  </si>
-  <si>
-    <t>mini_cog_3</t>
-  </si>
-  <si>
-    <t>Benar semua kata</t>
-  </si>
-  <si>
-    <t>ina_1</t>
-  </si>
-  <si>
-    <t>ina_2</t>
-  </si>
-  <si>
-    <t>ina_3</t>
-  </si>
-  <si>
-    <t>ina_4</t>
-  </si>
-  <si>
-    <t>ina_5</t>
-  </si>
-  <si>
-    <t>ina_6</t>
-  </si>
-  <si>
-    <t>ina_7</t>
-  </si>
-  <si>
-    <t>ina_8</t>
-  </si>
-  <si>
-    <t>Tidak, Berubah</t>
-  </si>
-  <si>
-    <t>Tidak Tahu</t>
-  </si>
-  <si>
-    <t>Tidak Berubah</t>
-  </si>
-  <si>
-    <t>sppb_1</t>
-  </si>
-  <si>
-    <t>sppb_2</t>
-  </si>
-  <si>
-    <t>sppb_3</t>
-  </si>
-  <si>
-    <t>sppb_4</t>
-  </si>
-  <si>
-    <t>sppb_5</t>
-  </si>
-  <si>
-    <t>Bertahan 10 detik</t>
-  </si>
-  <si>
-    <t>4.83 - 6.20 detik</t>
-  </si>
-  <si>
-    <t>&lt;11.19 detik</t>
-  </si>
-  <si>
-    <t>mna_sf_1</t>
-  </si>
-  <si>
-    <t>mna_sf_2</t>
-  </si>
-  <si>
-    <t>mna_sf_3</t>
-  </si>
-  <si>
-    <t>mna_sf_4</t>
-  </si>
-  <si>
-    <t>mna_sf_5</t>
-  </si>
-  <si>
-    <t>mna_sf_6</t>
-  </si>
-  <si>
-    <t>mna_sf_7</t>
-  </si>
-  <si>
-    <t>Nafsu Makan Yang Sangat Berkurang</t>
-  </si>
-  <si>
-    <t>Penurunan BB &gt; 3 Kg</t>
-  </si>
-  <si>
-    <t>Harus berbaring di tempat tidur atau menggunakan kursi roda</t>
-  </si>
-  <si>
-    <t>Dementia atau depresi berat</t>
-  </si>
-  <si>
-    <t>IMT &lt;19</t>
-  </si>
-  <si>
-    <t>&lt;31 cm</t>
-  </si>
-  <si>
-    <t>depresi_lanjutan_1</t>
-  </si>
-  <si>
-    <t>depresi_lanjutan_2</t>
-  </si>
-  <si>
-    <t>depresi_lanjutan_3</t>
-  </si>
-  <si>
-    <t>depresi_lanjutan_4</t>
+    <t>SUCCESS</t>
   </si>
 </sst>
 </file>
@@ -1471,7 +1474,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="1" tint="0.14996795556505021"/>
+        <fgColor theme="1" tint="0.14993743705557422"/>
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
@@ -1509,7 +1512,7 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="1"/>
   </cellXfs>
   <cellStyles count="2">
-    <cellStyle name="Dark Mode" xfId="1" xr:uid="{C1BE6BC5-A9D3-5A4E-8C2B-AB85F7B3EB34}"/>
+    <cellStyle name="Dark Mode" xfId="1" xr:uid="{00000000-0005-0000-0000-000001000000}"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -1842,7 +1845,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:HK2"/>
+  <dimension ref="A1:GX2"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="17.5" style="1" bestFit="1" customWidth="1"/>
@@ -1852,8 +1855,7 @@
     <col min="5" max="5" width="16.6640625" style="1" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="15.83203125" style="1" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="15.83203125" style="1" customWidth="1"/>
-    <col min="8" max="8" width="10.83203125" style="1" customWidth="1"/>
-    <col min="9" max="9" width="10.83203125" style="1"/>
+    <col min="8" max="9" width="10.83203125" style="1" customWidth="1"/>
     <col min="10" max="10" width="8.1640625" style="1" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="21" style="1" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="16" style="1" bestFit="1" customWidth="1"/>
@@ -1862,7 +1864,7 @@
     <col min="15" max="15" width="13.83203125" style="1" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="11.5" style="1" bestFit="1" customWidth="1"/>
     <col min="17" max="17" width="16.5" style="1" bestFit="1" customWidth="1"/>
-    <col min="18" max="19" width="10.83203125" style="1"/>
+    <col min="18" max="19" width="10.83203125" style="1" customWidth="1"/>
     <col min="20" max="20" width="14.5" style="1" bestFit="1" customWidth="1"/>
     <col min="21" max="21" width="14.5" style="1" customWidth="1"/>
     <col min="22" max="22" width="17" style="1" bestFit="1" customWidth="1"/>
@@ -1872,7 +1874,7 @@
     <col min="28" max="28" width="19.1640625" style="1" bestFit="1" customWidth="1"/>
     <col min="29" max="29" width="11.5" style="1" bestFit="1" customWidth="1"/>
     <col min="30" max="30" width="5.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="10.83203125" style="1"/>
+    <col min="31" max="31" width="10.83203125" style="1" customWidth="1"/>
     <col min="32" max="32" width="25.1640625" style="1" bestFit="1" customWidth="1"/>
     <col min="33" max="33" width="49" style="1" bestFit="1" customWidth="1"/>
     <col min="34" max="34" width="12.33203125" style="1" bestFit="1" customWidth="1"/>
@@ -1891,7 +1893,7 @@
     <col min="47" max="47" width="13.83203125" style="1" bestFit="1" customWidth="1"/>
     <col min="48" max="48" width="15.5" style="1" bestFit="1" customWidth="1"/>
     <col min="49" max="49" width="16" style="1" bestFit="1" customWidth="1"/>
-    <col min="50" max="50" width="10.83203125" style="1"/>
+    <col min="50" max="50" width="10.83203125" style="1" customWidth="1"/>
     <col min="51" max="51" width="13.83203125" style="1" bestFit="1" customWidth="1"/>
     <col min="52" max="52" width="18.33203125" style="1" bestFit="1" customWidth="1"/>
     <col min="53" max="53" width="14.33203125" style="1" bestFit="1" customWidth="1"/>
@@ -2009,22 +2011,11 @@
     <col min="203" max="203" width="43.1640625" style="1" bestFit="1" customWidth="1"/>
     <col min="204" max="204" width="18.1640625" style="1" customWidth="1"/>
     <col min="205" max="205" width="9.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="206" max="206" width="16" style="1" bestFit="1" customWidth="1"/>
-    <col min="207" max="207" width="21" style="1" bestFit="1" customWidth="1"/>
-    <col min="208" max="208" width="23.6640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="209" max="209" width="13.6640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="210" max="210" width="20.5" style="1" bestFit="1" customWidth="1"/>
-    <col min="211" max="211" width="18" style="1" bestFit="1" customWidth="1"/>
-    <col min="212" max="212" width="15.5" style="1" bestFit="1" customWidth="1"/>
-    <col min="213" max="213" width="21.83203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="214" max="214" width="21.1640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="215" max="216" width="10.83203125" style="1"/>
-    <col min="217" max="217" width="24.83203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="218" max="218" width="29.1640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="219" max="16384" width="10.83203125" style="1"/>
+    <col min="206" max="206" width="10.83203125" style="1" customWidth="1"/>
+    <col min="207" max="16384" width="10.83203125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:219" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:206" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2251,492 +2242,492 @@
         <v>74</v>
       </c>
       <c r="BY1" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="BZ1" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="CA1" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="CB1" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="CC1" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="CD1" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="CE1" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="CF1" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="CG1" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="CH1" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="CI1" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="CJ1" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="CK1" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="CL1" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="CM1" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="CN1" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="CO1" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="CP1" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="CQ1" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="CR1" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="CS1" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="CT1" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="CU1" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="CV1" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="CW1" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="CX1" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="CY1" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="CZ1" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="DA1" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="DB1" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="DC1" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="DD1" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="DE1" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="DF1" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="DG1" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="DH1" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="DI1" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="DJ1" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="DK1" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="DL1" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="DM1" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="DN1" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="DO1" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="DP1" s="1" t="s">
+        <v>118</v>
+      </c>
+      <c r="DQ1" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="DR1" s="1" t="s">
+        <v>120</v>
+      </c>
+      <c r="DS1" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="DT1" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="DU1" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="DV1" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="DW1" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="DX1" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="DY1" s="1" t="s">
+        <v>127</v>
+      </c>
+      <c r="DZ1" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="EA1" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="EB1" s="1" t="s">
+        <v>130</v>
+      </c>
+      <c r="EC1" s="1" t="s">
+        <v>131</v>
+      </c>
+      <c r="ED1" s="1" t="s">
+        <v>132</v>
+      </c>
+      <c r="EE1" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="EF1" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="EG1" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="EH1" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="EI1" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="EJ1" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="EK1" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="EL1" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="EM1" s="1" t="s">
+        <v>141</v>
+      </c>
+      <c r="EN1" s="1" t="s">
+        <v>142</v>
+      </c>
+      <c r="EO1" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="EP1" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="EQ1" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="ER1" s="1" t="s">
+        <v>146</v>
+      </c>
+      <c r="ES1" s="1" t="s">
+        <v>147</v>
+      </c>
+      <c r="ET1" s="1" t="s">
+        <v>148</v>
+      </c>
+      <c r="EU1" s="1" t="s">
+        <v>149</v>
+      </c>
+      <c r="EV1" s="1" t="s">
+        <v>150</v>
+      </c>
+      <c r="EW1" s="1" t="s">
+        <v>151</v>
+      </c>
+      <c r="EX1" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="EY1" s="1" t="s">
+        <v>153</v>
+      </c>
+      <c r="EZ1" s="1" t="s">
+        <v>154</v>
+      </c>
+      <c r="FA1" s="1" t="s">
+        <v>155</v>
+      </c>
+      <c r="FB1" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="FC1" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="FD1" s="1" t="s">
         <v>158</v>
       </c>
-      <c r="BZ1" s="1" t="s">
+      <c r="FE1" s="1" t="s">
         <v>159</v>
       </c>
-      <c r="CA1" s="1" t="s">
+      <c r="FF1" s="1" t="s">
         <v>160</v>
       </c>
-      <c r="CB1" s="1" t="s">
+      <c r="FG1" s="1" t="s">
         <v>161</v>
       </c>
-      <c r="CC1" s="1" t="s">
+      <c r="FH1" s="1" t="s">
         <v>162</v>
       </c>
-      <c r="CD1" s="1" t="s">
+      <c r="FI1" s="1" t="s">
         <v>163</v>
       </c>
-      <c r="CE1" s="1" t="s">
+      <c r="FJ1" s="1" t="s">
         <v>164</v>
       </c>
-      <c r="CF1" s="1" t="s">
+      <c r="FK1" s="1" t="s">
         <v>165</v>
       </c>
-      <c r="CG1" s="1" t="s">
+      <c r="FL1" s="1" t="s">
         <v>166</v>
       </c>
-      <c r="CH1" s="1" t="s">
+      <c r="FM1" s="1" t="s">
         <v>167</v>
       </c>
-      <c r="CI1" s="1" t="s">
+      <c r="FN1" s="1" t="s">
         <v>168</v>
       </c>
-      <c r="CJ1" s="1" t="s">
+      <c r="FO1" s="1" t="s">
         <v>169</v>
       </c>
-      <c r="CK1" s="1" t="s">
+      <c r="FP1" s="1" t="s">
         <v>170</v>
       </c>
-      <c r="CL1" s="1" t="s">
-        <v>238</v>
-      </c>
-      <c r="CM1" s="1" t="s">
-        <v>239</v>
-      </c>
-      <c r="CN1" s="1" t="s">
-        <v>240</v>
-      </c>
-      <c r="CO1" s="1" t="s">
-        <v>242</v>
-      </c>
-      <c r="CP1" s="1" t="s">
-        <v>244</v>
-      </c>
-      <c r="CQ1" s="1" t="s">
-        <v>246</v>
-      </c>
-      <c r="CR1" s="1" t="s">
-        <v>247</v>
-      </c>
-      <c r="CS1" s="1" t="s">
-        <v>249</v>
-      </c>
-      <c r="CT1" s="1" t="s">
-        <v>251</v>
-      </c>
-      <c r="CU1" s="1" t="s">
-        <v>253</v>
-      </c>
-      <c r="CV1" s="1" t="s">
-        <v>254</v>
-      </c>
-      <c r="CW1" s="1" t="s">
-        <v>255</v>
-      </c>
-      <c r="CX1" s="1" t="s">
-        <v>256</v>
-      </c>
-      <c r="CY1" s="1" t="s">
-        <v>257</v>
-      </c>
-      <c r="CZ1" s="1" t="s">
-        <v>258</v>
-      </c>
-      <c r="DA1" s="1" t="s">
-        <v>259</v>
-      </c>
-      <c r="DB1" s="1" t="s">
-        <v>260</v>
-      </c>
-      <c r="DC1" s="1" t="s">
-        <v>264</v>
-      </c>
-      <c r="DD1" s="1" t="s">
-        <v>265</v>
-      </c>
-      <c r="DE1" s="1" t="s">
-        <v>266</v>
-      </c>
-      <c r="DF1" s="1" t="s">
-        <v>267</v>
-      </c>
-      <c r="DG1" s="1" t="s">
-        <v>268</v>
-      </c>
-      <c r="DH1" s="1" t="s">
-        <v>272</v>
-      </c>
-      <c r="DI1" s="1" t="s">
-        <v>273</v>
-      </c>
-      <c r="DJ1" s="1" t="s">
-        <v>274</v>
-      </c>
-      <c r="DK1" s="1" t="s">
-        <v>275</v>
-      </c>
-      <c r="DL1" s="1" t="s">
-        <v>276</v>
-      </c>
-      <c r="DM1" s="1" t="s">
-        <v>277</v>
-      </c>
-      <c r="DN1" s="1" t="s">
-        <v>278</v>
-      </c>
-      <c r="DO1" s="1" t="s">
-        <v>285</v>
-      </c>
-      <c r="DP1" s="1" t="s">
-        <v>286</v>
-      </c>
-      <c r="DQ1" s="1" t="s">
-        <v>287</v>
-      </c>
-      <c r="DR1" s="1" t="s">
-        <v>288</v>
-      </c>
-      <c r="DS1" s="1" t="s">
-        <v>75</v>
-      </c>
-      <c r="DT1" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="DU1" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="DV1" s="1" t="s">
-        <v>78</v>
-      </c>
-      <c r="DW1" s="1" t="s">
-        <v>79</v>
-      </c>
-      <c r="DX1" s="1" t="s">
-        <v>80</v>
-      </c>
-      <c r="DY1" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="DZ1" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="EA1" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="EB1" s="1" t="s">
-        <v>84</v>
-      </c>
-      <c r="EC1" s="1" t="s">
-        <v>85</v>
-      </c>
-      <c r="ED1" s="1" t="s">
-        <v>86</v>
-      </c>
-      <c r="EE1" s="1" t="s">
-        <v>87</v>
-      </c>
-      <c r="EF1" s="1" t="s">
-        <v>88</v>
-      </c>
-      <c r="EG1" s="1" t="s">
-        <v>89</v>
-      </c>
-      <c r="EH1" s="1" t="s">
-        <v>90</v>
-      </c>
-      <c r="EI1" s="1" t="s">
-        <v>91</v>
-      </c>
-      <c r="EJ1" s="1" t="s">
-        <v>92</v>
-      </c>
-      <c r="EK1" s="1" t="s">
-        <v>93</v>
-      </c>
-      <c r="EL1" s="1" t="s">
-        <v>94</v>
-      </c>
-      <c r="EM1" s="1" t="s">
-        <v>95</v>
-      </c>
-      <c r="EN1" s="1" t="s">
-        <v>96</v>
-      </c>
-      <c r="EO1" s="1" t="s">
-        <v>97</v>
-      </c>
-      <c r="EP1" s="1" t="s">
-        <v>98</v>
-      </c>
-      <c r="EQ1" s="1" t="s">
-        <v>99</v>
-      </c>
-      <c r="ER1" s="1" t="s">
-        <v>100</v>
-      </c>
-      <c r="ES1" s="1" t="s">
-        <v>101</v>
-      </c>
-      <c r="ET1" s="1" t="s">
-        <v>102</v>
-      </c>
-      <c r="EU1" s="1" t="s">
-        <v>103</v>
-      </c>
-      <c r="EV1" s="1" t="s">
-        <v>104</v>
-      </c>
-      <c r="EW1" s="1" t="s">
-        <v>105</v>
-      </c>
-      <c r="EX1" s="1" t="s">
-        <v>106</v>
-      </c>
-      <c r="EY1" s="1" t="s">
-        <v>107</v>
-      </c>
-      <c r="EZ1" s="1" t="s">
-        <v>108</v>
-      </c>
-      <c r="FA1" s="1" t="s">
-        <v>109</v>
-      </c>
-      <c r="FB1" s="1" t="s">
-        <v>110</v>
-      </c>
-      <c r="FC1" s="1" t="s">
-        <v>111</v>
-      </c>
-      <c r="FD1" s="1" t="s">
-        <v>112</v>
-      </c>
-      <c r="FE1" s="1" t="s">
-        <v>113</v>
-      </c>
-      <c r="FF1" s="1" t="s">
-        <v>114</v>
-      </c>
-      <c r="FG1" s="1" t="s">
-        <v>115</v>
-      </c>
-      <c r="FH1" s="1" t="s">
-        <v>116</v>
-      </c>
-      <c r="FI1" s="1" t="s">
-        <v>117</v>
-      </c>
-      <c r="FJ1" s="1" t="s">
-        <v>118</v>
-      </c>
-      <c r="FK1" s="1" t="s">
-        <v>119</v>
-      </c>
-      <c r="FL1" s="1" t="s">
-        <v>120</v>
-      </c>
-      <c r="FM1" s="1" t="s">
-        <v>121</v>
-      </c>
-      <c r="FN1" s="1" t="s">
-        <v>122</v>
-      </c>
-      <c r="FO1" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="FP1" s="1" t="s">
-        <v>124</v>
-      </c>
       <c r="FQ1" s="1" t="s">
-        <v>125</v>
+        <v>171</v>
       </c>
       <c r="FR1" s="1" t="s">
-        <v>126</v>
+        <v>172</v>
       </c>
       <c r="FS1" s="1" t="s">
-        <v>127</v>
+        <v>173</v>
       </c>
       <c r="FT1" s="1" t="s">
-        <v>128</v>
+        <v>174</v>
       </c>
       <c r="FU1" s="1" t="s">
-        <v>129</v>
+        <v>175</v>
       </c>
       <c r="FV1" s="1" t="s">
-        <v>130</v>
+        <v>176</v>
       </c>
       <c r="FW1" s="1" t="s">
-        <v>131</v>
+        <v>177</v>
       </c>
       <c r="FX1" s="1" t="s">
-        <v>132</v>
+        <v>178</v>
       </c>
       <c r="FY1" s="1" t="s">
-        <v>133</v>
+        <v>179</v>
       </c>
       <c r="FZ1" s="1" t="s">
-        <v>134</v>
+        <v>180</v>
       </c>
       <c r="GA1" s="1" t="s">
-        <v>135</v>
+        <v>181</v>
       </c>
       <c r="GB1" s="1" t="s">
-        <v>136</v>
+        <v>182</v>
       </c>
       <c r="GC1" s="1" t="s">
-        <v>137</v>
+        <v>183</v>
       </c>
       <c r="GD1" s="1" t="s">
-        <v>138</v>
+        <v>184</v>
       </c>
       <c r="GE1" s="1" t="s">
-        <v>139</v>
+        <v>185</v>
       </c>
       <c r="GF1" s="1" t="s">
-        <v>140</v>
+        <v>186</v>
       </c>
       <c r="GG1" s="1" t="s">
-        <v>141</v>
+        <v>187</v>
       </c>
       <c r="GH1" s="1" t="s">
-        <v>142</v>
+        <v>188</v>
       </c>
       <c r="GI1" s="1" t="s">
-        <v>143</v>
+        <v>189</v>
       </c>
       <c r="GJ1" s="1" t="s">
-        <v>144</v>
+        <v>190</v>
       </c>
       <c r="GK1" s="1" t="s">
-        <v>145</v>
+        <v>191</v>
       </c>
       <c r="GL1" s="1" t="s">
-        <v>146</v>
+        <v>192</v>
       </c>
       <c r="GM1" s="1" t="s">
-        <v>147</v>
+        <v>193</v>
       </c>
       <c r="GN1" s="1" t="s">
-        <v>148</v>
+        <v>194</v>
       </c>
       <c r="GO1" s="1" t="s">
-        <v>149</v>
+        <v>195</v>
       </c>
       <c r="GP1" s="1" t="s">
-        <v>150</v>
+        <v>196</v>
       </c>
       <c r="GQ1" s="1" t="s">
-        <v>151</v>
+        <v>197</v>
       </c>
       <c r="GR1" s="1" t="s">
-        <v>152</v>
+        <v>198</v>
       </c>
       <c r="GS1" s="1" t="s">
-        <v>153</v>
+        <v>199</v>
       </c>
       <c r="GT1" s="1" t="s">
-        <v>154</v>
+        <v>200</v>
       </c>
       <c r="GU1" s="1" t="s">
-        <v>155</v>
+        <v>201</v>
       </c>
       <c r="GV1" s="1" t="s">
-        <v>156</v>
+        <v>202</v>
       </c>
       <c r="GW1" s="1" t="s">
-        <v>157</v>
-      </c>
-      <c r="HK1" s="1" t="s">
-        <v>171</v>
+        <v>203</v>
+      </c>
+      <c r="GX1" s="1" t="s">
+        <v>204</v>
       </c>
     </row>
-    <row r="2" spans="1:219" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:206" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
-        <v>172</v>
+        <v>205</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>173</v>
+        <v>206</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>233</v>
+        <v>207</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>174</v>
+        <v>208</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>175</v>
+        <v>209</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>175</v>
+        <v>209</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>176</v>
+        <v>210</v>
       </c>
       <c r="I2" s="1" t="s">
-        <v>177</v>
+        <v>211</v>
       </c>
       <c r="J2" s="1" t="s">
-        <v>175</v>
+        <v>209</v>
       </c>
       <c r="K2" s="1" t="s">
-        <v>178</v>
+        <v>212</v>
       </c>
       <c r="L2" s="1" t="s">
-        <v>175</v>
+        <v>209</v>
       </c>
       <c r="M2" s="1" t="s">
-        <v>175</v>
+        <v>209</v>
       </c>
       <c r="N2" s="1" t="s">
-        <v>175</v>
+        <v>209</v>
       </c>
       <c r="O2" s="1" t="s">
-        <v>175</v>
+        <v>209</v>
       </c>
       <c r="P2" s="1" t="s">
-        <v>175</v>
+        <v>209</v>
       </c>
       <c r="Q2" s="1" t="s">
-        <v>175</v>
+        <v>209</v>
       </c>
       <c r="R2" s="1" t="s">
-        <v>175</v>
+        <v>209</v>
       </c>
       <c r="S2" s="1" t="s">
-        <v>175</v>
+        <v>209</v>
       </c>
       <c r="T2" s="1" t="s">
-        <v>175</v>
+        <v>209</v>
       </c>
       <c r="U2" s="1" t="s">
-        <v>175</v>
+        <v>209</v>
       </c>
       <c r="V2" s="1" t="s">
-        <v>179</v>
+        <v>213</v>
       </c>
       <c r="W2" s="1" t="s">
-        <v>179</v>
+        <v>213</v>
       </c>
       <c r="X2" s="1" t="s">
-        <v>179</v>
+        <v>213</v>
       </c>
       <c r="Y2" s="1" t="s">
-        <v>179</v>
+        <v>213</v>
       </c>
       <c r="Z2" s="1" t="s">
-        <v>177</v>
+        <v>211</v>
       </c>
       <c r="AA2" s="1" t="s">
-        <v>175</v>
+        <v>209</v>
       </c>
       <c r="AB2" s="1" t="s">
-        <v>175</v>
+        <v>209</v>
       </c>
       <c r="AC2" s="1" t="s">
-        <v>175</v>
+        <v>209</v>
       </c>
       <c r="AD2" s="1" t="s">
-        <v>175</v>
+        <v>209</v>
       </c>
       <c r="AE2" s="1" t="s">
-        <v>175</v>
+        <v>209</v>
       </c>
       <c r="AF2" s="1" t="s">
-        <v>177</v>
+        <v>211</v>
       </c>
       <c r="AG2" s="1" t="s">
-        <v>180</v>
+        <v>214</v>
       </c>
       <c r="AH2" s="1">
         <v>3</v>
@@ -2745,19 +2736,19 @@
         <v>15</v>
       </c>
       <c r="AJ2" s="1" t="s">
-        <v>177</v>
+        <v>211</v>
       </c>
       <c r="AK2" s="1">
         <v>3</v>
       </c>
       <c r="AL2" s="1" t="s">
-        <v>181</v>
+        <v>215</v>
       </c>
       <c r="AM2" s="1" t="s">
-        <v>177</v>
+        <v>211</v>
       </c>
       <c r="AN2" s="1" t="s">
-        <v>177</v>
+        <v>211</v>
       </c>
       <c r="AO2" s="1">
         <v>5</v>
@@ -2766,7 +2757,7 @@
         <v>60</v>
       </c>
       <c r="AQ2" s="1" t="s">
-        <v>177</v>
+        <v>211</v>
       </c>
       <c r="AR2" s="1">
         <v>6</v>
@@ -2775,7 +2766,7 @@
         <v>30</v>
       </c>
       <c r="AT2" s="1" t="s">
-        <v>177</v>
+        <v>211</v>
       </c>
       <c r="AU2" s="1">
         <v>3</v>
@@ -2784,7 +2775,7 @@
         <v>120</v>
       </c>
       <c r="AW2" s="1" t="s">
-        <v>177</v>
+        <v>211</v>
       </c>
       <c r="AX2" s="1">
         <v>2</v>
@@ -2793,7 +2784,7 @@
         <v>100</v>
       </c>
       <c r="AZ2" s="1" t="s">
-        <v>177</v>
+        <v>211</v>
       </c>
       <c r="BA2" s="1">
         <v>1</v>
@@ -2802,7 +2793,7 @@
         <v>20</v>
       </c>
       <c r="BC2" s="1" t="s">
-        <v>177</v>
+        <v>211</v>
       </c>
       <c r="BD2" s="1">
         <v>1</v>
@@ -2811,454 +2802,457 @@
         <v>20</v>
       </c>
       <c r="BG2" s="1" t="s">
-        <v>182</v>
+        <v>216</v>
       </c>
       <c r="BH2" s="1" t="s">
-        <v>183</v>
+        <v>217</v>
       </c>
       <c r="BI2" s="1" t="s">
-        <v>184</v>
+        <v>218</v>
       </c>
       <c r="BJ2" s="1" t="s">
-        <v>185</v>
+        <v>219</v>
       </c>
       <c r="BK2" s="1" t="s">
-        <v>182</v>
+        <v>216</v>
       </c>
       <c r="BL2" s="1" t="s">
-        <v>177</v>
+        <v>211</v>
       </c>
       <c r="BM2" s="1" t="s">
-        <v>186</v>
+        <v>220</v>
       </c>
       <c r="BN2" s="1" t="s">
-        <v>187</v>
+        <v>221</v>
       </c>
       <c r="BP2" s="1" t="s">
-        <v>185</v>
+        <v>219</v>
       </c>
       <c r="BR2" s="1" t="s">
-        <v>182</v>
+        <v>216</v>
       </c>
       <c r="BS2" s="1" t="s">
-        <v>177</v>
+        <v>211</v>
       </c>
       <c r="BT2" s="1" t="s">
-        <v>186</v>
+        <v>220</v>
       </c>
       <c r="BU2" s="1" t="s">
-        <v>188</v>
+        <v>222</v>
       </c>
       <c r="BV2" s="1" t="s">
-        <v>183</v>
+        <v>217</v>
       </c>
       <c r="BY2" s="1" t="s">
-        <v>177</v>
+        <v>211</v>
       </c>
       <c r="BZ2" s="1" t="s">
+        <v>223</v>
+      </c>
+      <c r="CA2" s="1" t="s">
+        <v>211</v>
+      </c>
+      <c r="CB2" s="1" t="s">
+        <v>211</v>
+      </c>
+      <c r="CC2" s="1" t="s">
+        <v>211</v>
+      </c>
+      <c r="CD2" s="1" t="s">
+        <v>211</v>
+      </c>
+      <c r="CE2" s="1" t="s">
+        <v>211</v>
+      </c>
+      <c r="CF2" s="1" t="s">
+        <v>211</v>
+      </c>
+      <c r="CG2" s="1" t="s">
+        <v>211</v>
+      </c>
+      <c r="CH2" s="1" t="s">
+        <v>224</v>
+      </c>
+      <c r="CI2" s="1" t="s">
+        <v>225</v>
+      </c>
+      <c r="CJ2" s="1" t="s">
+        <v>226</v>
+      </c>
+      <c r="CK2" s="1" t="s">
+        <v>226</v>
+      </c>
+      <c r="CL2" s="1" t="s">
+        <v>226</v>
+      </c>
+      <c r="CM2" s="1" t="s">
+        <v>226</v>
+      </c>
+      <c r="CN2" s="1" t="s">
+        <v>227</v>
+      </c>
+      <c r="CO2" s="1" t="s">
+        <v>228</v>
+      </c>
+      <c r="CP2" s="1" t="s">
+        <v>229</v>
+      </c>
+      <c r="CQ2" s="1" t="s">
+        <v>226</v>
+      </c>
+      <c r="CR2" s="1" t="s">
+        <v>230</v>
+      </c>
+      <c r="CS2" s="1" t="s">
+        <v>231</v>
+      </c>
+      <c r="CT2" s="1" t="s">
+        <v>232</v>
+      </c>
+      <c r="CU2" s="1" t="s">
+        <v>233</v>
+      </c>
+      <c r="CV2" s="1" t="s">
         <v>234</v>
       </c>
-      <c r="CA2" s="1" t="s">
-        <v>177</v>
-      </c>
-      <c r="CB2" s="1" t="s">
-        <v>177</v>
-      </c>
-      <c r="CC2" s="1" t="s">
-        <v>177</v>
-      </c>
-      <c r="CD2" s="1" t="s">
-        <v>177</v>
-      </c>
-      <c r="CE2" s="1" t="s">
-        <v>177</v>
-      </c>
-      <c r="CF2" s="1" t="s">
-        <v>177</v>
-      </c>
-      <c r="CG2" s="1" t="s">
-        <v>177</v>
-      </c>
-      <c r="CH2" s="1" t="s">
+      <c r="CW2" s="1" t="s">
+        <v>234</v>
+      </c>
+      <c r="CX2" s="1" t="s">
         <v>235</v>
       </c>
-      <c r="CI2" s="1" t="s">
+      <c r="CY2" s="1" t="s">
+        <v>235</v>
+      </c>
+      <c r="CZ2" s="1" t="s">
+        <v>235</v>
+      </c>
+      <c r="DA2" s="1" t="s">
+        <v>235</v>
+      </c>
+      <c r="DB2" s="1" t="s">
+        <v>235</v>
+      </c>
+      <c r="DC2" s="1" t="s">
         <v>236</v>
       </c>
-      <c r="CJ2" s="1" t="s">
+      <c r="DD2" s="1" t="s">
+        <v>236</v>
+      </c>
+      <c r="DE2" s="1" t="s">
+        <v>236</v>
+      </c>
+      <c r="DF2" s="1" t="s">
         <v>237</v>
       </c>
-      <c r="CK2" s="1" t="s">
-        <v>237</v>
-      </c>
-      <c r="CL2" s="1" t="s">
-        <v>237</v>
-      </c>
-      <c r="CM2" s="1" t="s">
-        <v>237</v>
-      </c>
-      <c r="CN2" s="1" t="s">
+      <c r="DG2" s="1" t="s">
+        <v>238</v>
+      </c>
+      <c r="DH2" s="1" t="s">
+        <v>239</v>
+      </c>
+      <c r="DI2" s="1" t="s">
+        <v>240</v>
+      </c>
+      <c r="DJ2" s="1" t="s">
         <v>241</v>
       </c>
-      <c r="CO2" s="1" t="s">
+      <c r="DK2" s="1" t="s">
+        <v>211</v>
+      </c>
+      <c r="DL2" s="1" t="s">
+        <v>242</v>
+      </c>
+      <c r="DM2" s="1" t="s">
         <v>243</v>
       </c>
-      <c r="CP2" s="1" t="s">
+      <c r="DN2" s="1" t="s">
+        <v>244</v>
+      </c>
+      <c r="DO2" s="1" t="s">
+        <v>211</v>
+      </c>
+      <c r="DP2" s="1" t="s">
+        <v>211</v>
+      </c>
+      <c r="DQ2" s="1" t="s">
+        <v>211</v>
+      </c>
+      <c r="DR2" s="1" t="s">
+        <v>211</v>
+      </c>
+      <c r="DS2" s="1" t="s">
+        <v>216</v>
+      </c>
+      <c r="DT2" s="1" t="s">
         <v>245</v>
       </c>
-      <c r="CQ2" s="1" t="s">
-        <v>237</v>
-      </c>
-      <c r="CR2" s="1" t="s">
+      <c r="DU2" s="1" t="s">
+        <v>211</v>
+      </c>
+      <c r="DV2" s="1" t="s">
+        <v>211</v>
+      </c>
+      <c r="DW2" s="1" t="s">
+        <v>211</v>
+      </c>
+      <c r="DX2" s="1" t="s">
+        <v>211</v>
+      </c>
+      <c r="DY2" s="1" t="s">
+        <v>211</v>
+      </c>
+      <c r="DZ2" s="1" t="s">
+        <v>246</v>
+      </c>
+      <c r="EA2" s="1" t="s">
+        <v>216</v>
+      </c>
+      <c r="EB2" s="1" t="s">
+        <v>247</v>
+      </c>
+      <c r="EC2" s="1" t="s">
         <v>248</v>
       </c>
-      <c r="CS2" s="1" t="s">
+      <c r="ED2" s="1" t="s">
+        <v>249</v>
+      </c>
+      <c r="EE2" s="1" t="s">
         <v>250</v>
       </c>
-      <c r="CT2" s="1" t="s">
+      <c r="EF2" s="1" t="s">
+        <v>216</v>
+      </c>
+      <c r="EG2" s="1" t="s">
+        <v>251</v>
+      </c>
+      <c r="EH2" s="1" t="s">
         <v>252</v>
       </c>
-      <c r="CU2" s="1" t="s">
+      <c r="EI2" s="1" t="s">
+        <v>216</v>
+      </c>
+      <c r="EJ2" s="1" t="s">
+        <v>253</v>
+      </c>
+      <c r="EK2" s="1" t="s">
+        <v>254</v>
+      </c>
+      <c r="EL2" s="1" t="s">
+        <v>216</v>
+      </c>
+      <c r="EM2" s="1" t="s">
+        <v>255</v>
+      </c>
+      <c r="EN2" s="1" t="s">
+        <v>216</v>
+      </c>
+      <c r="EO2" s="1" t="s">
+        <v>256</v>
+      </c>
+      <c r="EP2" s="1" t="s">
+        <v>257</v>
+      </c>
+      <c r="EQ2" s="1" t="s">
+        <v>258</v>
+      </c>
+      <c r="ER2" s="1" t="s">
+        <v>259</v>
+      </c>
+      <c r="ES2" s="1" t="s">
+        <v>260</v>
+      </c>
+      <c r="ET2" s="1" t="s">
         <v>261</v>
       </c>
-      <c r="CV2" s="1" t="s">
+      <c r="EU2" s="1" t="s">
+        <v>262</v>
+      </c>
+      <c r="EV2" s="1" t="s">
         <v>263</v>
       </c>
-      <c r="CW2" s="1" t="s">
-        <v>263</v>
-      </c>
-      <c r="CX2" s="1" t="s">
-        <v>262</v>
-      </c>
-      <c r="CY2" s="1" t="s">
-        <v>262</v>
-      </c>
-      <c r="CZ2" s="1" t="s">
-        <v>262</v>
-      </c>
-      <c r="DA2" s="1" t="s">
-        <v>262</v>
-      </c>
-      <c r="DB2" s="1" t="s">
-        <v>262</v>
-      </c>
-      <c r="DC2" s="1" t="s">
+      <c r="EW2" s="1" t="s">
+        <v>246</v>
+      </c>
+      <c r="EX2" s="1" t="s">
+        <v>264</v>
+      </c>
+      <c r="EY2" s="1" t="s">
+        <v>216</v>
+      </c>
+      <c r="EZ2" s="1" t="s">
+        <v>211</v>
+      </c>
+      <c r="FA2" s="1" t="s">
+        <v>209</v>
+      </c>
+      <c r="FB2" s="1" t="s">
+        <v>216</v>
+      </c>
+      <c r="FC2" s="1" t="s">
+        <v>211</v>
+      </c>
+      <c r="FD2" s="1" t="s">
+        <v>211</v>
+      </c>
+      <c r="FE2" s="1" t="s">
+        <v>216</v>
+      </c>
+      <c r="FF2" s="1" t="s">
+        <v>265</v>
+      </c>
+      <c r="FG2" s="1" t="s">
+        <v>266</v>
+      </c>
+      <c r="FH2" s="1" t="s">
+        <v>211</v>
+      </c>
+      <c r="FI2" s="1" t="s">
+        <v>211</v>
+      </c>
+      <c r="FJ2" s="1" t="s">
+        <v>211</v>
+      </c>
+      <c r="FK2" s="1" t="s">
+        <v>211</v>
+      </c>
+      <c r="FL2" s="1" t="s">
+        <v>216</v>
+      </c>
+      <c r="FM2" s="1" t="s">
+        <v>219</v>
+      </c>
+      <c r="FN2" s="1" t="s">
+        <v>216</v>
+      </c>
+      <c r="FO2" s="1" t="s">
+        <v>267</v>
+      </c>
+      <c r="FP2" s="1" t="s">
+        <v>267</v>
+      </c>
+      <c r="FQ2" s="1" t="s">
+        <v>268</v>
+      </c>
+      <c r="FR2" s="1" t="s">
         <v>269</v>
       </c>
-      <c r="DD2" s="1" t="s">
-        <v>269</v>
-      </c>
-      <c r="DE2" s="1" t="s">
-        <v>269</v>
-      </c>
-      <c r="DF2" s="1" t="s">
+      <c r="FS2" s="1" t="s">
+        <v>216</v>
+      </c>
+      <c r="FT2" s="1" t="s">
         <v>270</v>
       </c>
-      <c r="DG2" s="1" t="s">
+      <c r="FU2" s="1" t="s">
         <v>271</v>
       </c>
-      <c r="DH2" s="1" t="s">
+      <c r="FV2" s="1" t="s">
+        <v>216</v>
+      </c>
+      <c r="FW2" s="1" t="s">
+        <v>272</v>
+      </c>
+      <c r="FX2" s="1" t="s">
+        <v>273</v>
+      </c>
+      <c r="FY2" s="1" t="s">
+        <v>274</v>
+      </c>
+      <c r="FZ2" s="1" t="s">
+        <v>216</v>
+      </c>
+      <c r="GA2" s="1" t="s">
+        <v>275</v>
+      </c>
+      <c r="GB2" s="1" t="s">
+        <v>267</v>
+      </c>
+      <c r="GC2" s="1" t="s">
+        <v>219</v>
+      </c>
+      <c r="GD2" s="1" t="s">
+        <v>276</v>
+      </c>
+      <c r="GE2" s="1" t="s">
+        <v>216</v>
+      </c>
+      <c r="GF2" s="1" t="s">
+        <v>276</v>
+      </c>
+      <c r="GG2" s="1" t="s">
+        <v>277</v>
+      </c>
+      <c r="GH2" s="1" t="s">
+        <v>216</v>
+      </c>
+      <c r="GI2" s="1" t="s">
+        <v>246</v>
+      </c>
+      <c r="GJ2" s="1" t="s">
+        <v>278</v>
+      </c>
+      <c r="GK2" s="1" t="s">
+        <v>216</v>
+      </c>
+      <c r="GL2" s="1" t="s">
         <v>279</v>
       </c>
-      <c r="DI2" s="1" t="s">
+      <c r="GM2" s="1" t="s">
         <v>280</v>
       </c>
-      <c r="DJ2" s="1" t="s">
+      <c r="GN2" s="1" t="s">
         <v>281</v>
       </c>
-      <c r="DK2" s="1" t="s">
-        <v>177</v>
-      </c>
-      <c r="DL2" s="1" t="s">
+      <c r="GO2" s="1" t="s">
+        <v>216</v>
+      </c>
+      <c r="GP2" s="1" t="s">
         <v>282</v>
       </c>
-      <c r="DM2" s="1" t="s">
+      <c r="GQ2" s="1" t="s">
         <v>283</v>
       </c>
-      <c r="DN2" s="1" t="s">
+      <c r="GR2" s="1" t="s">
         <v>284</v>
       </c>
-      <c r="DO2" s="1" t="s">
-        <v>177</v>
-      </c>
-      <c r="DP2" s="1" t="s">
-        <v>177</v>
-      </c>
-      <c r="DQ2" s="1" t="s">
-        <v>177</v>
-      </c>
-      <c r="DR2" s="1" t="s">
-        <v>177</v>
-      </c>
-      <c r="DS2" s="1" t="s">
-        <v>182</v>
-      </c>
-      <c r="DT2" s="1" t="s">
-        <v>189</v>
-      </c>
-      <c r="DU2" s="1" t="s">
-        <v>177</v>
-      </c>
-      <c r="DV2" s="1" t="s">
-        <v>177</v>
-      </c>
-      <c r="DW2" s="1" t="s">
-        <v>177</v>
-      </c>
-      <c r="DX2" s="1" t="s">
-        <v>177</v>
-      </c>
-      <c r="DY2" s="1" t="s">
-        <v>177</v>
-      </c>
-      <c r="DZ2" s="1" t="s">
-        <v>190</v>
-      </c>
-      <c r="EA2" s="1" t="s">
-        <v>182</v>
-      </c>
-      <c r="EB2" s="1" t="s">
-        <v>191</v>
-      </c>
-      <c r="EC2" s="1" t="s">
-        <v>192</v>
-      </c>
-      <c r="ED2" s="1" t="s">
-        <v>193</v>
-      </c>
-      <c r="EE2" s="1" t="s">
-        <v>194</v>
-      </c>
-      <c r="EF2" s="1" t="s">
-        <v>182</v>
-      </c>
-      <c r="EG2" s="1" t="s">
-        <v>195</v>
-      </c>
-      <c r="EH2" s="1" t="s">
-        <v>196</v>
-      </c>
-      <c r="EI2" s="1" t="s">
-        <v>182</v>
-      </c>
-      <c r="EJ2" s="1" t="s">
-        <v>197</v>
-      </c>
-      <c r="EK2" s="1" t="s">
-        <v>198</v>
-      </c>
-      <c r="EL2" s="1" t="s">
-        <v>182</v>
-      </c>
-      <c r="EM2" s="1" t="s">
-        <v>199</v>
-      </c>
-      <c r="EN2" s="1" t="s">
-        <v>182</v>
-      </c>
-      <c r="EO2" s="1" t="s">
-        <v>200</v>
-      </c>
-      <c r="EP2" s="1" t="s">
-        <v>201</v>
-      </c>
-      <c r="EQ2" s="1" t="s">
-        <v>202</v>
-      </c>
-      <c r="ER2" s="1" t="s">
-        <v>203</v>
-      </c>
-      <c r="ES2" s="1" t="s">
-        <v>204</v>
-      </c>
-      <c r="ET2" s="1" t="s">
-        <v>205</v>
-      </c>
-      <c r="EU2" s="1" t="s">
-        <v>206</v>
-      </c>
-      <c r="EV2" s="1" t="s">
-        <v>207</v>
-      </c>
-      <c r="EW2" s="1" t="s">
-        <v>190</v>
-      </c>
-      <c r="EX2" s="1" t="s">
-        <v>208</v>
-      </c>
-      <c r="EY2" s="1" t="s">
-        <v>182</v>
-      </c>
-      <c r="EZ2" s="1" t="s">
-        <v>177</v>
-      </c>
-      <c r="FA2" s="1" t="s">
-        <v>175</v>
-      </c>
-      <c r="FB2" s="1" t="s">
-        <v>182</v>
-      </c>
-      <c r="FC2" s="1" t="s">
-        <v>177</v>
-      </c>
-      <c r="FD2" s="1" t="s">
-        <v>177</v>
-      </c>
-      <c r="FE2" s="1" t="s">
-        <v>182</v>
-      </c>
-      <c r="FF2" s="1" t="s">
-        <v>209</v>
-      </c>
-      <c r="FG2" s="1" t="s">
-        <v>210</v>
-      </c>
-      <c r="FH2" s="1" t="s">
-        <v>177</v>
-      </c>
-      <c r="FI2" s="1" t="s">
-        <v>177</v>
-      </c>
-      <c r="FJ2" s="1" t="s">
-        <v>177</v>
-      </c>
-      <c r="FK2" s="1" t="s">
-        <v>177</v>
-      </c>
-      <c r="FL2" s="1" t="s">
-        <v>182</v>
-      </c>
-      <c r="FM2" s="1" t="s">
-        <v>185</v>
-      </c>
-      <c r="FN2" s="1" t="s">
-        <v>182</v>
-      </c>
-      <c r="FO2" s="1" t="s">
-        <v>211</v>
-      </c>
-      <c r="FP2" s="1" t="s">
-        <v>211</v>
-      </c>
-      <c r="FQ2" s="1" t="s">
-        <v>212</v>
-      </c>
-      <c r="FR2" s="1" t="s">
-        <v>213</v>
-      </c>
-      <c r="FS2" s="1" t="s">
-        <v>182</v>
-      </c>
-      <c r="FT2" s="1" t="s">
-        <v>214</v>
-      </c>
-      <c r="FU2" s="1" t="s">
-        <v>215</v>
-      </c>
-      <c r="FV2" s="1" t="s">
-        <v>182</v>
-      </c>
-      <c r="FW2" s="1" t="s">
-        <v>216</v>
-      </c>
-      <c r="FX2" s="1" t="s">
-        <v>217</v>
-      </c>
-      <c r="FY2" s="1" t="s">
-        <v>218</v>
-      </c>
-      <c r="FZ2" s="1" t="s">
-        <v>182</v>
-      </c>
-      <c r="GA2" s="1" t="s">
-        <v>219</v>
-      </c>
-      <c r="GB2" s="1" t="s">
-        <v>211</v>
-      </c>
-      <c r="GC2" s="1" t="s">
-        <v>185</v>
-      </c>
-      <c r="GD2" s="1" t="s">
-        <v>220</v>
-      </c>
-      <c r="GE2" s="1" t="s">
-        <v>182</v>
-      </c>
-      <c r="GF2" s="1" t="s">
-        <v>220</v>
-      </c>
-      <c r="GG2" s="1" t="s">
-        <v>221</v>
-      </c>
-      <c r="GH2" s="1" t="s">
-        <v>182</v>
-      </c>
-      <c r="GI2" s="1" t="s">
-        <v>190</v>
-      </c>
-      <c r="GJ2" s="1" t="s">
-        <v>223</v>
-      </c>
-      <c r="GK2" s="1" t="s">
-        <v>182</v>
-      </c>
-      <c r="GL2" s="1" t="s">
-        <v>224</v>
-      </c>
-      <c r="GM2" s="1" t="s">
-        <v>225</v>
-      </c>
-      <c r="GN2" s="1" t="s">
-        <v>222</v>
-      </c>
-      <c r="GO2" s="1" t="s">
-        <v>182</v>
-      </c>
-      <c r="GP2" s="1" t="s">
-        <v>226</v>
-      </c>
-      <c r="GQ2" s="1" t="s">
-        <v>227</v>
-      </c>
-      <c r="GR2" s="1" t="s">
-        <v>228</v>
-      </c>
       <c r="GS2" s="1" t="s">
-        <v>229</v>
+        <v>285</v>
       </c>
       <c r="GT2" s="1" t="s">
-        <v>230</v>
+        <v>286</v>
       </c>
       <c r="GU2" s="1" t="s">
-        <v>231</v>
+        <v>287</v>
       </c>
       <c r="GV2" s="1" t="s">
-        <v>232</v>
+        <v>288</v>
       </c>
       <c r="GW2" s="1" t="s">
-        <v>190</v>
+        <v>246</v>
+      </c>
+      <c r="GX2" t="s">
+        <v>289</v>
       </c>
     </row>
   </sheetData>
-  <dataValidations count="68">
+  <dataValidations count="63">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E2" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"Belum Menikah,Menikah,Cerai Mati,Cerai Hidup"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I2:J2 F2:G2 CA2:CG2 BY2 FH2:FK2 FC2:FD2 EZ2:FA2 DU2:DY2 BS2 BL2 BC2 AZ2 AW2 AT2 AQ2 AM2:AN2 AJ2 Z2:AF2 L2:U2 DK2 DO2:DR2" xr:uid="{00000000-0002-0000-0000-000001000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F2:G2 I2:J2 L2:U2 Z2:AF2 AJ2 AM2:AN2 AQ2 AT2 AW2 AZ2 BC2 BL2 BS2 BY2 CA2:CG2 DK2 DO2:DR2 DU2:DY2 EZ2:FA2 FC2:FD2 FH2:FK2" xr:uid="{00000000-0002-0000-0000-000001000000}">
       <formula1>"Ya,Tidak"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H2" xr:uid="{00000000-0002-0000-0000-000002000000}">
       <formula1>"Non disabilitas,Penyandang disabilitas"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AG2 K2 GV2 GS2 EE2 DT2" xr:uid="{00000000-0002-0000-0000-000003000000}"/>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K2 AG2 DT2 EE2 GS2 GV2 DJ2 DF2:DG2 CU2:DB2" xr:uid="{00000000-0002-0000-0000-000003000000}"/>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="V2:Y2" xr:uid="{00000000-0002-0000-0000-000004000000}">
       <formula1>"Tidak sama sekali,Kurang dari 1 minggu,Lebih dari 1 minggu,Hampir setiap hari"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AL2" xr:uid="{00000000-0002-0000-0000-000005000000}">
       <formula1>"1 s.d &lt;10 tahun lalu,10 s.d &lt;15 tahun lalu,15 tahun lalu atau lebih"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BK2 BG2 GO2 GK2 GH2 GE2 FZ2 FV2 FS2 FN2 FL2 FE2 FB2 EY2 EN2 EL2 EI2 EF2 EA2 DS2 BQ2:BR2" xr:uid="{00000000-0002-0000-0000-000006000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BG2 BK2 BQ2:BR2 DS2 EA2 EF2 EI2 EL2 EN2 EY2 FB2 FE2 FL2 FN2 FS2 FV2 FZ2 GE2 GH2 GK2 GO2" xr:uid="{00000000-0002-0000-0000-000006000000}">
       <formula1>"True,False"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DZ2" xr:uid="{00000000-0002-0000-0000-000007000000}">
@@ -3366,117 +3360,67 @@
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="GW2" xr:uid="{00000000-0002-0000-0000-000029000000}">
       <formula1>"Normal,Tidak Normal"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BZ2" xr:uid="{00000000-0002-0000-0000-00002F000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BZ2" xr:uid="{00000000-0002-0000-0000-00002A000000}">
       <formula1>"Benar semua,Salah satu/Dua,Tidak Tahu"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CH2" xr:uid="{00000000-0002-0000-0000-000030000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CH2" xr:uid="{00000000-0002-0000-0000-00002B000000}">
       <formula1>"Tidak terkendali/tak teratur (perlu pencahar),Kadang-kadang tak terkendali (1 x / minggu),Terkendali teratur"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CI2" xr:uid="{00000000-0002-0000-0000-000031000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CI2" xr:uid="{00000000-0002-0000-0000-00002C000000}">
       <formula1>"Tak terkendali atau pakai kateter,Kadang-kadang tak terkendali (hanya 1 x / 24 jam),Mandiri"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CJ2" xr:uid="{D5F9328F-CFE0-3E42-B6C5-718CA619F09B}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CJ2" xr:uid="{00000000-0002-0000-0000-00002D000000}">
       <formula1>"Mandiri,Butuh pertolongan orang lain"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CK2" xr:uid="{2DC01EBC-833D-B248-8F23-B5CE5DC04C49}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CK2" xr:uid="{00000000-0002-0000-0000-00002E000000}">
       <formula1>"Tergantung pertolongan orang lain,Perlu pertolongan pada beberapa kegiatan tetapi dapat mengerjakan sendiri beberapa kegiatan yang lain,Mandiri"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CL2" xr:uid="{D90C7BBE-572E-8C4E-9249-FBD9094A4C67}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CL2" xr:uid="{00000000-0002-0000-0000-00002F000000}">
       <formula1>"Tidak mampu,Perlu ditolong memotong makanan,Mandiri"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CM2" xr:uid="{3E00A2DE-C4E4-5A4A-B588-596FE1B218FF}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CM2" xr:uid="{00000000-0002-0000-0000-000030000000}">
       <formula1>"Tidak mampu,Perlu banyak bantuan untuk bias duduk (2 orang),Bantuan minimal 1 orang,Mandiri"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CN2" xr:uid="{04314765-AF8B-3549-9476-48F529B74C37}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CN2" xr:uid="{00000000-0002-0000-0000-000031000000}">
       <formula1>"Tidak mampu,Bisa (pindah) dengan kursi roda,Bantuan minimal 1 orang,Mandiri"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CO2" xr:uid="{B81AE730-9A28-D842-8AA5-04FE085F008E}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CO2" xr:uid="{00000000-0002-0000-0000-000032000000}">
       <formula1>"Tergantung orang lain,Sebagian dibantu (misalnya: mengancing baju),Mandiri"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CP2" xr:uid="{5DB2E062-3448-1D4D-B277-DEC2964D83FD}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CP2" xr:uid="{00000000-0002-0000-0000-000033000000}">
       <formula1>"Tidak mampu,Butuh pertolongan,Mandiri"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CQ2" xr:uid="{E3168C9C-E69C-2842-A9D2-61F77E74E63A}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CQ2" xr:uid="{00000000-0002-0000-0000-000034000000}">
       <formula1>"Tergantung orang lain,Mandiri"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CR2" xr:uid="{2AD5FD51-2487-F946-A59E-66EC8F2B18FF}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CR2" xr:uid="{00000000-0002-0000-0000-000035000000}">
       <formula1>"SUDAH DITANYAKAN"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CS2" xr:uid="{5D02A377-1B01-6045-8B5C-A1DAAB2E1A25}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CS2" xr:uid="{00000000-0002-0000-0000-000036000000}">
       <formula1>"Benar,Salah"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CT2" xr:uid="{BCA8F2B4-8F7A-784C-A25B-401D65D9303E}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CT2" xr:uid="{00000000-0002-0000-0000-000037000000}">
       <formula1>"Benar 1 kata,Benar 2 Kata,Benar semua kata,Tidak dapat mengingat/mengulang kata"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CU2" xr:uid="{6687EA59-EF11-E449-8DBB-7EB5708FB3E8}">
-      <mc:AlternateContent xmlns:x12ac="http://schemas.microsoft.com/office/spreadsheetml/2011/1/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-        <mc:Choice Requires="x12ac">
-          <x12ac:list>"Ya, Berubah","Tidak, Berubah",Tidak Tahu</x12ac:list>
-        </mc:Choice>
-        <mc:Fallback>
-          <formula1>"Ya, Berubah,Tidak, Berubah,Tidak Tahu"</formula1>
-        </mc:Fallback>
-      </mc:AlternateContent>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CV2:DB2" xr:uid="{CAD820FA-74F9-4E40-802A-0B5BF221CCC3}">
-      <mc:AlternateContent xmlns:x12ac="http://schemas.microsoft.com/office/spreadsheetml/2011/1/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-        <mc:Choice Requires="x12ac">
-          <x12ac:list>"Ya, Berubah",Tidak Berubah,Tidak Tahu</x12ac:list>
-        </mc:Choice>
-        <mc:Fallback>
-          <formula1>"Ya, Berubah,Tidak Berubah,Tidak Tahu"</formula1>
-        </mc:Fallback>
-      </mc:AlternateContent>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DC2:DD2" xr:uid="{8624A411-ABFC-AD42-9F33-B885D13D9656}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DC2:DD2" xr:uid="{00000000-0002-0000-0000-00003A000000}">
       <formula1>"Bertahan 10 detik,Tidak bertahan 10 detik,Tidak dilakukan"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DE2" xr:uid="{27C5DDB0-8CF7-684B-A261-24A7DB1D3F89}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DE2" xr:uid="{00000000-0002-0000-0000-00003B000000}">
       <formula1>"Bertahan 10 detik,Bertahan 3 - 9.99 detik,Bertahan &lt; 3 detik"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DF2" xr:uid="{F158B156-CDAF-B64E-9412-DC98B28AAB2D}">
-      <mc:AlternateContent xmlns:x12ac="http://schemas.microsoft.com/office/spreadsheetml/2011/1/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-        <mc:Choice Requires="x12ac">
-          <x12ac:list>"4,82 detik",4.83 - 6.20 detik,6.21 - 8.70 detik,"&gt;8,70 detik",Tidak dapat menyelesaikan</x12ac:list>
-        </mc:Choice>
-        <mc:Fallback>
-          <formula1>"4,82 detik,4.83 - 6.20 detik,6.21 - 8.70 detik,&gt;8,70 detik,Tidak dapat menyelesaikan"</formula1>
-        </mc:Fallback>
-      </mc:AlternateContent>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DG2" xr:uid="{FA3B3CBF-2776-6F44-B496-E4AACD7B8DE5}">
-      <mc:AlternateContent xmlns:x12ac="http://schemas.microsoft.com/office/spreadsheetml/2011/1/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-        <mc:Choice Requires="x12ac">
-          <x12ac:list>&lt;11.19 detik,"11.2 - 13,69 detik",13.7 - 16.69 detik,16.7 - 59.9 detik,&gt;60 detik atau tidak menyelesaikan</x12ac:list>
-        </mc:Choice>
-        <mc:Fallback>
-          <formula1>"&lt;11.19 detik,11.2 - 13,69 detik,13.7 - 16.69 detik,16.7 - 59.9 detik,&gt;60 detik atau tidak menyelesaikan"</formula1>
-        </mc:Fallback>
-      </mc:AlternateContent>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DH2" xr:uid="{E7F1499F-D1E2-2A45-B604-5C8D9095D6FE}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DH2" xr:uid="{00000000-0002-0000-0000-00003E000000}">
       <formula1>"Nafsu Makan Yang Sangat Berkurang,Nafsu Makan Sedikit Berkurang,Nafsu Makan Biasa saja"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DI2" xr:uid="{7BA75764-D8E9-1244-889F-533206C29E1E}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DI2" xr:uid="{00000000-0002-0000-0000-00003F000000}">
       <formula1>"Penurunan BB &gt; 3 Kg,Tidak Tahu,Penurunan BB antara 1 - 3 Kg"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DJ2" xr:uid="{B6F2B7AB-5238-904C-898F-2DD19DAB3A37}">
-      <mc:AlternateContent xmlns:x12ac="http://schemas.microsoft.com/office/spreadsheetml/2011/1/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-        <mc:Choice Requires="x12ac">
-          <x12ac:list>Harus berbaring di tempat tidur atau menggunakan kursi roda,"Bisa bangun dari tempat tidur atau kursi roda, tetapi tidak bisa keluar rumah",Bisa bepergian keluar rumah</x12ac:list>
-        </mc:Choice>
-        <mc:Fallback>
-          <formula1>"Harus berbaring di tempat tidur atau menggunakan kursi roda,Bisa bangun dari tempat tidur atau kursi roda, tetapi tidak bisa keluar rumah,Bisa bepergian keluar rumah"</formula1>
-        </mc:Fallback>
-      </mc:AlternateContent>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DL2" xr:uid="{2747DE2C-9959-3048-987D-CB575AA915B8}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DL2" xr:uid="{00000000-0002-0000-0000-000041000000}">
       <formula1>"Dementia atau depresi berat,Demensia/kepikunan ringan,Tidak ada masalah psikologis"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DM2" xr:uid="{5F47AFFC-E088-F741-819D-BC4A4B3B866E}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DM2" xr:uid="{00000000-0002-0000-0000-000042000000}">
       <formula1>"IMT &lt;19,IMT 19 - &lt;21,IMT 21 - &lt;23,IMT &gt;= 23"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DN2" xr:uid="{DC939003-7519-6246-A4A2-66B3FBE91AAA}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DN2" xr:uid="{00000000-0002-0000-0000-000043000000}">
       <formula1>"&lt;31 cm,&gt;= 31 cm"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Here is a suggested commit message for the changes made:
```text
docs: add Excel column usage cleanup reports and utility script

- Created cleanup analysis reports for 'remaja', 'dewasa', 'anak', and 'lansia' datasets to identify unused columns.
- Saved cleanup reports under `dist/dataset/excel_cleanup.md` and the `dataset/` directory.
- Added a reusable relative-path analysis utility script `scripts/read_excel.py` to allow running programmatic Excel column usage checks on the datasets.
```
</commit_message>
<xml_diff>
--- a/dataset/lansia.xlsx
+++ b/dataset/lansia.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10531"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10613"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/macbokprom12021/PycharmProjects/CKG-Helper/dataset/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1BD2E58A-9B45-1843-ADA0-EEA4206E484D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A5F81D03-7DA6-6B48-825E-C4ACE42E54E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="780" windowWidth="36000" windowHeight="21080" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4500" yWindow="-21000" windowWidth="36000" windowHeight="21000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,37 +25,7 @@
     <author>Microsoft Office User</author>
   </authors>
   <commentList>
-    <comment ref="F1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000001000000}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="12"/>
-            <color theme="1"/>
-            <rFont val="Aptos Narrow"/>
-            <family val="2"/>
-            <scheme val="minor"/>
-          </rPr>
-          <t>Microsoft Office User:
-wajib diisi jika status_perkawinan selain Menikah</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="G1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000002000000}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="12"/>
-            <color theme="1"/>
-            <rFont val="Aptos Narrow"/>
-            <family val="2"/>
-            <scheme val="minor"/>
-          </rPr>
-          <t>Microsoft Office User:
-khusus perempuan</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="AA1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000003000000}">
+    <comment ref="W1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000003000000}">
       <text>
         <r>
           <rPr>
@@ -70,7 +40,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AG1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000004000000}">
+    <comment ref="AC1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000004000000}">
       <text>
         <r>
           <rPr>
@@ -85,7 +55,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AH1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000005000000}">
+    <comment ref="AD1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000005000000}">
       <text>
         <r>
           <rPr>
@@ -101,7 +71,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AI1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000006000000}">
+    <comment ref="AE1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000006000000}">
       <text>
         <r>
           <rPr>
@@ -117,7 +87,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AJ1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000007000000}">
+    <comment ref="AF1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000007000000}">
       <text>
         <r>
           <rPr>
@@ -132,7 +102,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AK1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000008000000}">
+    <comment ref="AG1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000008000000}">
       <text>
         <r>
           <rPr>
@@ -147,7 +117,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AL1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000009000000}">
+    <comment ref="AH1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000009000000}">
       <text>
         <r>
           <rPr>
@@ -163,7 +133,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AO1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00000A000000}">
+    <comment ref="AK1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00000A000000}">
       <text>
         <r>
           <rPr>
@@ -178,7 +148,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AP1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00000B000000}">
+    <comment ref="AL1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00000B000000}">
       <text>
         <r>
           <rPr>
@@ -193,7 +163,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AR1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00000C000000}">
+    <comment ref="AN1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00000C000000}">
       <text>
         <r>
           <rPr>
@@ -208,7 +178,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AS1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00000D000000}">
+    <comment ref="AO1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00000D000000}">
       <text>
         <r>
           <rPr>
@@ -223,7 +193,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AU1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00000E000000}">
+    <comment ref="AQ1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00000E000000}">
       <text>
         <r>
           <rPr>
@@ -238,7 +208,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AV1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00000F000000}">
+    <comment ref="AR1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00000F000000}">
       <text>
         <r>
           <rPr>
@@ -253,7 +223,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AX1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000010000000}">
+    <comment ref="AT1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000010000000}">
       <text>
         <r>
           <rPr>
@@ -268,7 +238,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AY1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000011000000}">
+    <comment ref="AU1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000011000000}">
       <text>
         <r>
           <rPr>
@@ -283,7 +253,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="BA1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000012000000}">
+    <comment ref="AW1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000012000000}">
       <text>
         <r>
           <rPr>
@@ -298,7 +268,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="BB1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000013000000}">
+    <comment ref="AX1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000013000000}">
       <text>
         <r>
           <rPr>
@@ -313,7 +283,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="BD1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000014000000}">
+    <comment ref="AZ1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000014000000}">
       <text>
         <r>
           <rPr>
@@ -328,7 +298,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="BE1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000015000000}">
+    <comment ref="BA1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000015000000}">
       <text>
         <r>
           <rPr>
@@ -343,7 +313,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="BM1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000016000000}">
+    <comment ref="BH1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000016000000}">
       <text>
         <r>
           <rPr>
@@ -358,7 +328,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="BN1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000017000000}">
+    <comment ref="BI1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000017000000}">
       <text>
         <r>
           <rPr>
@@ -373,7 +343,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="BO1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000018000000}">
+    <comment ref="BJ1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000018000000}">
       <text>
         <r>
           <rPr>
@@ -388,7 +358,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="BT1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000019000000}">
+    <comment ref="BN1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000019000000}">
       <text>
         <r>
           <rPr>
@@ -403,7 +373,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="DZ1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00001A000000}">
+    <comment ref="DS1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00001A000000}">
       <text>
         <r>
           <rPr>
@@ -418,7 +388,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="EC1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00001B000000}">
+    <comment ref="DU1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00001B000000}">
       <text>
         <r>
           <rPr>
@@ -433,7 +403,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="EH1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00001C000000}">
+    <comment ref="DY1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00001C000000}">
       <text>
         <r>
           <rPr>
@@ -448,7 +418,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="EK1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00001D000000}">
+    <comment ref="EA1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00001D000000}">
       <text>
         <r>
           <rPr>
@@ -463,7 +433,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="ER1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00001E000000}">
+    <comment ref="EF1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00001E000000}">
       <text>
         <r>
           <rPr>
@@ -478,7 +448,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="ET1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00001F000000}">
+    <comment ref="EH1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00001F000000}">
       <text>
         <r>
           <rPr>
@@ -493,7 +463,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="EU1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000020000000}">
+    <comment ref="EI1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000020000000}">
       <text>
         <r>
           <rPr>
@@ -508,7 +478,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="EV1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000021000000}">
+    <comment ref="EJ1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000021000000}">
       <text>
         <r>
           <rPr>
@@ -523,7 +493,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="EW1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000022000000}">
+    <comment ref="EK1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000022000000}">
       <text>
         <r>
           <rPr>
@@ -538,7 +508,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="FG1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000023000000}">
+    <comment ref="ER1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000023000000}">
       <text>
         <r>
           <rPr>
@@ -553,7 +523,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="FY1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000024000000}">
+    <comment ref="FF1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000024000000}">
       <text>
         <r>
           <rPr>
@@ -573,7 +543,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="389" uniqueCount="289">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="342" uniqueCount="265">
   <si>
     <t>batas_awal</t>
   </si>
@@ -584,18 +554,9 @@
     <t>nama</t>
   </si>
   <si>
-    <t>nik</t>
-  </si>
-  <si>
     <t>status_perkawinan</t>
   </si>
   <si>
-    <t>rencana_menikah</t>
-  </si>
-  <si>
-    <t>sedang_hamil</t>
-  </si>
-  <si>
     <t>disabilitas</t>
   </si>
   <si>
@@ -635,9 +596,6 @@
     <t>kolesterol_tinggi</t>
   </si>
   <si>
-    <t>pernah_seks</t>
-  </si>
-  <si>
     <t>tidak_bersemangat</t>
   </si>
   <si>
@@ -746,9 +704,6 @@
     <t>menit_olahraga_berat</t>
   </si>
   <si>
-    <t>periksa_gizi_laki</t>
-  </si>
-  <si>
     <t>berat_badan</t>
   </si>
   <si>
@@ -779,9 +734,6 @@
     <t>gula_darah_pp</t>
   </si>
   <si>
-    <t>periksa_tensi</t>
-  </si>
-  <si>
     <t>pernah_hipertensi</t>
   </si>
   <si>
@@ -938,9 +890,6 @@
     <t>depresi_lanjutan_4</t>
   </si>
   <si>
-    <t>periksa_risiko_tbc</t>
-  </si>
-  <si>
     <t>pernah_batuk_tidak_sembuh</t>
   </si>
   <si>
@@ -962,9 +911,6 @@
     <t>hasil_rontgen</t>
   </si>
   <si>
-    <t>periksa_tbc</t>
-  </si>
-  <si>
     <t>kontak_tbc</t>
   </si>
   <si>
@@ -977,33 +923,21 @@
     <t>hasil_pemeriksaan_tbc</t>
   </si>
   <si>
-    <t>periksa_frambusia</t>
-  </si>
-  <si>
     <t>ada_papul</t>
   </si>
   <si>
     <t>hasil_pemeriksaan_rdt</t>
   </si>
   <si>
-    <t>periksa_kusta</t>
-  </si>
-  <si>
     <t>bercak_putih</t>
   </si>
   <si>
     <t>hasil_bta</t>
   </si>
   <si>
-    <t>periksa_skabies</t>
-  </si>
-  <si>
     <t>ada_ruam</t>
   </si>
   <si>
-    <t>periksa_telinga_mata</t>
-  </si>
-  <si>
     <t>serumen_impaksi</t>
   </si>
   <si>
@@ -1034,27 +968,18 @@
     <t>pupil</t>
   </si>
   <si>
-    <t>periksa_karies</t>
-  </si>
-  <si>
     <t>gigi_karies</t>
   </si>
   <si>
     <t>gigi_hilang</t>
   </si>
   <si>
-    <t>periksa_periodontal</t>
-  </si>
-  <si>
     <t>penyakit_periodontal</t>
   </si>
   <si>
     <t>gigi_goyang</t>
   </si>
   <si>
-    <t>periksa_ppok</t>
-  </si>
-  <si>
     <t>ppok_merokok</t>
   </si>
   <si>
@@ -1073,15 +998,9 @@
     <t>periksa_spirometri</t>
   </si>
   <si>
-    <t>periksa_co</t>
-  </si>
-  <si>
     <t>kadar_co</t>
   </si>
   <si>
-    <t>periksa_lipid</t>
-  </si>
-  <si>
     <t>kolesterol</t>
   </si>
   <si>
@@ -1094,18 +1013,12 @@
     <t>trigliserida</t>
   </si>
   <si>
-    <t>periksa_fibrosis</t>
-  </si>
-  <si>
     <t>sgot</t>
   </si>
   <si>
     <t>trombosit</t>
   </si>
   <si>
-    <t>periksa_hepatitis</t>
-  </si>
-  <si>
     <t>hepatitis_b</t>
   </si>
   <si>
@@ -1115,9 +1028,6 @@
     <t>vl_hepatitis_c</t>
   </si>
   <si>
-    <t>periksa_fungsi_ginjal</t>
-  </si>
-  <si>
     <t>kreatinin</t>
   </si>
   <si>
@@ -1130,27 +1040,18 @@
     <t>e_lfg</t>
   </si>
   <si>
-    <t>periksa_kerusakan_ginjal</t>
-  </si>
-  <si>
     <t>albumin</t>
   </si>
   <si>
     <t>kreatinin_urin</t>
   </si>
   <si>
-    <t>periksa_jantung</t>
-  </si>
-  <si>
     <t>ekg</t>
   </si>
   <si>
     <t>pemeriksaan_ekg</t>
   </si>
   <si>
-    <t>periksa_kanker_usus</t>
-  </si>
-  <si>
     <t>bersedia_colok_dubur</t>
   </si>
   <si>
@@ -1158,9 +1059,6 @@
   </si>
   <si>
     <t>darah_samar</t>
-  </si>
-  <si>
-    <t>periksa_kanker_paru</t>
   </si>
   <si>
     <t>kanker_paru</t>
@@ -1841,176 +1739,153 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:GX2"/>
+  <dimension ref="A1:FZ2"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="17.5" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="12.6640625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="11.5" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.5" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="16.6640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="15.83203125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="15.83203125" customWidth="1"/>
-    <col min="8" max="9" width="10.83203125" customWidth="1"/>
-    <col min="10" max="10" width="8.1640625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="21" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="16" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.5" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="19.5" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="13.83203125" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="11.5" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="16.5" bestFit="1" customWidth="1"/>
-    <col min="18" max="19" width="10.83203125" customWidth="1"/>
-    <col min="20" max="20" width="14.5" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="14.5" customWidth="1"/>
-    <col min="22" max="22" width="17" bestFit="1" customWidth="1"/>
-    <col min="23" max="25" width="15.5" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="23.1640625" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="16.83203125" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="19.1640625" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="11.5" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="5.33203125" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="10.83203125" customWidth="1"/>
-    <col min="32" max="32" width="25.1640625" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="49" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="12.33203125" bestFit="1" customWidth="1"/>
-    <col min="35" max="35" width="13.1640625" bestFit="1" customWidth="1"/>
-    <col min="36" max="36" width="14.5" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="23.6640625" bestFit="1" customWidth="1"/>
-    <col min="38" max="38" width="13.83203125" bestFit="1" customWidth="1"/>
-    <col min="39" max="39" width="23" bestFit="1" customWidth="1"/>
-    <col min="40" max="40" width="16.6640625" bestFit="1" customWidth="1"/>
-    <col min="41" max="41" width="12.6640625" bestFit="1" customWidth="1"/>
-    <col min="42" max="42" width="14.33203125" bestFit="1" customWidth="1"/>
-    <col min="43" max="43" width="17.1640625" bestFit="1" customWidth="1"/>
-    <col min="44" max="44" width="13.1640625" bestFit="1" customWidth="1"/>
-    <col min="45" max="45" width="14.83203125" bestFit="1" customWidth="1"/>
-    <col min="46" max="46" width="17.83203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="16.6640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="6" width="10.83203125" customWidth="1"/>
+    <col min="7" max="7" width="8.1640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="21" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="16" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="13.5" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="19.5" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="13.83203125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="11.5" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="16.5" bestFit="1" customWidth="1"/>
+    <col min="15" max="16" width="10.83203125" customWidth="1"/>
+    <col min="17" max="17" width="14.5" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="17" bestFit="1" customWidth="1"/>
+    <col min="19" max="21" width="15.5" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="23.1640625" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="16.83203125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="19.1640625" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="11.5" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="5.33203125" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="10.83203125" customWidth="1"/>
+    <col min="28" max="28" width="25.1640625" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="49" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="12.33203125" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="13.1640625" bestFit="1" customWidth="1"/>
+    <col min="32" max="32" width="14.5" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="23.6640625" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="13.83203125" bestFit="1" customWidth="1"/>
+    <col min="35" max="35" width="23" bestFit="1" customWidth="1"/>
+    <col min="36" max="36" width="16.6640625" bestFit="1" customWidth="1"/>
+    <col min="37" max="37" width="12.6640625" bestFit="1" customWidth="1"/>
+    <col min="38" max="38" width="14.33203125" bestFit="1" customWidth="1"/>
+    <col min="39" max="39" width="17.1640625" bestFit="1" customWidth="1"/>
+    <col min="40" max="40" width="13.1640625" bestFit="1" customWidth="1"/>
+    <col min="41" max="41" width="14.83203125" bestFit="1" customWidth="1"/>
+    <col min="42" max="42" width="17.83203125" bestFit="1" customWidth="1"/>
+    <col min="43" max="43" width="13.83203125" bestFit="1" customWidth="1"/>
+    <col min="44" max="44" width="15.5" bestFit="1" customWidth="1"/>
+    <col min="45" max="45" width="16" bestFit="1" customWidth="1"/>
+    <col min="46" max="46" width="10.83203125" customWidth="1"/>
     <col min="47" max="47" width="13.83203125" bestFit="1" customWidth="1"/>
-    <col min="48" max="48" width="15.5" bestFit="1" customWidth="1"/>
-    <col min="49" max="49" width="16" bestFit="1" customWidth="1"/>
-    <col min="50" max="50" width="10.83203125" customWidth="1"/>
-    <col min="51" max="51" width="13.83203125" bestFit="1" customWidth="1"/>
-    <col min="52" max="52" width="18.33203125" bestFit="1" customWidth="1"/>
-    <col min="53" max="53" width="14.33203125" bestFit="1" customWidth="1"/>
-    <col min="54" max="54" width="16" bestFit="1" customWidth="1"/>
-    <col min="55" max="55" width="18.33203125" bestFit="1" customWidth="1"/>
-    <col min="56" max="56" width="12.1640625" bestFit="1" customWidth="1"/>
-    <col min="57" max="57" width="19.33203125" bestFit="1" customWidth="1"/>
-    <col min="58" max="58" width="13.83203125" customWidth="1"/>
-    <col min="59" max="59" width="14.33203125" bestFit="1" customWidth="1"/>
-    <col min="60" max="62" width="14.33203125" customWidth="1"/>
-    <col min="63" max="63" width="17.1640625" bestFit="1" customWidth="1"/>
-    <col min="64" max="64" width="14.83203125" bestFit="1" customWidth="1"/>
-    <col min="65" max="65" width="18.5" bestFit="1" customWidth="1"/>
-    <col min="66" max="66" width="18" bestFit="1" customWidth="1"/>
-    <col min="67" max="67" width="19.83203125" bestFit="1" customWidth="1"/>
-    <col min="68" max="69" width="17.1640625" customWidth="1"/>
-    <col min="70" max="70" width="12" bestFit="1" customWidth="1"/>
+    <col min="48" max="48" width="18.33203125" bestFit="1" customWidth="1"/>
+    <col min="49" max="49" width="14.33203125" bestFit="1" customWidth="1"/>
+    <col min="50" max="50" width="16" bestFit="1" customWidth="1"/>
+    <col min="51" max="51" width="18.33203125" bestFit="1" customWidth="1"/>
+    <col min="52" max="52" width="12.1640625" bestFit="1" customWidth="1"/>
+    <col min="53" max="53" width="19.33203125" bestFit="1" customWidth="1"/>
+    <col min="54" max="54" width="13.83203125" customWidth="1"/>
+    <col min="55" max="57" width="14.33203125" customWidth="1"/>
+    <col min="58" max="58" width="17.1640625" bestFit="1" customWidth="1"/>
+    <col min="59" max="59" width="14.83203125" bestFit="1" customWidth="1"/>
+    <col min="60" max="60" width="18.5" bestFit="1" customWidth="1"/>
+    <col min="61" max="61" width="18" bestFit="1" customWidth="1"/>
+    <col min="62" max="62" width="19.83203125" bestFit="1" customWidth="1"/>
+    <col min="63" max="64" width="17.1640625" customWidth="1"/>
+    <col min="65" max="65" width="16" bestFit="1" customWidth="1"/>
+    <col min="66" max="66" width="19.6640625" bestFit="1" customWidth="1"/>
+    <col min="67" max="67" width="6.83203125" bestFit="1" customWidth="1"/>
+    <col min="68" max="68" width="8" bestFit="1" customWidth="1"/>
+    <col min="69" max="69" width="8.83203125" bestFit="1" customWidth="1"/>
+    <col min="70" max="70" width="9.83203125" bestFit="1" customWidth="1"/>
     <col min="71" max="71" width="16" bestFit="1" customWidth="1"/>
-    <col min="72" max="72" width="19.6640625" bestFit="1" customWidth="1"/>
-    <col min="73" max="73" width="6.83203125" bestFit="1" customWidth="1"/>
-    <col min="74" max="74" width="8" bestFit="1" customWidth="1"/>
-    <col min="75" max="75" width="8.83203125" bestFit="1" customWidth="1"/>
-    <col min="76" max="76" width="9.83203125" bestFit="1" customWidth="1"/>
-    <col min="77" max="77" width="16" bestFit="1" customWidth="1"/>
-    <col min="78" max="78" width="21" bestFit="1" customWidth="1"/>
-    <col min="79" max="79" width="23.6640625" bestFit="1" customWidth="1"/>
-    <col min="80" max="80" width="13.6640625" bestFit="1" customWidth="1"/>
-    <col min="81" max="81" width="20.5" bestFit="1" customWidth="1"/>
-    <col min="82" max="82" width="18" bestFit="1" customWidth="1"/>
-    <col min="83" max="83" width="15.5" bestFit="1" customWidth="1"/>
-    <col min="84" max="84" width="21.83203125" bestFit="1" customWidth="1"/>
-    <col min="85" max="85" width="21.1640625" bestFit="1" customWidth="1"/>
-    <col min="86" max="86" width="11" bestFit="1" customWidth="1"/>
-    <col min="87" max="87" width="42.1640625" bestFit="1" customWidth="1"/>
-    <col min="88" max="88" width="17.1640625" bestFit="1" customWidth="1"/>
-    <col min="89" max="89" width="18.1640625" bestFit="1" customWidth="1"/>
-    <col min="90" max="91" width="18.1640625" customWidth="1"/>
-    <col min="92" max="92" width="27.1640625" bestFit="1" customWidth="1"/>
-    <col min="93" max="93" width="40" bestFit="1" customWidth="1"/>
-    <col min="94" max="94" width="16" bestFit="1" customWidth="1"/>
-    <col min="95" max="95" width="16" customWidth="1"/>
-    <col min="96" max="96" width="18.1640625" bestFit="1" customWidth="1"/>
-    <col min="97" max="97" width="10.5" bestFit="1" customWidth="1"/>
-    <col min="98" max="98" width="15.83203125" bestFit="1" customWidth="1"/>
-    <col min="99" max="102" width="15.83203125" customWidth="1"/>
-    <col min="103" max="122" width="10.5" customWidth="1"/>
-    <col min="123" max="123" width="16" bestFit="1" customWidth="1"/>
-    <col min="124" max="124" width="25" bestFit="1" customWidth="1"/>
-    <col min="125" max="125" width="8.33203125" bestFit="1" customWidth="1"/>
-    <col min="126" max="126" width="19.6640625" bestFit="1" customWidth="1"/>
-    <col min="127" max="127" width="17.1640625" bestFit="1" customWidth="1"/>
-    <col min="128" max="128" width="23.5" bestFit="1" customWidth="1"/>
-    <col min="129" max="129" width="14.83203125" bestFit="1" customWidth="1"/>
-    <col min="130" max="130" width="14.83203125" customWidth="1"/>
-    <col min="131" max="131" width="10.5" bestFit="1" customWidth="1"/>
-    <col min="132" max="132" width="21.33203125" bestFit="1" customWidth="1"/>
-    <col min="133" max="133" width="11.6640625" bestFit="1" customWidth="1"/>
-    <col min="134" max="134" width="22.83203125" bestFit="1" customWidth="1"/>
-    <col min="135" max="135" width="22.83203125" customWidth="1"/>
-    <col min="136" max="136" width="16.1640625" bestFit="1" customWidth="1"/>
-    <col min="137" max="137" width="16.1640625" customWidth="1"/>
-    <col min="138" max="138" width="19.83203125" bestFit="1" customWidth="1"/>
-    <col min="139" max="139" width="12.33203125" bestFit="1" customWidth="1"/>
-    <col min="140" max="141" width="12.33203125" customWidth="1"/>
-    <col min="142" max="142" width="14.1640625" bestFit="1" customWidth="1"/>
-    <col min="143" max="143" width="14.1640625" customWidth="1"/>
-    <col min="144" max="144" width="18.83203125" bestFit="1" customWidth="1"/>
-    <col min="145" max="145" width="23.6640625" bestFit="1" customWidth="1"/>
-    <col min="146" max="146" width="23.6640625" customWidth="1"/>
-    <col min="147" max="147" width="26" bestFit="1" customWidth="1"/>
-    <col min="148" max="148" width="26" customWidth="1"/>
-    <col min="149" max="149" width="36.1640625" bestFit="1" customWidth="1"/>
-    <col min="150" max="150" width="41.5" bestFit="1" customWidth="1"/>
-    <col min="151" max="151" width="29" bestFit="1" customWidth="1"/>
-    <col min="152" max="152" width="20.33203125" bestFit="1" customWidth="1"/>
-    <col min="153" max="153" width="9.83203125" bestFit="1" customWidth="1"/>
-    <col min="154" max="155" width="12.83203125" bestFit="1" customWidth="1"/>
-    <col min="156" max="157" width="12.83203125" customWidth="1"/>
-    <col min="158" max="158" width="17.5" bestFit="1" customWidth="1"/>
-    <col min="159" max="159" width="18.5" bestFit="1" customWidth="1"/>
-    <col min="160" max="160" width="17.5" customWidth="1"/>
-    <col min="161" max="161" width="11.83203125" bestFit="1" customWidth="1"/>
-    <col min="162" max="162" width="13" bestFit="1" customWidth="1"/>
-    <col min="163" max="163" width="19.5" bestFit="1" customWidth="1"/>
-    <col min="164" max="164" width="12.33203125" bestFit="1" customWidth="1"/>
-    <col min="165" max="167" width="19.5" customWidth="1"/>
-    <col min="168" max="168" width="9.83203125" bestFit="1" customWidth="1"/>
-    <col min="169" max="169" width="9.83203125" customWidth="1"/>
-    <col min="170" max="170" width="11.5" bestFit="1" customWidth="1"/>
-    <col min="171" max="174" width="11.5" customWidth="1"/>
-    <col min="175" max="175" width="13.83203125" bestFit="1" customWidth="1"/>
-    <col min="176" max="176" width="4.5" bestFit="1" customWidth="1"/>
-    <col min="177" max="177" width="9" bestFit="1" customWidth="1"/>
-    <col min="178" max="178" width="15.1640625" bestFit="1" customWidth="1"/>
-    <col min="179" max="179" width="16.1640625" bestFit="1" customWidth="1"/>
-    <col min="180" max="180" width="18.1640625" bestFit="1" customWidth="1"/>
-    <col min="181" max="181" width="18.1640625" customWidth="1"/>
-    <col min="182" max="182" width="18.1640625" bestFit="1" customWidth="1"/>
-    <col min="183" max="183" width="8.33203125" bestFit="1" customWidth="1"/>
-    <col min="184" max="186" width="8.33203125" customWidth="1"/>
-    <col min="187" max="187" width="22" bestFit="1" customWidth="1"/>
-    <col min="188" max="188" width="7.6640625" bestFit="1" customWidth="1"/>
-    <col min="189" max="189" width="12.33203125" bestFit="1" customWidth="1"/>
-    <col min="190" max="190" width="14" bestFit="1" customWidth="1"/>
-    <col min="191" max="191" width="14" customWidth="1"/>
-    <col min="192" max="192" width="15.5" bestFit="1" customWidth="1"/>
-    <col min="193" max="193" width="18.1640625" bestFit="1" customWidth="1"/>
-    <col min="194" max="194" width="18.1640625" customWidth="1"/>
-    <col min="195" max="195" width="17.6640625" bestFit="1" customWidth="1"/>
-    <col min="196" max="196" width="11.83203125" bestFit="1" customWidth="1"/>
-    <col min="197" max="197" width="18.1640625" bestFit="1" customWidth="1"/>
-    <col min="198" max="200" width="18.1640625" customWidth="1"/>
-    <col min="201" max="201" width="46.33203125" bestFit="1" customWidth="1"/>
-    <col min="202" max="202" width="35" bestFit="1" customWidth="1"/>
-    <col min="203" max="203" width="43.1640625" bestFit="1" customWidth="1"/>
-    <col min="204" max="204" width="18.1640625" customWidth="1"/>
-    <col min="205" max="205" width="9.33203125" bestFit="1" customWidth="1"/>
-    <col min="206" max="206" width="10.83203125" customWidth="1"/>
+    <col min="72" max="72" width="21" bestFit="1" customWidth="1"/>
+    <col min="73" max="73" width="23.6640625" bestFit="1" customWidth="1"/>
+    <col min="74" max="74" width="13.6640625" bestFit="1" customWidth="1"/>
+    <col min="75" max="75" width="20.5" bestFit="1" customWidth="1"/>
+    <col min="76" max="76" width="18" bestFit="1" customWidth="1"/>
+    <col min="77" max="77" width="15.5" bestFit="1" customWidth="1"/>
+    <col min="78" max="78" width="21.83203125" bestFit="1" customWidth="1"/>
+    <col min="79" max="79" width="21.1640625" bestFit="1" customWidth="1"/>
+    <col min="80" max="80" width="11" bestFit="1" customWidth="1"/>
+    <col min="81" max="81" width="42.1640625" bestFit="1" customWidth="1"/>
+    <col min="82" max="82" width="17.1640625" bestFit="1" customWidth="1"/>
+    <col min="83" max="83" width="18.1640625" bestFit="1" customWidth="1"/>
+    <col min="84" max="85" width="18.1640625" customWidth="1"/>
+    <col min="86" max="86" width="27.1640625" bestFit="1" customWidth="1"/>
+    <col min="87" max="87" width="40" bestFit="1" customWidth="1"/>
+    <col min="88" max="88" width="16" bestFit="1" customWidth="1"/>
+    <col min="89" max="89" width="16" customWidth="1"/>
+    <col min="90" max="90" width="18.1640625" bestFit="1" customWidth="1"/>
+    <col min="91" max="91" width="10.5" bestFit="1" customWidth="1"/>
+    <col min="92" max="92" width="15.83203125" bestFit="1" customWidth="1"/>
+    <col min="93" max="96" width="15.83203125" customWidth="1"/>
+    <col min="97" max="116" width="10.5" customWidth="1"/>
+    <col min="117" max="117" width="25" bestFit="1" customWidth="1"/>
+    <col min="118" max="118" width="8.33203125" bestFit="1" customWidth="1"/>
+    <col min="119" max="119" width="19.6640625" bestFit="1" customWidth="1"/>
+    <col min="120" max="120" width="17.1640625" bestFit="1" customWidth="1"/>
+    <col min="121" max="121" width="23.5" bestFit="1" customWidth="1"/>
+    <col min="122" max="122" width="14.83203125" bestFit="1" customWidth="1"/>
+    <col min="123" max="123" width="14.83203125" customWidth="1"/>
+    <col min="124" max="124" width="21.33203125" bestFit="1" customWidth="1"/>
+    <col min="125" max="125" width="11.6640625" bestFit="1" customWidth="1"/>
+    <col min="126" max="126" width="22.83203125" bestFit="1" customWidth="1"/>
+    <col min="127" max="127" width="22.83203125" customWidth="1"/>
+    <col min="128" max="128" width="16.1640625" customWidth="1"/>
+    <col min="129" max="129" width="19.83203125" bestFit="1" customWidth="1"/>
+    <col min="130" max="131" width="12.33203125" customWidth="1"/>
+    <col min="132" max="132" width="14.1640625" customWidth="1"/>
+    <col min="133" max="133" width="23.6640625" bestFit="1" customWidth="1"/>
+    <col min="134" max="134" width="23.6640625" customWidth="1"/>
+    <col min="135" max="135" width="26" bestFit="1" customWidth="1"/>
+    <col min="136" max="136" width="26" customWidth="1"/>
+    <col min="137" max="137" width="36.1640625" bestFit="1" customWidth="1"/>
+    <col min="138" max="138" width="41.5" bestFit="1" customWidth="1"/>
+    <col min="139" max="139" width="29" bestFit="1" customWidth="1"/>
+    <col min="140" max="140" width="20.33203125" bestFit="1" customWidth="1"/>
+    <col min="141" max="141" width="9.83203125" bestFit="1" customWidth="1"/>
+    <col min="142" max="142" width="12.83203125" bestFit="1" customWidth="1"/>
+    <col min="143" max="144" width="12.83203125" customWidth="1"/>
+    <col min="145" max="145" width="18.5" bestFit="1" customWidth="1"/>
+    <col min="146" max="146" width="17.5" customWidth="1"/>
+    <col min="147" max="147" width="13" bestFit="1" customWidth="1"/>
+    <col min="148" max="148" width="19.5" bestFit="1" customWidth="1"/>
+    <col min="149" max="149" width="12.33203125" bestFit="1" customWidth="1"/>
+    <col min="150" max="152" width="19.5" customWidth="1"/>
+    <col min="153" max="153" width="9.83203125" customWidth="1"/>
+    <col min="154" max="157" width="11.5" customWidth="1"/>
+    <col min="158" max="158" width="4.5" bestFit="1" customWidth="1"/>
+    <col min="159" max="159" width="9" bestFit="1" customWidth="1"/>
+    <col min="160" max="160" width="16.1640625" bestFit="1" customWidth="1"/>
+    <col min="161" max="161" width="18.1640625" bestFit="1" customWidth="1"/>
+    <col min="162" max="162" width="18.1640625" customWidth="1"/>
+    <col min="163" max="163" width="8.33203125" bestFit="1" customWidth="1"/>
+    <col min="164" max="166" width="8.33203125" customWidth="1"/>
+    <col min="167" max="167" width="7.6640625" bestFit="1" customWidth="1"/>
+    <col min="168" max="168" width="12.33203125" bestFit="1" customWidth="1"/>
+    <col min="169" max="169" width="14" customWidth="1"/>
+    <col min="170" max="170" width="15.5" bestFit="1" customWidth="1"/>
+    <col min="171" max="171" width="18.1640625" customWidth="1"/>
+    <col min="172" max="172" width="17.6640625" bestFit="1" customWidth="1"/>
+    <col min="173" max="173" width="11.83203125" bestFit="1" customWidth="1"/>
+    <col min="174" max="176" width="18.1640625" customWidth="1"/>
+    <col min="177" max="177" width="46.33203125" bestFit="1" customWidth="1"/>
+    <col min="178" max="178" width="35" bestFit="1" customWidth="1"/>
+    <col min="179" max="179" width="43.1640625" bestFit="1" customWidth="1"/>
+    <col min="180" max="180" width="18.1640625" customWidth="1"/>
+    <col min="181" max="181" width="9.33203125" bestFit="1" customWidth="1"/>
+    <col min="182" max="182" width="10.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:206" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:182" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -2170,16 +2045,16 @@
       <c r="BA1" t="s">
         <v>52</v>
       </c>
-      <c r="BB1" t="s">
+      <c r="BC1" t="s">
         <v>53</v>
       </c>
-      <c r="BC1" t="s">
+      <c r="BD1" t="s">
         <v>54</v>
       </c>
-      <c r="BD1" t="s">
+      <c r="BE1" t="s">
         <v>55</v>
       </c>
-      <c r="BE1" t="s">
+      <c r="BF1" t="s">
         <v>56</v>
       </c>
       <c r="BG1" t="s">
@@ -2554,865 +2429,724 @@
       <c r="FZ1" t="s">
         <v>180</v>
       </c>
-      <c r="GA1" t="s">
+    </row>
+    <row r="2" spans="1:182" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
         <v>181</v>
       </c>
-      <c r="GB1" t="s">
+      <c r="B2" t="s">
         <v>182</v>
       </c>
-      <c r="GC1" t="s">
+      <c r="C2" t="s">
         <v>183</v>
       </c>
-      <c r="GD1" t="s">
+      <c r="D2" t="s">
         <v>184</v>
       </c>
-      <c r="GE1" t="s">
+      <c r="E2" t="s">
+        <v>186</v>
+      </c>
+      <c r="F2" t="s">
+        <v>187</v>
+      </c>
+      <c r="G2" t="s">
         <v>185</v>
       </c>
-      <c r="GF1" t="s">
-        <v>186</v>
-      </c>
-      <c r="GG1" t="s">
-        <v>187</v>
-      </c>
-      <c r="GH1" t="s">
+      <c r="H2" t="s">
         <v>188</v>
       </c>
-      <c r="GI1" t="s">
+      <c r="I2" t="s">
+        <v>185</v>
+      </c>
+      <c r="J2" t="s">
+        <v>185</v>
+      </c>
+      <c r="K2" t="s">
+        <v>185</v>
+      </c>
+      <c r="L2" t="s">
+        <v>185</v>
+      </c>
+      <c r="M2" t="s">
+        <v>185</v>
+      </c>
+      <c r="N2" t="s">
+        <v>185</v>
+      </c>
+      <c r="O2" t="s">
+        <v>185</v>
+      </c>
+      <c r="P2" t="s">
+        <v>185</v>
+      </c>
+      <c r="Q2" t="s">
+        <v>185</v>
+      </c>
+      <c r="R2" t="s">
         <v>189</v>
       </c>
-      <c r="GJ1" t="s">
+      <c r="S2" t="s">
+        <v>189</v>
+      </c>
+      <c r="T2" t="s">
+        <v>189</v>
+      </c>
+      <c r="U2" t="s">
+        <v>189</v>
+      </c>
+      <c r="V2" t="s">
+        <v>187</v>
+      </c>
+      <c r="W2" t="s">
+        <v>185</v>
+      </c>
+      <c r="X2" t="s">
+        <v>185</v>
+      </c>
+      <c r="Y2" t="s">
+        <v>185</v>
+      </c>
+      <c r="Z2" t="s">
+        <v>185</v>
+      </c>
+      <c r="AA2" t="s">
+        <v>185</v>
+      </c>
+      <c r="AB2" t="s">
+        <v>187</v>
+      </c>
+      <c r="AC2" t="s">
         <v>190</v>
       </c>
-      <c r="GK1" t="s">
+      <c r="AD2">
+        <v>3</v>
+      </c>
+      <c r="AE2">
+        <v>15</v>
+      </c>
+      <c r="AF2" t="s">
+        <v>187</v>
+      </c>
+      <c r="AG2">
+        <v>3</v>
+      </c>
+      <c r="AH2" t="s">
         <v>191</v>
       </c>
-      <c r="GL1" t="s">
+      <c r="AI2" t="s">
+        <v>187</v>
+      </c>
+      <c r="AJ2" t="s">
+        <v>187</v>
+      </c>
+      <c r="AK2">
+        <v>5</v>
+      </c>
+      <c r="AL2">
+        <v>60</v>
+      </c>
+      <c r="AM2" t="s">
+        <v>187</v>
+      </c>
+      <c r="AN2">
+        <v>6</v>
+      </c>
+      <c r="AO2">
+        <v>30</v>
+      </c>
+      <c r="AP2" t="s">
+        <v>187</v>
+      </c>
+      <c r="AQ2">
+        <v>3</v>
+      </c>
+      <c r="AR2">
+        <v>120</v>
+      </c>
+      <c r="AS2" t="s">
+        <v>187</v>
+      </c>
+      <c r="AT2">
+        <v>2</v>
+      </c>
+      <c r="AU2">
+        <v>100</v>
+      </c>
+      <c r="AV2" t="s">
+        <v>187</v>
+      </c>
+      <c r="AW2">
+        <v>1</v>
+      </c>
+      <c r="AX2">
+        <v>20</v>
+      </c>
+      <c r="AY2" t="s">
+        <v>187</v>
+      </c>
+      <c r="AZ2">
+        <v>1</v>
+      </c>
+      <c r="BA2">
+        <v>20</v>
+      </c>
+      <c r="BC2" t="s">
+        <v>193</v>
+      </c>
+      <c r="BD2" t="s">
+        <v>194</v>
+      </c>
+      <c r="BE2" t="s">
+        <v>195</v>
+      </c>
+      <c r="BF2" t="s">
         <v>192</v>
       </c>
-      <c r="GM1" t="s">
+      <c r="BG2" t="s">
+        <v>187</v>
+      </c>
+      <c r="BH2" t="s">
+        <v>196</v>
+      </c>
+      <c r="BI2" t="s">
+        <v>197</v>
+      </c>
+      <c r="BK2" t="s">
+        <v>195</v>
+      </c>
+      <c r="BM2" t="s">
+        <v>187</v>
+      </c>
+      <c r="BN2" t="s">
+        <v>196</v>
+      </c>
+      <c r="BO2" t="s">
+        <v>198</v>
+      </c>
+      <c r="BP2" t="s">
         <v>193</v>
       </c>
-      <c r="GN1" t="s">
-        <v>194</v>
-      </c>
-      <c r="GO1" t="s">
+      <c r="BS2" t="s">
+        <v>187</v>
+      </c>
+      <c r="BT2" t="s">
+        <v>199</v>
+      </c>
+      <c r="BU2" t="s">
+        <v>187</v>
+      </c>
+      <c r="BV2" t="s">
+        <v>187</v>
+      </c>
+      <c r="BW2" t="s">
+        <v>187</v>
+      </c>
+      <c r="BX2" t="s">
+        <v>187</v>
+      </c>
+      <c r="BY2" t="s">
+        <v>187</v>
+      </c>
+      <c r="BZ2" t="s">
+        <v>187</v>
+      </c>
+      <c r="CA2" t="s">
+        <v>187</v>
+      </c>
+      <c r="CB2" t="s">
+        <v>200</v>
+      </c>
+      <c r="CC2" t="s">
+        <v>201</v>
+      </c>
+      <c r="CD2" t="s">
+        <v>202</v>
+      </c>
+      <c r="CE2" t="s">
+        <v>202</v>
+      </c>
+      <c r="CF2" t="s">
+        <v>202</v>
+      </c>
+      <c r="CG2" t="s">
+        <v>202</v>
+      </c>
+      <c r="CH2" t="s">
+        <v>203</v>
+      </c>
+      <c r="CI2" t="s">
+        <v>204</v>
+      </c>
+      <c r="CJ2" t="s">
+        <v>205</v>
+      </c>
+      <c r="CK2" t="s">
+        <v>202</v>
+      </c>
+      <c r="CL2" t="s">
+        <v>206</v>
+      </c>
+      <c r="CM2" t="s">
+        <v>207</v>
+      </c>
+      <c r="CN2" t="s">
+        <v>208</v>
+      </c>
+      <c r="CO2" t="s">
+        <v>209</v>
+      </c>
+      <c r="CP2" t="s">
+        <v>210</v>
+      </c>
+      <c r="CQ2" t="s">
+        <v>210</v>
+      </c>
+      <c r="CR2" t="s">
+        <v>211</v>
+      </c>
+      <c r="CS2" t="s">
+        <v>211</v>
+      </c>
+      <c r="CT2" t="s">
+        <v>211</v>
+      </c>
+      <c r="CU2" t="s">
+        <v>211</v>
+      </c>
+      <c r="CV2" t="s">
+        <v>211</v>
+      </c>
+      <c r="CW2" t="s">
+        <v>212</v>
+      </c>
+      <c r="CX2" t="s">
+        <v>212</v>
+      </c>
+      <c r="CY2" t="s">
+        <v>212</v>
+      </c>
+      <c r="CZ2" t="s">
+        <v>213</v>
+      </c>
+      <c r="DA2" t="s">
+        <v>214</v>
+      </c>
+      <c r="DB2" t="s">
+        <v>215</v>
+      </c>
+      <c r="DC2" t="s">
+        <v>216</v>
+      </c>
+      <c r="DD2" t="s">
+        <v>217</v>
+      </c>
+      <c r="DE2" t="s">
+        <v>187</v>
+      </c>
+      <c r="DF2" t="s">
+        <v>218</v>
+      </c>
+      <c r="DG2" t="s">
+        <v>219</v>
+      </c>
+      <c r="DH2" t="s">
+        <v>220</v>
+      </c>
+      <c r="DI2" t="s">
+        <v>187</v>
+      </c>
+      <c r="DJ2" t="s">
+        <v>187</v>
+      </c>
+      <c r="DK2" t="s">
+        <v>187</v>
+      </c>
+      <c r="DL2" t="s">
+        <v>187</v>
+      </c>
+      <c r="DM2" t="s">
+        <v>221</v>
+      </c>
+      <c r="DN2" t="s">
+        <v>187</v>
+      </c>
+      <c r="DO2" t="s">
+        <v>187</v>
+      </c>
+      <c r="DP2" t="s">
+        <v>187</v>
+      </c>
+      <c r="DQ2" t="s">
+        <v>187</v>
+      </c>
+      <c r="DR2" t="s">
+        <v>187</v>
+      </c>
+      <c r="DS2" t="s">
+        <v>222</v>
+      </c>
+      <c r="DT2" t="s">
+        <v>223</v>
+      </c>
+      <c r="DU2" t="s">
+        <v>224</v>
+      </c>
+      <c r="DV2" t="s">
+        <v>225</v>
+      </c>
+      <c r="DW2" t="s">
+        <v>226</v>
+      </c>
+      <c r="DX2" t="s">
+        <v>227</v>
+      </c>
+      <c r="DY2" t="s">
+        <v>228</v>
+      </c>
+      <c r="DZ2" t="s">
+        <v>229</v>
+      </c>
+      <c r="EA2" t="s">
+        <v>230</v>
+      </c>
+      <c r="EB2" t="s">
+        <v>231</v>
+      </c>
+      <c r="EC2" t="s">
+        <v>232</v>
+      </c>
+      <c r="ED2" t="s">
+        <v>233</v>
+      </c>
+      <c r="EE2" t="s">
+        <v>234</v>
+      </c>
+      <c r="EF2" t="s">
+        <v>235</v>
+      </c>
+      <c r="EG2" t="s">
+        <v>236</v>
+      </c>
+      <c r="EH2" t="s">
+        <v>237</v>
+      </c>
+      <c r="EI2" t="s">
+        <v>238</v>
+      </c>
+      <c r="EJ2" t="s">
+        <v>239</v>
+      </c>
+      <c r="EK2" t="s">
+        <v>222</v>
+      </c>
+      <c r="EL2" t="s">
+        <v>240</v>
+      </c>
+      <c r="EM2" t="s">
+        <v>187</v>
+      </c>
+      <c r="EN2" t="s">
+        <v>185</v>
+      </c>
+      <c r="EO2" t="s">
+        <v>187</v>
+      </c>
+      <c r="EP2" t="s">
+        <v>187</v>
+      </c>
+      <c r="EQ2" t="s">
+        <v>241</v>
+      </c>
+      <c r="ER2" t="s">
+        <v>242</v>
+      </c>
+      <c r="ES2" t="s">
+        <v>187</v>
+      </c>
+      <c r="ET2" t="s">
+        <v>187</v>
+      </c>
+      <c r="EU2" t="s">
+        <v>187</v>
+      </c>
+      <c r="EV2" t="s">
+        <v>187</v>
+      </c>
+      <c r="EW2" t="s">
         <v>195</v>
       </c>
-      <c r="GP1" t="s">
-        <v>196</v>
-      </c>
-      <c r="GQ1" t="s">
-        <v>197</v>
-      </c>
-      <c r="GR1" t="s">
-        <v>198</v>
-      </c>
-      <c r="GS1" t="s">
-        <v>199</v>
-      </c>
-      <c r="GT1" t="s">
-        <v>200</v>
-      </c>
-      <c r="GU1" t="s">
-        <v>201</v>
-      </c>
-      <c r="GV1" t="s">
-        <v>202</v>
-      </c>
-      <c r="GW1" t="s">
-        <v>203</v>
-      </c>
-      <c r="GX1" t="s">
-        <v>204</v>
-      </c>
-    </row>
-    <row r="2" spans="1:206" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
-        <v>205</v>
-      </c>
-      <c r="B2" t="s">
-        <v>206</v>
-      </c>
-      <c r="C2" t="s">
-        <v>207</v>
-      </c>
-      <c r="E2" t="s">
-        <v>208</v>
-      </c>
-      <c r="F2" t="s">
-        <v>209</v>
-      </c>
-      <c r="G2" t="s">
-        <v>209</v>
-      </c>
-      <c r="H2" t="s">
-        <v>210</v>
-      </c>
-      <c r="I2" t="s">
-        <v>211</v>
-      </c>
-      <c r="J2" t="s">
-        <v>209</v>
-      </c>
-      <c r="K2" t="s">
-        <v>212</v>
-      </c>
-      <c r="L2" t="s">
-        <v>209</v>
-      </c>
-      <c r="M2" t="s">
-        <v>209</v>
-      </c>
-      <c r="N2" t="s">
-        <v>209</v>
-      </c>
-      <c r="O2" t="s">
-        <v>209</v>
-      </c>
-      <c r="P2" t="s">
-        <v>209</v>
-      </c>
-      <c r="Q2" t="s">
-        <v>209</v>
-      </c>
-      <c r="R2" t="s">
-        <v>209</v>
-      </c>
-      <c r="S2" t="s">
-        <v>209</v>
-      </c>
-      <c r="T2" t="s">
-        <v>209</v>
-      </c>
-      <c r="U2" t="s">
-        <v>209</v>
-      </c>
-      <c r="V2" t="s">
-        <v>213</v>
-      </c>
-      <c r="W2" t="s">
-        <v>213</v>
-      </c>
-      <c r="X2" t="s">
-        <v>213</v>
-      </c>
-      <c r="Y2" t="s">
-        <v>213</v>
-      </c>
-      <c r="Z2" t="s">
-        <v>211</v>
-      </c>
-      <c r="AA2" t="s">
-        <v>209</v>
-      </c>
-      <c r="AB2" t="s">
-        <v>209</v>
-      </c>
-      <c r="AC2" t="s">
-        <v>209</v>
-      </c>
-      <c r="AD2" t="s">
-        <v>209</v>
-      </c>
-      <c r="AE2" t="s">
-        <v>209</v>
-      </c>
-      <c r="AF2" t="s">
-        <v>211</v>
-      </c>
-      <c r="AG2" t="s">
-        <v>214</v>
-      </c>
-      <c r="AH2">
-        <v>3</v>
-      </c>
-      <c r="AI2">
-        <v>15</v>
-      </c>
-      <c r="AJ2" t="s">
-        <v>211</v>
-      </c>
-      <c r="AK2">
-        <v>3</v>
-      </c>
-      <c r="AL2" t="s">
-        <v>215</v>
-      </c>
-      <c r="AM2" t="s">
-        <v>211</v>
-      </c>
-      <c r="AN2" t="s">
-        <v>211</v>
-      </c>
-      <c r="AO2">
-        <v>5</v>
-      </c>
-      <c r="AP2">
-        <v>60</v>
-      </c>
-      <c r="AQ2" t="s">
-        <v>211</v>
-      </c>
-      <c r="AR2">
-        <v>6</v>
-      </c>
-      <c r="AS2">
-        <v>30</v>
-      </c>
-      <c r="AT2" t="s">
-        <v>211</v>
-      </c>
-      <c r="AU2">
-        <v>3</v>
-      </c>
-      <c r="AV2">
-        <v>120</v>
-      </c>
-      <c r="AW2" t="s">
-        <v>211</v>
-      </c>
-      <c r="AX2">
-        <v>2</v>
-      </c>
-      <c r="AY2">
-        <v>100</v>
-      </c>
-      <c r="AZ2" t="s">
-        <v>211</v>
-      </c>
-      <c r="BA2">
-        <v>1</v>
-      </c>
-      <c r="BB2">
-        <v>20</v>
-      </c>
-      <c r="BC2" t="s">
-        <v>211</v>
-      </c>
-      <c r="BD2">
-        <v>1</v>
-      </c>
-      <c r="BE2">
-        <v>20</v>
-      </c>
-      <c r="BG2" t="s">
-        <v>216</v>
-      </c>
-      <c r="BH2" t="s">
-        <v>217</v>
-      </c>
-      <c r="BI2" t="s">
-        <v>218</v>
-      </c>
-      <c r="BJ2" t="s">
-        <v>219</v>
-      </c>
-      <c r="BK2" t="s">
-        <v>216</v>
-      </c>
-      <c r="BL2" t="s">
-        <v>211</v>
-      </c>
-      <c r="BM2" t="s">
-        <v>220</v>
-      </c>
-      <c r="BN2" t="s">
-        <v>221</v>
-      </c>
-      <c r="BP2" t="s">
-        <v>219</v>
-      </c>
-      <c r="BR2" t="s">
-        <v>216</v>
-      </c>
-      <c r="BS2" t="s">
-        <v>211</v>
-      </c>
-      <c r="BT2" t="s">
-        <v>220</v>
-      </c>
-      <c r="BU2" t="s">
+      <c r="EX2" t="s">
+        <v>243</v>
+      </c>
+      <c r="EY2" t="s">
+        <v>243</v>
+      </c>
+      <c r="EZ2" t="s">
+        <v>244</v>
+      </c>
+      <c r="FA2" t="s">
+        <v>245</v>
+      </c>
+      <c r="FB2" t="s">
+        <v>246</v>
+      </c>
+      <c r="FC2" t="s">
+        <v>247</v>
+      </c>
+      <c r="FD2" t="s">
+        <v>248</v>
+      </c>
+      <c r="FE2" t="s">
+        <v>249</v>
+      </c>
+      <c r="FF2" t="s">
+        <v>250</v>
+      </c>
+      <c r="FG2" t="s">
+        <v>251</v>
+      </c>
+      <c r="FH2" t="s">
+        <v>243</v>
+      </c>
+      <c r="FI2" t="s">
+        <v>195</v>
+      </c>
+      <c r="FJ2" t="s">
+        <v>252</v>
+      </c>
+      <c r="FK2" t="s">
+        <v>252</v>
+      </c>
+      <c r="FL2" t="s">
+        <v>253</v>
+      </c>
+      <c r="FM2" t="s">
         <v>222</v>
       </c>
-      <c r="BV2" t="s">
-        <v>217</v>
-      </c>
-      <c r="BY2" t="s">
-        <v>211</v>
-      </c>
-      <c r="BZ2" t="s">
-        <v>223</v>
-      </c>
-      <c r="CA2" t="s">
-        <v>211</v>
-      </c>
-      <c r="CB2" t="s">
-        <v>211</v>
-      </c>
-      <c r="CC2" t="s">
-        <v>211</v>
-      </c>
-      <c r="CD2" t="s">
-        <v>211</v>
-      </c>
-      <c r="CE2" t="s">
-        <v>211</v>
-      </c>
-      <c r="CF2" t="s">
-        <v>211</v>
-      </c>
-      <c r="CG2" t="s">
-        <v>211</v>
-      </c>
-      <c r="CH2" t="s">
-        <v>224</v>
-      </c>
-      <c r="CI2" t="s">
-        <v>225</v>
-      </c>
-      <c r="CJ2" t="s">
-        <v>226</v>
-      </c>
-      <c r="CK2" t="s">
-        <v>226</v>
-      </c>
-      <c r="CL2" t="s">
-        <v>226</v>
-      </c>
-      <c r="CM2" t="s">
-        <v>226</v>
-      </c>
-      <c r="CN2" t="s">
-        <v>227</v>
-      </c>
-      <c r="CO2" t="s">
-        <v>228</v>
-      </c>
-      <c r="CP2" t="s">
-        <v>229</v>
-      </c>
-      <c r="CQ2" t="s">
-        <v>226</v>
-      </c>
-      <c r="CR2" t="s">
-        <v>230</v>
-      </c>
-      <c r="CS2" t="s">
-        <v>231</v>
-      </c>
-      <c r="CT2" t="s">
-        <v>232</v>
-      </c>
-      <c r="CU2" t="s">
-        <v>233</v>
-      </c>
-      <c r="CV2" t="s">
-        <v>234</v>
-      </c>
-      <c r="CW2" t="s">
-        <v>234</v>
-      </c>
-      <c r="CX2" t="s">
-        <v>235</v>
-      </c>
-      <c r="CY2" t="s">
-        <v>235</v>
-      </c>
-      <c r="CZ2" t="s">
-        <v>235</v>
-      </c>
-      <c r="DA2" t="s">
-        <v>235</v>
-      </c>
-      <c r="DB2" t="s">
-        <v>235</v>
-      </c>
-      <c r="DC2" t="s">
-        <v>236</v>
-      </c>
-      <c r="DD2" t="s">
-        <v>236</v>
-      </c>
-      <c r="DE2" t="s">
-        <v>236</v>
-      </c>
-      <c r="DF2" t="s">
-        <v>237</v>
-      </c>
-      <c r="DG2" t="s">
-        <v>238</v>
-      </c>
-      <c r="DH2" t="s">
-        <v>239</v>
-      </c>
-      <c r="DI2" t="s">
-        <v>240</v>
-      </c>
-      <c r="DJ2" t="s">
-        <v>241</v>
-      </c>
-      <c r="DK2" t="s">
-        <v>211</v>
-      </c>
-      <c r="DL2" t="s">
-        <v>242</v>
-      </c>
-      <c r="DM2" t="s">
-        <v>243</v>
-      </c>
-      <c r="DN2" t="s">
-        <v>244</v>
-      </c>
-      <c r="DO2" t="s">
-        <v>211</v>
-      </c>
-      <c r="DP2" t="s">
-        <v>211</v>
-      </c>
-      <c r="DQ2" t="s">
-        <v>211</v>
-      </c>
-      <c r="DR2" t="s">
-        <v>211</v>
-      </c>
-      <c r="DS2" t="s">
-        <v>216</v>
-      </c>
-      <c r="DT2" t="s">
-        <v>245</v>
-      </c>
-      <c r="DU2" t="s">
-        <v>211</v>
-      </c>
-      <c r="DV2" t="s">
-        <v>211</v>
-      </c>
-      <c r="DW2" t="s">
-        <v>211</v>
-      </c>
-      <c r="DX2" t="s">
-        <v>211</v>
-      </c>
-      <c r="DY2" t="s">
-        <v>211</v>
-      </c>
-      <c r="DZ2" t="s">
-        <v>246</v>
-      </c>
-      <c r="EA2" t="s">
-        <v>216</v>
-      </c>
-      <c r="EB2" t="s">
-        <v>247</v>
-      </c>
-      <c r="EC2" t="s">
-        <v>248</v>
-      </c>
-      <c r="ED2" t="s">
-        <v>249</v>
-      </c>
-      <c r="EE2" t="s">
-        <v>250</v>
-      </c>
-      <c r="EF2" t="s">
-        <v>216</v>
-      </c>
-      <c r="EG2" t="s">
-        <v>251</v>
-      </c>
-      <c r="EH2" t="s">
-        <v>252</v>
-      </c>
-      <c r="EI2" t="s">
-        <v>216</v>
-      </c>
-      <c r="EJ2" t="s">
-        <v>253</v>
-      </c>
-      <c r="EK2" t="s">
+      <c r="FN2" t="s">
         <v>254</v>
       </c>
-      <c r="EL2" t="s">
-        <v>216</v>
-      </c>
-      <c r="EM2" t="s">
+      <c r="FO2" t="s">
         <v>255</v>
       </c>
-      <c r="EN2" t="s">
-        <v>216</v>
-      </c>
-      <c r="EO2" t="s">
+      <c r="FP2" t="s">
         <v>256</v>
       </c>
-      <c r="EP2" t="s">
+      <c r="FQ2" t="s">
         <v>257</v>
       </c>
-      <c r="EQ2" t="s">
+      <c r="FR2" t="s">
         <v>258</v>
       </c>
-      <c r="ER2" t="s">
+      <c r="FS2" t="s">
         <v>259</v>
       </c>
-      <c r="ES2" t="s">
+      <c r="FT2" t="s">
         <v>260</v>
       </c>
-      <c r="ET2" t="s">
+      <c r="FU2" t="s">
         <v>261</v>
       </c>
-      <c r="EU2" t="s">
+      <c r="FV2" t="s">
         <v>262</v>
       </c>
-      <c r="EV2" t="s">
+      <c r="FW2" t="s">
         <v>263</v>
       </c>
-      <c r="EW2" t="s">
-        <v>246</v>
-      </c>
-      <c r="EX2" t="s">
+      <c r="FX2" t="s">
         <v>264</v>
       </c>
-      <c r="EY2" t="s">
-        <v>216</v>
-      </c>
-      <c r="EZ2" t="s">
-        <v>211</v>
-      </c>
-      <c r="FA2" t="s">
-        <v>209</v>
-      </c>
-      <c r="FB2" t="s">
-        <v>216</v>
-      </c>
-      <c r="FC2" t="s">
-        <v>211</v>
-      </c>
-      <c r="FD2" t="s">
-        <v>211</v>
-      </c>
-      <c r="FE2" t="s">
-        <v>216</v>
-      </c>
-      <c r="FF2" t="s">
-        <v>265</v>
-      </c>
-      <c r="FG2" t="s">
-        <v>266</v>
-      </c>
-      <c r="FH2" t="s">
-        <v>211</v>
-      </c>
-      <c r="FI2" t="s">
-        <v>211</v>
-      </c>
-      <c r="FJ2" t="s">
-        <v>211</v>
-      </c>
-      <c r="FK2" t="s">
-        <v>211</v>
-      </c>
-      <c r="FL2" t="s">
-        <v>216</v>
-      </c>
-      <c r="FM2" t="s">
-        <v>219</v>
-      </c>
-      <c r="FN2" t="s">
-        <v>216</v>
-      </c>
-      <c r="FO2" t="s">
-        <v>267</v>
-      </c>
-      <c r="FP2" t="s">
-        <v>267</v>
-      </c>
-      <c r="FQ2" t="s">
-        <v>268</v>
-      </c>
-      <c r="FR2" t="s">
-        <v>269</v>
-      </c>
-      <c r="FS2" t="s">
-        <v>216</v>
-      </c>
-      <c r="FT2" t="s">
-        <v>270</v>
-      </c>
-      <c r="FU2" t="s">
-        <v>271</v>
-      </c>
-      <c r="FV2" t="s">
-        <v>216</v>
-      </c>
-      <c r="FW2" t="s">
-        <v>272</v>
-      </c>
-      <c r="FX2" t="s">
-        <v>273</v>
-      </c>
       <c r="FY2" t="s">
-        <v>274</v>
-      </c>
-      <c r="FZ2" t="s">
-        <v>216</v>
-      </c>
-      <c r="GA2" t="s">
-        <v>275</v>
-      </c>
-      <c r="GB2" t="s">
-        <v>267</v>
-      </c>
-      <c r="GC2" t="s">
-        <v>219</v>
-      </c>
-      <c r="GD2" t="s">
-        <v>276</v>
-      </c>
-      <c r="GE2" t="s">
-        <v>216</v>
-      </c>
-      <c r="GF2" t="s">
-        <v>276</v>
-      </c>
-      <c r="GG2" t="s">
-        <v>277</v>
-      </c>
-      <c r="GH2" t="s">
-        <v>216</v>
-      </c>
-      <c r="GI2" t="s">
-        <v>246</v>
-      </c>
-      <c r="GJ2" t="s">
-        <v>278</v>
-      </c>
-      <c r="GK2" t="s">
-        <v>216</v>
-      </c>
-      <c r="GL2" t="s">
-        <v>279</v>
-      </c>
-      <c r="GM2" t="s">
-        <v>280</v>
-      </c>
-      <c r="GN2" t="s">
-        <v>281</v>
-      </c>
-      <c r="GO2" t="s">
-        <v>216</v>
-      </c>
-      <c r="GP2" t="s">
-        <v>282</v>
-      </c>
-      <c r="GQ2" t="s">
-        <v>283</v>
-      </c>
-      <c r="GR2" t="s">
-        <v>284</v>
-      </c>
-      <c r="GS2" t="s">
-        <v>285</v>
-      </c>
-      <c r="GT2" t="s">
-        <v>286</v>
-      </c>
-      <c r="GU2" t="s">
-        <v>287</v>
-      </c>
-      <c r="GV2" t="s">
-        <v>288</v>
-      </c>
-      <c r="GW2" t="s">
-        <v>246</v>
+        <v>222</v>
       </c>
     </row>
   </sheetData>
   <dataValidations count="63">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E2" xr:uid="{00000000-0002-0000-0000-000000000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D2" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"Belum Menikah,Menikah,Cerai Mati,Cerai Hidup"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F2:G2 I2:J2 L2:U2 Z2:AF2 AJ2 AM2:AN2 AQ2 AT2 AW2 AZ2 BC2 BL2 BS2 BY2 CA2:CG2 DK2 DO2:DR2 DU2:DY2 EZ2:FA2 FC2:FD2 FH2:FK2" xr:uid="{00000000-0002-0000-0000-000001000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F2:G2 I2:Q2 V2:AB2 AF2 AI2:AJ2 AM2 AP2 AS2 AV2 AY2 BG2 BM2 BS2 BU2:CA2 DE2 DI2:DL2 DN2:DR2 EM2:EN2 EO2:EP2 ES2:EV2" xr:uid="{00000000-0002-0000-0000-000001000000}">
       <formula1>"Ya,Tidak"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H2" xr:uid="{00000000-0002-0000-0000-000002000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E2" xr:uid="{00000000-0002-0000-0000-000002000000}">
       <formula1>"Non disabilitas,Penyandang disabilitas"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K2 AG2 CU2:DB2 DF2:DG2 DJ2 DT2 GS2 GV2 EE2" xr:uid="{00000000-0002-0000-0000-000003000000}"/>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="V2:Y2" xr:uid="{00000000-0002-0000-0000-000004000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H2 AC2 CO2:CV2 CZ2:DA2 DD2 DM2 FU2 FX2 DW2" xr:uid="{00000000-0002-0000-0000-000003000000}"/>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="R2:U2" xr:uid="{00000000-0002-0000-0000-000004000000}">
       <formula1>"Tidak sama sekali,Kurang dari 1 minggu,Lebih dari 1 minggu,Hampir setiap hari"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AL2" xr:uid="{00000000-0002-0000-0000-000005000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AH2" xr:uid="{00000000-0002-0000-0000-000005000000}">
       <formula1>"1 s.d &lt;10 tahun lalu,10 s.d &lt;15 tahun lalu,15 tahun lalu atau lebih"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BG2 BK2 BQ2:BR2 DS2 EA2 EF2 EI2 EL2 EN2 EY2 FB2 FE2 FL2 FN2 FS2 FV2 FZ2 GE2 GH2 GK2 GO2" xr:uid="{00000000-0002-0000-0000-000006000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BF2 BL2" xr:uid="{00000000-0002-0000-0000-000006000000}">
       <formula1>"True,False"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DZ2" xr:uid="{00000000-0002-0000-0000-000007000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DS2" xr:uid="{00000000-0002-0000-0000-000007000000}">
       <formula1>"Normal,Abnormal TBC,Abnormal non TBC"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="EB2" xr:uid="{00000000-0002-0000-0000-000008000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DT2" xr:uid="{00000000-0002-0000-0000-000008000000}">
       <formula1>"Riwayat kontak serumah,Riwayat kontak erat,Tidak ada,Tidak diketahui"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="EC2" xr:uid="{00000000-0002-0000-0000-000009000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DU2" xr:uid="{00000000-0002-0000-0000-000009000000}">
       <formula1>"Bakteriologis,Klinis"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="ED2" xr:uid="{00000000-0002-0000-0000-00000A000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DV2" xr:uid="{00000000-0002-0000-0000-00000A000000}">
       <formula1>"TCM,BTA,NPOC,Tidak dilakukan"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="EG2" xr:uid="{00000000-0002-0000-0000-00000B000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DX2" xr:uid="{00000000-0002-0000-0000-00000B000000}">
       <formula1>"Suspek frambusia,Bukan frambusia,Tidak Ada"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="EH2" xr:uid="{00000000-0002-0000-0000-00000C000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DY2" xr:uid="{00000000-0002-0000-0000-00000C000000}">
       <formula1>"Reaktif,Non Reaktif"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="EJ2" xr:uid="{00000000-0002-0000-0000-00000D000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DZ2" xr:uid="{00000000-0002-0000-0000-00000D000000}">
       <formula1>"Kusta,Bukan kusta,Meragukan,Tidak Ada"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="EK2" xr:uid="{00000000-0002-0000-0000-00000E000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="EA2" xr:uid="{00000000-0002-0000-0000-00000E000000}">
       <formula1>"Kusta,Bukan kusta,Meragukan"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="EM2" xr:uid="{00000000-0002-0000-0000-00000F000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="EB2" xr:uid="{00000000-0002-0000-0000-00000F000000}">
       <formula1>"Skabies,Bukan Skabies,Meragukan,Tidak Ada"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="EO2" xr:uid="{00000000-0002-0000-0000-000010000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="EC2" xr:uid="{00000000-0002-0000-0000-000010000000}">
       <formula1>"Tidak ada serumen impaksi,Ada serumen impaksi"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="EP2" xr:uid="{00000000-0002-0000-0000-000011000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="ED2" xr:uid="{00000000-0002-0000-0000-000011000000}">
       <formula1>"Tidak ada infeksi telinga,Ada infeksi telinga"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="EQ2" xr:uid="{00000000-0002-0000-0000-000012000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="EE2" xr:uid="{00000000-0002-0000-0000-000012000000}">
       <formula1>"Normal,Curiga gangguan pendengaran"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="ER2" xr:uid="{00000000-0002-0000-0000-000013000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="EF2" xr:uid="{00000000-0002-0000-0000-000013000000}">
       <formula1>"Normal,Gangguan Pendengaran"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="ES2" xr:uid="{00000000-0002-0000-0000-000014000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="EG2" xr:uid="{00000000-0002-0000-0000-000014000000}">
       <formula1>"Normal (visus 6/6 - 6/12),Curiga gangguan penglihatan (visus &lt;6/12)"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="ET2" xr:uid="{00000000-0002-0000-0000-000015000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="EH2" xr:uid="{00000000-0002-0000-0000-000015000000}">
       <formula1>"Normal (visus 6/6 - 6/12),Gangguan penglihatan ringan (visus &lt;6/12 - 6/18),Gangguan penglihatan sedang (&lt;6/18 - 6/60),Gangguan penglihatan berat (&lt;6/60 - 3/60),Buta (&lt;3/60)"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="EU2" xr:uid="{00000000-0002-0000-0000-000016000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="EI2" xr:uid="{00000000-0002-0000-0000-000016000000}">
       <formula1>"Visus membaik,Visus tidak membaik (visus tetap)"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="EV2" xr:uid="{00000000-0002-0000-0000-000017000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="EJ2" xr:uid="{00000000-0002-0000-0000-000017000000}">
       <formula1>"Kelainan refraksi ringan (0.50 - 3.00 Dioptri),Kelainan refraksi sedang (3.00 - 6.00 Dioptri),Kelainan refraksi berat (&gt;6.00 Dioptri)"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="EW2" xr:uid="{00000000-0002-0000-0000-000018000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="EK2" xr:uid="{00000000-0002-0000-0000-000018000000}">
       <formula1>"Normal,Curiga kelainan mata"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="EX2" xr:uid="{00000000-0002-0000-0000-000019000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="EL2" xr:uid="{00000000-0002-0000-0000-000019000000}">
       <formula1>"Curiga katarak,Normal"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="FF2" xr:uid="{00000000-0002-0000-0000-00001A000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="EQ2" xr:uid="{00000000-0002-0000-0000-00001A000000}">
       <formula1>"Iya,Tidak"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="FG2" xr:uid="{00000000-0002-0000-0000-00001B000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="ER2" xr:uid="{00000000-0002-0000-0000-00001B000000}">
       <formula1>"&lt;20 bungkus per tahun,20-30 bungkus per tahun,&gt;30 bungkus per tahun"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="FW2" xr:uid="{00000000-0002-0000-0000-00001C000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="FD2" xr:uid="{00000000-0002-0000-0000-00001C000000}">
       <formula1>"HBsAg Non Reaktif,HBsAg Reaktif"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="FX2" xr:uid="{00000000-0002-0000-0000-00001D000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="FE2" xr:uid="{00000000-0002-0000-0000-00001D000000}">
       <formula1>"Anti HCV Non Reaktif,Anti HCV Reaktif"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="FY2" xr:uid="{00000000-0002-0000-0000-00001E000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="FF2" xr:uid="{00000000-0002-0000-0000-00001E000000}">
       <formula1>"VL HCV RNA Negatif,VL HCV RNA Positif"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="GI2" xr:uid="{00000000-0002-0000-0000-00001F000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="FM2" xr:uid="{00000000-0002-0000-0000-00001F000000}">
       <formula1>"Normal,Abnormal"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="GJ2" xr:uid="{00000000-0002-0000-0000-000020000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="FN2" xr:uid="{00000000-0002-0000-0000-000020000000}">
       <formula1>"Normal,Abnormal ST Depresi,Abnormal T Inversi,Abnormal Hipertrofi Ventrikel Kiri,Abnormal Atrial Fibrilasi,Abnormal Q-Patologis,Abnormal ST Elevasi,Abnormal Gambaran Abnormal Lainnya"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="GL2" xr:uid="{00000000-0002-0000-0000-000021000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="FO2" xr:uid="{00000000-0002-0000-0000-000021000000}">
       <formula1>"Bersedia,Menolak,Tidak tahu"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="GM2" xr:uid="{00000000-0002-0000-0000-000022000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="FP2" xr:uid="{00000000-0002-0000-0000-000022000000}">
       <formula1>"Ditemukan benjolan,Tidak ditemukan benjolan"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="GN2" xr:uid="{00000000-0002-0000-0000-000023000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="FQ2" xr:uid="{00000000-0002-0000-0000-000023000000}">
       <formula1>"Negatif,Positif"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="GP2" xr:uid="{00000000-0002-0000-0000-000024000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="FR2" xr:uid="{00000000-0002-0000-0000-000024000000}">
       <formula1>"Memiliki diagnosis kanker &gt;5 tahun yang lalu,Memiliki diagnosis kanker &lt;5 tahun yang lalu,Tidak pernah didiagnosis menderita kanker"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="GQ2" xr:uid="{00000000-0002-0000-0000-000025000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="FS2" xr:uid="{00000000-0002-0000-0000-000025000000}">
       <formula1>"Memiliki keluarga yang terdiagnosis kanker paru,Memiliki keluarga yang terdiagnosis kanker lain,Tidak ada keluarga yang terdiagnosis kanker"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="GR2" xr:uid="{00000000-0002-0000-0000-000026000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="FT2" xr:uid="{00000000-0002-0000-0000-000026000000}">
       <formula1>"Perokok aktif (dalam 1 tahun ini masih merokok),Perokok/bekas perokok berhenti &lt;10 tahun lalu,Perokok pasif dari lingkungan rumah/tempat kerja,Tidak pernah merokok"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="GT2" xr:uid="{00000000-0002-0000-0000-000027000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="FV2" xr:uid="{00000000-0002-0000-0000-000027000000}">
       <formula1>"Memiliki tempat tinggal berpotensi tinggi,Tidak yakin memiliki tempat tinggal berpotensi tinggi,Tidak memiliki tempat tinggal berpotensi tinggi"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="GU2" xr:uid="{00000000-0002-0000-0000-000028000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="FW2" xr:uid="{00000000-0002-0000-0000-000028000000}">
       <formula1>"Memiliki lingkungan dalam rumah yang tidak sehat,Tidak yakin memiliki lingkungan dalam rumah yang tidak sehat,Memiliki lingkungan dalam rumah yang sehat"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="GW2" xr:uid="{00000000-0002-0000-0000-000029000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="FY2" xr:uid="{00000000-0002-0000-0000-000029000000}">
       <formula1>"Normal,Tidak Normal"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BZ2" xr:uid="{00000000-0002-0000-0000-00002A000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BT2" xr:uid="{00000000-0002-0000-0000-00002A000000}">
       <formula1>"Benar semua,Salah satu/Dua,Tidak Tahu"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CH2" xr:uid="{00000000-0002-0000-0000-00002B000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CB2" xr:uid="{00000000-0002-0000-0000-00002B000000}">
       <formula1>"Tidak terkendali/tak teratur (perlu pencahar),Kadang-kadang tak terkendali (1 x / minggu),Terkendali teratur"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CI2" xr:uid="{00000000-0002-0000-0000-00002C000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CC2" xr:uid="{00000000-0002-0000-0000-00002C000000}">
       <formula1>"Tak terkendali atau pakai kateter,Kadang-kadang tak terkendali (hanya 1 x / 24 jam),Mandiri"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CJ2" xr:uid="{00000000-0002-0000-0000-00002D000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CD2" xr:uid="{00000000-0002-0000-0000-00002D000000}">
       <formula1>"Mandiri,Butuh pertolongan orang lain"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CK2" xr:uid="{00000000-0002-0000-0000-00002E000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CE2" xr:uid="{00000000-0002-0000-0000-00002E000000}">
       <formula1>"Tergantung pertolongan orang lain,Perlu pertolongan pada beberapa kegiatan tetapi dapat mengerjakan sendiri beberapa kegiatan yang lain,Mandiri"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CL2" xr:uid="{00000000-0002-0000-0000-00002F000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CF2" xr:uid="{00000000-0002-0000-0000-00002F000000}">
       <formula1>"Tidak mampu,Perlu ditolong memotong makanan,Mandiri"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CM2" xr:uid="{00000000-0002-0000-0000-000030000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CG2" xr:uid="{00000000-0002-0000-0000-000030000000}">
       <formula1>"Tidak mampu,Perlu banyak bantuan untuk bias duduk (2 orang),Bantuan minimal 1 orang,Mandiri"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CN2" xr:uid="{00000000-0002-0000-0000-000031000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CH2" xr:uid="{00000000-0002-0000-0000-000031000000}">
       <formula1>"Tidak mampu,Bisa (pindah) dengan kursi roda,Bantuan minimal 1 orang,Mandiri"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CO2" xr:uid="{00000000-0002-0000-0000-000032000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CI2" xr:uid="{00000000-0002-0000-0000-000032000000}">
       <formula1>"Tergantung orang lain,Sebagian dibantu (misalnya: mengancing baju),Mandiri"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CP2" xr:uid="{00000000-0002-0000-0000-000033000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CJ2" xr:uid="{00000000-0002-0000-0000-000033000000}">
       <formula1>"Tidak mampu,Butuh pertolongan,Mandiri"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CQ2" xr:uid="{00000000-0002-0000-0000-000034000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CK2" xr:uid="{00000000-0002-0000-0000-000034000000}">
       <formula1>"Tergantung orang lain,Mandiri"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CR2" xr:uid="{00000000-0002-0000-0000-000035000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CL2" xr:uid="{00000000-0002-0000-0000-000035000000}">
       <formula1>"SUDAH DITANYAKAN"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CS2" xr:uid="{00000000-0002-0000-0000-000036000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CM2" xr:uid="{00000000-0002-0000-0000-000036000000}">
       <formula1>"Benar,Salah"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CT2" xr:uid="{00000000-0002-0000-0000-000037000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CN2" xr:uid="{00000000-0002-0000-0000-000037000000}">
       <formula1>"Benar 1 kata,Benar 2 Kata,Benar semua kata,Tidak dapat mengingat/mengulang kata"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DC2:DD2" xr:uid="{00000000-0002-0000-0000-000038000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CW2:CX2" xr:uid="{00000000-0002-0000-0000-000038000000}">
       <formula1>"Bertahan 10 detik,Tidak bertahan 10 detik,Tidak dilakukan"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DE2" xr:uid="{00000000-0002-0000-0000-000039000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CY2" xr:uid="{00000000-0002-0000-0000-000039000000}">
       <formula1>"Bertahan 10 detik,Bertahan 3 - 9.99 detik,Bertahan &lt; 3 detik"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DH2" xr:uid="{00000000-0002-0000-0000-00003A000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DB2" xr:uid="{00000000-0002-0000-0000-00003A000000}">
       <formula1>"Nafsu Makan Yang Sangat Berkurang,Nafsu Makan Sedikit Berkurang,Nafsu Makan Biasa saja"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DI2" xr:uid="{00000000-0002-0000-0000-00003B000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DC2" xr:uid="{00000000-0002-0000-0000-00003B000000}">
       <formula1>"Penurunan BB &gt; 3 Kg,Tidak Tahu,Penurunan BB antara 1 - 3 Kg"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DL2" xr:uid="{00000000-0002-0000-0000-00003C000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DF2" xr:uid="{00000000-0002-0000-0000-00003C000000}">
       <formula1>"Dementia atau depresi berat,Demensia/kepikunan ringan,Tidak ada masalah psikologis"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DM2" xr:uid="{00000000-0002-0000-0000-00003D000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DG2" xr:uid="{00000000-0002-0000-0000-00003D000000}">
       <formula1>"IMT &lt;19,IMT 19 - &lt;21,IMT 21 - &lt;23,IMT &gt;= 23"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DN2" xr:uid="{00000000-0002-0000-0000-00003E000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DH2" xr:uid="{00000000-0002-0000-0000-00003E000000}">
       <formula1>"&lt;31 cm,&gt;= 31 cm"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
fix: stage 5 fixing skrining-filtering, doing excel modification for lansia and screening nakes
</commit_message>
<xml_diff>
--- a/dataset/lansia.xlsx
+++ b/dataset/lansia.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/macbokprom12021/PycharmProjects/CKG-Helper/dataset/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4599B17E-0406-F34F-ACA0-CBC5941630B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E1CCC735-F43A-9D4B-B979-9FBFEDDA1110}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="22500" yWindow="-21000" windowWidth="19200" windowHeight="21000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3300" yWindow="-21000" windowWidth="38400" windowHeight="21000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -358,7 +358,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="BV1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000017000000}">
+    <comment ref="BW1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000017000000}">
       <text>
         <r>
           <rPr>
@@ -373,7 +373,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="EA1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000018000000}">
+    <comment ref="EM1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000018000000}">
       <text>
         <r>
           <rPr>
@@ -388,7 +388,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="EC1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000019000000}">
+    <comment ref="EP1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000019000000}">
       <text>
         <r>
           <rPr>
@@ -403,7 +403,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="EG1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00001A000000}">
+    <comment ref="EU1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00001A000000}">
       <text>
         <r>
           <rPr>
@@ -418,7 +418,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="EI1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00001B000000}">
+    <comment ref="EX1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00001B000000}">
       <text>
         <r>
           <rPr>
@@ -433,7 +433,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="EN1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00001C000000}">
+    <comment ref="FE1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00001C000000}">
       <text>
         <r>
           <rPr>
@@ -448,7 +448,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="EP1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00001D000000}">
+    <comment ref="FG1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00001D000000}">
       <text>
         <r>
           <rPr>
@@ -463,7 +463,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="EQ1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00001E000000}">
+    <comment ref="FH1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00001E000000}">
       <text>
         <r>
           <rPr>
@@ -478,7 +478,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="ER1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00001F000000}">
+    <comment ref="FI1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00001F000000}">
       <text>
         <r>
           <rPr>
@@ -493,7 +493,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="ES1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000020000000}">
+    <comment ref="FJ1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000020000000}">
       <text>
         <r>
           <rPr>
@@ -508,7 +508,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="EZ1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000021000000}">
+    <comment ref="FT1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000021000000}">
       <text>
         <r>
           <rPr>
@@ -523,7 +523,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="FN1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000022000000}">
+    <comment ref="GL1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000022000000}">
       <text>
         <r>
           <rPr>
@@ -543,7 +543,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="686" uniqueCount="275">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="806" uniqueCount="301">
   <si>
     <t>batas_awal</t>
   </si>
@@ -713,9 +713,6 @@
     <t>lingkar_perut</t>
   </si>
   <si>
-    <t>periksa_gula_darah</t>
-  </si>
-  <si>
     <t>pernah_diabetes</t>
   </si>
   <si>
@@ -1130,9 +1127,6 @@
     <t>90</t>
   </si>
   <si>
-    <t>True</t>
-  </si>
-  <si>
     <t>12</t>
   </si>
   <si>
@@ -1368,6 +1362,90 @@
   </si>
   <si>
     <t>skrining_aktivitas_fisik</t>
+  </si>
+  <si>
+    <t>skrining_gizi</t>
+  </si>
+  <si>
+    <t>skrining_gula_darah_dewasa</t>
+  </si>
+  <si>
+    <t>skrining_tekanan_darah_dewasa</t>
+  </si>
+  <si>
+    <t>skrining_skilas_penurunan_kognitif</t>
+  </si>
+  <si>
+    <t>skrining_skilas_mobilisasi</t>
+  </si>
+  <si>
+    <t>skrining_skilas_malnutrisi</t>
+  </si>
+  <si>
+    <t>skrining_skilas_depresi</t>
+  </si>
+  <si>
+    <t>skrining_gangguan_fungsional</t>
+  </si>
+  <si>
+    <t>skrining_mini_cog</t>
+  </si>
+  <si>
+    <t>skrining_ad8_ina</t>
+  </si>
+  <si>
+    <t>skrining_mobilisasi_lanjutan</t>
+  </si>
+  <si>
+    <t>skrining_malnutrisi_lanjutan</t>
+  </si>
+  <si>
+    <t>skrining_depresi_lanjutan</t>
+  </si>
+  <si>
+    <t>skrining_tb</t>
+  </si>
+  <si>
+    <t>skrining_frambusia</t>
+  </si>
+  <si>
+    <t>skrining_kusta</t>
+  </si>
+  <si>
+    <t>skrining_skabies</t>
+  </si>
+  <si>
+    <t>skrining_telinga_mata</t>
+  </si>
+  <si>
+    <t>skrining_karies</t>
+  </si>
+  <si>
+    <t>skrining_periodontal</t>
+  </si>
+  <si>
+    <t>skrining_ppok</t>
+  </si>
+  <si>
+    <t>skrining_kadar_co</t>
+  </si>
+  <si>
+    <t>skrining_lipid</t>
+  </si>
+  <si>
+    <t>skrining_fibrosis</t>
+  </si>
+  <si>
+    <t>skrining_hepatitis</t>
+  </si>
+  <si>
+    <t>skrining_fungsi_ginjal</t>
+  </si>
+  <si>
+    <t>skrining_kerusakan_ginjal</t>
+  </si>
+  <si>
+    <t>skrining_jantung</t>
   </si>
 </sst>
 </file>
@@ -1778,7 +1856,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:GH19"/>
+  <dimension ref="A1:HK19"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="17.5" style="1" bestFit="1" customWidth="1"/>
@@ -1839,104 +1917,136 @@
     <col min="59" max="59" width="18.33203125" bestFit="1" customWidth="1"/>
     <col min="60" max="60" width="12.1640625" bestFit="1" customWidth="1"/>
     <col min="61" max="61" width="19.33203125" bestFit="1" customWidth="1"/>
-    <col min="62" max="62" width="13.83203125" customWidth="1"/>
+    <col min="62" max="62" width="14.83203125" style="3" bestFit="1" customWidth="1"/>
     <col min="63" max="65" width="14.33203125" customWidth="1"/>
-    <col min="66" max="66" width="17.1640625" bestFit="1" customWidth="1"/>
+    <col min="66" max="66" width="17.1640625" style="3" bestFit="1" customWidth="1"/>
     <col min="67" max="67" width="14.83203125" bestFit="1" customWidth="1"/>
     <col min="68" max="68" width="18.5" bestFit="1" customWidth="1"/>
     <col min="69" max="69" width="18" bestFit="1" customWidth="1"/>
     <col min="70" max="70" width="19.83203125" bestFit="1" customWidth="1"/>
     <col min="71" max="72" width="17.1640625" customWidth="1"/>
-    <col min="73" max="73" width="16" bestFit="1" customWidth="1"/>
-    <col min="74" max="74" width="19.6640625" bestFit="1" customWidth="1"/>
-    <col min="75" max="75" width="6.83203125" bestFit="1" customWidth="1"/>
-    <col min="76" max="76" width="8" bestFit="1" customWidth="1"/>
-    <col min="77" max="77" width="8.83203125" bestFit="1" customWidth="1"/>
-    <col min="78" max="78" width="9.83203125" bestFit="1" customWidth="1"/>
-    <col min="79" max="79" width="16" bestFit="1" customWidth="1"/>
-    <col min="80" max="80" width="21" bestFit="1" customWidth="1"/>
-    <col min="81" max="81" width="23.6640625" bestFit="1" customWidth="1"/>
-    <col min="82" max="82" width="13.6640625" bestFit="1" customWidth="1"/>
-    <col min="83" max="83" width="20.5" bestFit="1" customWidth="1"/>
-    <col min="84" max="84" width="18" bestFit="1" customWidth="1"/>
-    <col min="85" max="85" width="15.5" bestFit="1" customWidth="1"/>
-    <col min="86" max="86" width="21.83203125" bestFit="1" customWidth="1"/>
-    <col min="87" max="87" width="21.1640625" bestFit="1" customWidth="1"/>
-    <col min="88" max="88" width="11" bestFit="1" customWidth="1"/>
-    <col min="89" max="89" width="42.1640625" bestFit="1" customWidth="1"/>
-    <col min="90" max="90" width="17.1640625" bestFit="1" customWidth="1"/>
-    <col min="91" max="91" width="18.1640625" bestFit="1" customWidth="1"/>
-    <col min="92" max="93" width="18.1640625" customWidth="1"/>
-    <col min="94" max="94" width="27.1640625" bestFit="1" customWidth="1"/>
-    <col min="95" max="95" width="40" bestFit="1" customWidth="1"/>
-    <col min="96" max="96" width="16" bestFit="1" customWidth="1"/>
-    <col min="97" max="97" width="16" customWidth="1"/>
-    <col min="98" max="98" width="18.1640625" bestFit="1" customWidth="1"/>
-    <col min="99" max="99" width="10.5" bestFit="1" customWidth="1"/>
-    <col min="100" max="100" width="15.83203125" bestFit="1" customWidth="1"/>
-    <col min="101" max="104" width="15.83203125" customWidth="1"/>
-    <col min="105" max="108" width="12.6640625" bestFit="1" customWidth="1"/>
-    <col min="109" max="115" width="10.5" customWidth="1"/>
-    <col min="116" max="116" width="18.33203125" customWidth="1"/>
-    <col min="117" max="124" width="10.5" customWidth="1"/>
-    <col min="125" max="125" width="25" bestFit="1" customWidth="1"/>
-    <col min="126" max="126" width="8.33203125" bestFit="1" customWidth="1"/>
-    <col min="127" max="127" width="19.6640625" bestFit="1" customWidth="1"/>
-    <col min="128" max="128" width="17.1640625" bestFit="1" customWidth="1"/>
-    <col min="129" max="129" width="23.5" bestFit="1" customWidth="1"/>
-    <col min="130" max="130" width="14.83203125" bestFit="1" customWidth="1"/>
-    <col min="131" max="131" width="14.83203125" customWidth="1"/>
-    <col min="132" max="132" width="21.33203125" bestFit="1" customWidth="1"/>
-    <col min="133" max="133" width="11.6640625" bestFit="1" customWidth="1"/>
-    <col min="134" max="134" width="22.83203125" bestFit="1" customWidth="1"/>
-    <col min="135" max="135" width="22.83203125" customWidth="1"/>
-    <col min="136" max="136" width="16.1640625" customWidth="1"/>
-    <col min="137" max="137" width="19.83203125" bestFit="1" customWidth="1"/>
-    <col min="138" max="139" width="12.33203125" customWidth="1"/>
-    <col min="140" max="140" width="14.1640625" customWidth="1"/>
-    <col min="141" max="141" width="23.6640625" bestFit="1" customWidth="1"/>
-    <col min="142" max="142" width="23.6640625" customWidth="1"/>
-    <col min="143" max="143" width="26" bestFit="1" customWidth="1"/>
-    <col min="144" max="144" width="26" customWidth="1"/>
-    <col min="145" max="145" width="36.1640625" bestFit="1" customWidth="1"/>
-    <col min="146" max="146" width="41.5" bestFit="1" customWidth="1"/>
-    <col min="147" max="147" width="13.5" bestFit="1" customWidth="1"/>
-    <col min="148" max="148" width="20.33203125" bestFit="1" customWidth="1"/>
-    <col min="149" max="149" width="9.83203125" bestFit="1" customWidth="1"/>
-    <col min="150" max="150" width="12.83203125" bestFit="1" customWidth="1"/>
-    <col min="151" max="152" width="12.83203125" customWidth="1"/>
-    <col min="153" max="153" width="18.5" bestFit="1" customWidth="1"/>
-    <col min="154" max="154" width="17.5" customWidth="1"/>
-    <col min="155" max="155" width="13" bestFit="1" customWidth="1"/>
-    <col min="156" max="156" width="19.5" bestFit="1" customWidth="1"/>
-    <col min="157" max="157" width="12.33203125" bestFit="1" customWidth="1"/>
-    <col min="158" max="160" width="19.5" customWidth="1"/>
-    <col min="161" max="161" width="9.83203125" customWidth="1"/>
-    <col min="162" max="165" width="11.5" customWidth="1"/>
-    <col min="166" max="166" width="4.5" bestFit="1" customWidth="1"/>
-    <col min="167" max="167" width="9" bestFit="1" customWidth="1"/>
-    <col min="168" max="168" width="16.1640625" bestFit="1" customWidth="1"/>
-    <col min="169" max="169" width="18.1640625" bestFit="1" customWidth="1"/>
-    <col min="170" max="170" width="18.1640625" customWidth="1"/>
-    <col min="171" max="171" width="8.33203125" bestFit="1" customWidth="1"/>
-    <col min="172" max="174" width="8.33203125" customWidth="1"/>
-    <col min="175" max="175" width="7.6640625" bestFit="1" customWidth="1"/>
-    <col min="176" max="176" width="12.33203125" bestFit="1" customWidth="1"/>
-    <col min="177" max="177" width="14" customWidth="1"/>
-    <col min="178" max="178" width="15.5" bestFit="1" customWidth="1"/>
-    <col min="179" max="179" width="18.1640625" customWidth="1"/>
-    <col min="180" max="180" width="17.6640625" bestFit="1" customWidth="1"/>
-    <col min="181" max="181" width="11.83203125" bestFit="1" customWidth="1"/>
-    <col min="182" max="184" width="18.1640625" customWidth="1"/>
-    <col min="185" max="185" width="46.33203125" bestFit="1" customWidth="1"/>
-    <col min="186" max="186" width="35" bestFit="1" customWidth="1"/>
-    <col min="187" max="187" width="43.1640625" bestFit="1" customWidth="1"/>
-    <col min="188" max="188" width="18.1640625" customWidth="1"/>
-    <col min="189" max="189" width="9.33203125" bestFit="1" customWidth="1"/>
-    <col min="190" max="190" width="10.83203125" customWidth="1"/>
+    <col min="73" max="73" width="28.1640625" style="3" bestFit="1" customWidth="1"/>
+    <col min="74" max="74" width="16" bestFit="1" customWidth="1"/>
+    <col min="75" max="75" width="19.6640625" bestFit="1" customWidth="1"/>
+    <col min="76" max="76" width="6.83203125" bestFit="1" customWidth="1"/>
+    <col min="77" max="77" width="8" bestFit="1" customWidth="1"/>
+    <col min="78" max="78" width="8.83203125" bestFit="1" customWidth="1"/>
+    <col min="79" max="79" width="9.83203125" bestFit="1" customWidth="1"/>
+    <col min="80" max="80" width="30" style="3" bestFit="1" customWidth="1"/>
+    <col min="81" max="81" width="16" bestFit="1" customWidth="1"/>
+    <col min="82" max="82" width="21" bestFit="1" customWidth="1"/>
+    <col min="83" max="83" width="23.6640625" bestFit="1" customWidth="1"/>
+    <col min="84" max="84" width="23.6640625" style="3" customWidth="1"/>
+    <col min="85" max="85" width="13.6640625" bestFit="1" customWidth="1"/>
+    <col min="86" max="86" width="22" style="3" bestFit="1" customWidth="1"/>
+    <col min="87" max="87" width="20.5" bestFit="1" customWidth="1"/>
+    <col min="88" max="88" width="18" bestFit="1" customWidth="1"/>
+    <col min="89" max="89" width="15.5" bestFit="1" customWidth="1"/>
+    <col min="90" max="90" width="19.6640625" style="3" bestFit="1" customWidth="1"/>
+    <col min="91" max="91" width="21.83203125" bestFit="1" customWidth="1"/>
+    <col min="92" max="92" width="21.1640625" bestFit="1" customWidth="1"/>
+    <col min="93" max="93" width="25" style="3" bestFit="1" customWidth="1"/>
+    <col min="94" max="94" width="11" bestFit="1" customWidth="1"/>
+    <col min="95" max="95" width="42.1640625" bestFit="1" customWidth="1"/>
+    <col min="96" max="96" width="17.1640625" bestFit="1" customWidth="1"/>
+    <col min="97" max="97" width="18.1640625" bestFit="1" customWidth="1"/>
+    <col min="98" max="99" width="18.1640625" customWidth="1"/>
+    <col min="100" max="100" width="27.1640625" bestFit="1" customWidth="1"/>
+    <col min="101" max="101" width="40" bestFit="1" customWidth="1"/>
+    <col min="102" max="102" width="16" bestFit="1" customWidth="1"/>
+    <col min="103" max="103" width="16" customWidth="1"/>
+    <col min="104" max="104" width="16" style="3" customWidth="1"/>
+    <col min="105" max="105" width="18.1640625" bestFit="1" customWidth="1"/>
+    <col min="106" max="106" width="10.5" bestFit="1" customWidth="1"/>
+    <col min="107" max="107" width="15.83203125" bestFit="1" customWidth="1"/>
+    <col min="108" max="108" width="15.83203125" style="3" customWidth="1"/>
+    <col min="109" max="112" width="15.83203125" customWidth="1"/>
+    <col min="113" max="116" width="12.6640625" bestFit="1" customWidth="1"/>
+    <col min="117" max="117" width="24.1640625" style="3" bestFit="1" customWidth="1"/>
+    <col min="118" max="122" width="10.5" customWidth="1"/>
+    <col min="123" max="123" width="24.1640625" style="3" bestFit="1" customWidth="1"/>
+    <col min="124" max="125" width="10.5" customWidth="1"/>
+    <col min="126" max="126" width="18.33203125" customWidth="1"/>
+    <col min="127" max="130" width="10.5" customWidth="1"/>
+    <col min="131" max="131" width="22" style="3" bestFit="1" customWidth="1"/>
+    <col min="132" max="134" width="10.5" customWidth="1"/>
+    <col min="135" max="135" width="16.6640625" bestFit="1" customWidth="1"/>
+    <col min="136" max="136" width="15" style="3" bestFit="1" customWidth="1"/>
+    <col min="137" max="137" width="25" bestFit="1" customWidth="1"/>
+    <col min="138" max="138" width="8.33203125" bestFit="1" customWidth="1"/>
+    <col min="139" max="139" width="19.6640625" bestFit="1" customWidth="1"/>
+    <col min="140" max="140" width="17.1640625" bestFit="1" customWidth="1"/>
+    <col min="141" max="141" width="23.5" bestFit="1" customWidth="1"/>
+    <col min="142" max="142" width="14.83203125" bestFit="1" customWidth="1"/>
+    <col min="143" max="143" width="14.83203125" customWidth="1"/>
+    <col min="144" max="144" width="14.83203125" style="3" customWidth="1"/>
+    <col min="145" max="145" width="21.33203125" bestFit="1" customWidth="1"/>
+    <col min="146" max="146" width="11.6640625" bestFit="1" customWidth="1"/>
+    <col min="147" max="147" width="22.83203125" bestFit="1" customWidth="1"/>
+    <col min="148" max="148" width="22.83203125" customWidth="1"/>
+    <col min="149" max="149" width="22.83203125" style="3" customWidth="1"/>
+    <col min="150" max="150" width="16.1640625" customWidth="1"/>
+    <col min="151" max="151" width="19.83203125" bestFit="1" customWidth="1"/>
+    <col min="152" max="152" width="19.83203125" style="3" customWidth="1"/>
+    <col min="153" max="154" width="12.33203125" customWidth="1"/>
+    <col min="155" max="155" width="14.1640625" style="3" bestFit="1" customWidth="1"/>
+    <col min="156" max="156" width="14.1640625" customWidth="1"/>
+    <col min="157" max="157" width="18.83203125" style="3" bestFit="1" customWidth="1"/>
+    <col min="158" max="158" width="23.6640625" bestFit="1" customWidth="1"/>
+    <col min="159" max="159" width="23.6640625" customWidth="1"/>
+    <col min="160" max="160" width="26" bestFit="1" customWidth="1"/>
+    <col min="161" max="161" width="26" customWidth="1"/>
+    <col min="162" max="162" width="36.1640625" bestFit="1" customWidth="1"/>
+    <col min="163" max="163" width="41.5" bestFit="1" customWidth="1"/>
+    <col min="164" max="164" width="13.5" bestFit="1" customWidth="1"/>
+    <col min="165" max="165" width="20.33203125" bestFit="1" customWidth="1"/>
+    <col min="166" max="166" width="9.83203125" bestFit="1" customWidth="1"/>
+    <col min="167" max="167" width="12.83203125" bestFit="1" customWidth="1"/>
+    <col min="168" max="168" width="12.83203125" style="3" customWidth="1"/>
+    <col min="169" max="170" width="12.83203125" customWidth="1"/>
+    <col min="171" max="171" width="17.6640625" style="3" bestFit="1" customWidth="1"/>
+    <col min="172" max="172" width="18.5" bestFit="1" customWidth="1"/>
+    <col min="173" max="173" width="17.5" customWidth="1"/>
+    <col min="174" max="174" width="17.5" style="3" customWidth="1"/>
+    <col min="175" max="175" width="13" bestFit="1" customWidth="1"/>
+    <col min="176" max="176" width="19.5" bestFit="1" customWidth="1"/>
+    <col min="177" max="177" width="12.33203125" bestFit="1" customWidth="1"/>
+    <col min="178" max="180" width="19.5" customWidth="1"/>
+    <col min="181" max="181" width="19.5" style="3" customWidth="1"/>
+    <col min="182" max="182" width="9.83203125" customWidth="1"/>
+    <col min="183" max="183" width="11.6640625" style="3" bestFit="1" customWidth="1"/>
+    <col min="184" max="187" width="11.5" customWidth="1"/>
+    <col min="188" max="188" width="14" style="3" bestFit="1" customWidth="1"/>
+    <col min="189" max="189" width="4.5" bestFit="1" customWidth="1"/>
+    <col min="190" max="190" width="9" bestFit="1" customWidth="1"/>
+    <col min="191" max="191" width="15.33203125" style="3" bestFit="1" customWidth="1"/>
+    <col min="192" max="192" width="16.1640625" bestFit="1" customWidth="1"/>
+    <col min="193" max="193" width="18.1640625" bestFit="1" customWidth="1"/>
+    <col min="194" max="194" width="18.1640625" customWidth="1"/>
+    <col min="195" max="195" width="18.1640625" style="3" customWidth="1"/>
+    <col min="196" max="196" width="8.33203125" bestFit="1" customWidth="1"/>
+    <col min="197" max="199" width="8.33203125" customWidth="1"/>
+    <col min="200" max="200" width="21.83203125" style="3" bestFit="1" customWidth="1"/>
+    <col min="201" max="201" width="7.6640625" bestFit="1" customWidth="1"/>
+    <col min="202" max="202" width="12.33203125" bestFit="1" customWidth="1"/>
+    <col min="203" max="203" width="12.33203125" style="3" customWidth="1"/>
+    <col min="204" max="204" width="14" customWidth="1"/>
+    <col min="205" max="205" width="15.5" bestFit="1" customWidth="1"/>
+    <col min="206" max="206" width="18.1640625" style="3" bestFit="1" customWidth="1"/>
+    <col min="207" max="207" width="18.1640625" customWidth="1"/>
+    <col min="208" max="208" width="17.6640625" bestFit="1" customWidth="1"/>
+    <col min="209" max="209" width="11.83203125" bestFit="1" customWidth="1"/>
+    <col min="210" max="210" width="18.1640625" style="3" bestFit="1" customWidth="1"/>
+    <col min="211" max="213" width="18.1640625" customWidth="1"/>
+    <col min="214" max="214" width="46.33203125" bestFit="1" customWidth="1"/>
+    <col min="215" max="215" width="35" bestFit="1" customWidth="1"/>
+    <col min="216" max="216" width="43.1640625" bestFit="1" customWidth="1"/>
+    <col min="217" max="217" width="18.1640625" customWidth="1"/>
+    <col min="218" max="218" width="9.33203125" bestFit="1" customWidth="1"/>
+    <col min="219" max="219" width="10.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:190" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:219" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1947,7 +2057,7 @@
         <v>2</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="E1" t="s">
         <v>3</v>
@@ -1956,7 +2066,7 @@
         <v>4</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="H1" t="s">
         <v>5</v>
@@ -1965,13 +2075,13 @@
         <v>6</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="K1" t="s">
         <v>7</v>
       </c>
       <c r="L1" s="3" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="M1" t="s">
         <v>8</v>
@@ -2001,7 +2111,7 @@
         <v>16</v>
       </c>
       <c r="V1" s="3" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="W1" t="s">
         <v>17</v>
@@ -2016,7 +2126,7 @@
         <v>20</v>
       </c>
       <c r="AA1" s="3" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="AB1" t="s">
         <v>21</v>
@@ -2037,7 +2147,7 @@
         <v>26</v>
       </c>
       <c r="AH1" s="3" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="AI1" t="s">
         <v>27</v>
@@ -2064,7 +2174,7 @@
         <v>34</v>
       </c>
       <c r="AQ1" s="3" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
       <c r="AR1" t="s">
         <v>35</v>
@@ -2120,6 +2230,9 @@
       <c r="BI1" t="s">
         <v>52</v>
       </c>
+      <c r="BJ1" s="3" t="s">
+        <v>273</v>
+      </c>
       <c r="BK1" t="s">
         <v>53</v>
       </c>
@@ -2129,490 +2242,577 @@
       <c r="BM1" t="s">
         <v>55</v>
       </c>
-      <c r="BN1" t="s">
+      <c r="BN1" s="3" t="s">
+        <v>274</v>
+      </c>
+      <c r="BO1" t="s">
         <v>56</v>
       </c>
-      <c r="BO1" t="s">
+      <c r="BP1" t="s">
         <v>57</v>
       </c>
-      <c r="BP1" t="s">
+      <c r="BQ1" t="s">
         <v>58</v>
       </c>
-      <c r="BQ1" t="s">
+      <c r="BR1" t="s">
         <v>59</v>
       </c>
-      <c r="BR1" t="s">
+      <c r="BS1" t="s">
         <v>60</v>
       </c>
-      <c r="BS1" t="s">
+      <c r="BT1" t="s">
         <v>61</v>
       </c>
-      <c r="BT1" t="s">
+      <c r="BU1" s="3" t="s">
+        <v>275</v>
+      </c>
+      <c r="BV1" t="s">
         <v>62</v>
       </c>
-      <c r="BU1" t="s">
+      <c r="BW1" t="s">
         <v>63</v>
       </c>
-      <c r="BV1" t="s">
+      <c r="BX1" t="s">
         <v>64</v>
       </c>
-      <c r="BW1" t="s">
+      <c r="BY1" t="s">
         <v>65</v>
       </c>
-      <c r="BX1" t="s">
+      <c r="BZ1" t="s">
         <v>66</v>
       </c>
-      <c r="BY1" t="s">
+      <c r="CA1" t="s">
         <v>67</v>
       </c>
-      <c r="BZ1" t="s">
+      <c r="CB1" s="3" t="s">
+        <v>276</v>
+      </c>
+      <c r="CC1" t="s">
         <v>68</v>
       </c>
-      <c r="CA1" t="s">
+      <c r="CD1" t="s">
         <v>69</v>
       </c>
-      <c r="CB1" t="s">
+      <c r="CE1" t="s">
         <v>70</v>
       </c>
-      <c r="CC1" t="s">
+      <c r="CF1" s="3" t="s">
+        <v>277</v>
+      </c>
+      <c r="CG1" t="s">
         <v>71</v>
       </c>
-      <c r="CD1" t="s">
+      <c r="CH1" s="3" t="s">
+        <v>278</v>
+      </c>
+      <c r="CI1" t="s">
         <v>72</v>
       </c>
-      <c r="CE1" t="s">
+      <c r="CJ1" t="s">
         <v>73</v>
       </c>
-      <c r="CF1" t="s">
+      <c r="CK1" t="s">
         <v>74</v>
       </c>
-      <c r="CG1" t="s">
+      <c r="CL1" s="3" t="s">
+        <v>279</v>
+      </c>
+      <c r="CM1" t="s">
         <v>75</v>
       </c>
-      <c r="CH1" t="s">
+      <c r="CN1" t="s">
         <v>76</v>
       </c>
-      <c r="CI1" t="s">
+      <c r="CO1" s="3" t="s">
+        <v>280</v>
+      </c>
+      <c r="CP1" t="s">
         <v>77</v>
       </c>
-      <c r="CJ1" t="s">
+      <c r="CQ1" t="s">
         <v>78</v>
       </c>
-      <c r="CK1" t="s">
+      <c r="CR1" t="s">
         <v>79</v>
       </c>
-      <c r="CL1" t="s">
+      <c r="CS1" t="s">
         <v>80</v>
       </c>
-      <c r="CM1" t="s">
+      <c r="CT1" t="s">
         <v>81</v>
       </c>
-      <c r="CN1" t="s">
+      <c r="CU1" t="s">
         <v>82</v>
       </c>
-      <c r="CO1" t="s">
+      <c r="CV1" t="s">
         <v>83</v>
       </c>
-      <c r="CP1" t="s">
+      <c r="CW1" t="s">
         <v>84</v>
       </c>
-      <c r="CQ1" t="s">
+      <c r="CX1" t="s">
         <v>85</v>
       </c>
-      <c r="CR1" t="s">
+      <c r="CY1" t="s">
         <v>86</v>
       </c>
-      <c r="CS1" t="s">
+      <c r="CZ1" s="3" t="s">
+        <v>281</v>
+      </c>
+      <c r="DA1" t="s">
         <v>87</v>
       </c>
-      <c r="CT1" t="s">
+      <c r="DB1" t="s">
         <v>88</v>
       </c>
-      <c r="CU1" t="s">
+      <c r="DC1" t="s">
         <v>89</v>
       </c>
-      <c r="CV1" t="s">
+      <c r="DD1" s="3" t="s">
+        <v>282</v>
+      </c>
+      <c r="DE1" t="s">
         <v>90</v>
       </c>
-      <c r="CW1" t="s">
+      <c r="DF1" t="s">
         <v>91</v>
       </c>
-      <c r="CX1" t="s">
+      <c r="DG1" t="s">
         <v>92</v>
       </c>
-      <c r="CY1" t="s">
+      <c r="DH1" t="s">
         <v>93</v>
       </c>
-      <c r="CZ1" t="s">
+      <c r="DI1" t="s">
         <v>94</v>
       </c>
-      <c r="DA1" t="s">
+      <c r="DJ1" t="s">
         <v>95</v>
       </c>
-      <c r="DB1" t="s">
+      <c r="DK1" t="s">
         <v>96</v>
       </c>
-      <c r="DC1" t="s">
+      <c r="DL1" t="s">
         <v>97</v>
       </c>
-      <c r="DD1" t="s">
+      <c r="DM1" s="3" t="s">
+        <v>283</v>
+      </c>
+      <c r="DN1" t="s">
         <v>98</v>
       </c>
-      <c r="DE1" t="s">
+      <c r="DO1" t="s">
         <v>99</v>
       </c>
-      <c r="DF1" t="s">
+      <c r="DP1" t="s">
         <v>100</v>
       </c>
-      <c r="DG1" t="s">
+      <c r="DQ1" t="s">
         <v>101</v>
       </c>
-      <c r="DH1" t="s">
+      <c r="DR1" t="s">
         <v>102</v>
       </c>
-      <c r="DI1" t="s">
+      <c r="DS1" s="3" t="s">
+        <v>284</v>
+      </c>
+      <c r="DT1" t="s">
         <v>103</v>
       </c>
-      <c r="DJ1" t="s">
+      <c r="DU1" t="s">
         <v>104</v>
       </c>
-      <c r="DK1" t="s">
+      <c r="DV1" t="s">
         <v>105</v>
       </c>
-      <c r="DL1" t="s">
+      <c r="DW1" t="s">
         <v>106</v>
       </c>
-      <c r="DM1" t="s">
+      <c r="DX1" t="s">
         <v>107</v>
       </c>
-      <c r="DN1" t="s">
+      <c r="DY1" t="s">
         <v>108</v>
       </c>
-      <c r="DO1" t="s">
+      <c r="DZ1" t="s">
         <v>109</v>
       </c>
-      <c r="DP1" t="s">
+      <c r="EA1" s="3" t="s">
+        <v>285</v>
+      </c>
+      <c r="EB1" t="s">
         <v>110</v>
       </c>
-      <c r="DQ1" t="s">
+      <c r="EC1" t="s">
         <v>111</v>
       </c>
-      <c r="DR1" t="s">
+      <c r="ED1" t="s">
         <v>112</v>
       </c>
-      <c r="DS1" t="s">
+      <c r="EE1" t="s">
         <v>113</v>
       </c>
-      <c r="DT1" t="s">
+      <c r="EF1" s="3" t="s">
+        <v>267</v>
+      </c>
+      <c r="EG1" t="s">
         <v>114</v>
       </c>
-      <c r="DU1" t="s">
+      <c r="EH1" t="s">
         <v>115</v>
       </c>
-      <c r="DV1" t="s">
+      <c r="EI1" t="s">
         <v>116</v>
       </c>
-      <c r="DW1" t="s">
+      <c r="EJ1" t="s">
         <v>117</v>
       </c>
-      <c r="DX1" t="s">
+      <c r="EK1" t="s">
         <v>118</v>
       </c>
-      <c r="DY1" t="s">
+      <c r="EL1" t="s">
         <v>119</v>
       </c>
-      <c r="DZ1" t="s">
+      <c r="EM1" t="s">
         <v>120</v>
       </c>
-      <c r="EA1" t="s">
+      <c r="EN1" s="3" t="s">
+        <v>286</v>
+      </c>
+      <c r="EO1" t="s">
         <v>121</v>
       </c>
-      <c r="EB1" t="s">
+      <c r="EP1" t="s">
         <v>122</v>
       </c>
-      <c r="EC1" t="s">
+      <c r="EQ1" t="s">
         <v>123</v>
       </c>
-      <c r="ED1" t="s">
+      <c r="ER1" t="s">
         <v>124</v>
       </c>
-      <c r="EE1" t="s">
+      <c r="ES1" s="3" t="s">
+        <v>287</v>
+      </c>
+      <c r="ET1" t="s">
         <v>125</v>
       </c>
-      <c r="EF1" t="s">
+      <c r="EU1" t="s">
         <v>126</v>
       </c>
-      <c r="EG1" t="s">
+      <c r="EV1" s="3" t="s">
+        <v>288</v>
+      </c>
+      <c r="EW1" t="s">
         <v>127</v>
       </c>
-      <c r="EH1" t="s">
+      <c r="EX1" t="s">
         <v>128</v>
       </c>
-      <c r="EI1" t="s">
+      <c r="EY1" s="3" t="s">
+        <v>289</v>
+      </c>
+      <c r="EZ1" t="s">
         <v>129</v>
       </c>
-      <c r="EJ1" t="s">
+      <c r="FA1" s="3" t="s">
+        <v>290</v>
+      </c>
+      <c r="FB1" t="s">
         <v>130</v>
       </c>
-      <c r="EK1" t="s">
+      <c r="FC1" t="s">
         <v>131</v>
       </c>
-      <c r="EL1" t="s">
+      <c r="FD1" t="s">
         <v>132</v>
       </c>
-      <c r="EM1" t="s">
+      <c r="FE1" t="s">
         <v>133</v>
       </c>
-      <c r="EN1" t="s">
+      <c r="FF1" t="s">
         <v>134</v>
       </c>
-      <c r="EO1" t="s">
+      <c r="FG1" t="s">
         <v>135</v>
       </c>
-      <c r="EP1" t="s">
+      <c r="FH1" t="s">
         <v>136</v>
       </c>
-      <c r="EQ1" t="s">
+      <c r="FI1" t="s">
         <v>137</v>
       </c>
-      <c r="ER1" t="s">
+      <c r="FJ1" t="s">
         <v>138</v>
       </c>
-      <c r="ES1" t="s">
+      <c r="FK1" t="s">
         <v>139</v>
       </c>
-      <c r="ET1" t="s">
+      <c r="FL1" s="3" t="s">
+        <v>291</v>
+      </c>
+      <c r="FM1" t="s">
         <v>140</v>
       </c>
-      <c r="EU1" t="s">
+      <c r="FN1" t="s">
         <v>141</v>
       </c>
-      <c r="EV1" t="s">
+      <c r="FO1" s="3" t="s">
+        <v>292</v>
+      </c>
+      <c r="FP1" t="s">
         <v>142</v>
       </c>
-      <c r="EW1" t="s">
+      <c r="FQ1" t="s">
         <v>143</v>
       </c>
-      <c r="EX1" t="s">
+      <c r="FR1" s="3" t="s">
+        <v>293</v>
+      </c>
+      <c r="FS1" t="s">
         <v>144</v>
       </c>
-      <c r="EY1" t="s">
+      <c r="FT1" t="s">
         <v>145</v>
       </c>
-      <c r="EZ1" t="s">
+      <c r="FU1" t="s">
         <v>146</v>
       </c>
-      <c r="FA1" t="s">
+      <c r="FV1" t="s">
         <v>147</v>
       </c>
-      <c r="FB1" t="s">
+      <c r="FW1" t="s">
         <v>148</v>
       </c>
-      <c r="FC1" t="s">
+      <c r="FX1" t="s">
         <v>149</v>
       </c>
-      <c r="FD1" t="s">
+      <c r="FY1" s="3" t="s">
+        <v>294</v>
+      </c>
+      <c r="FZ1" t="s">
         <v>150</v>
       </c>
-      <c r="FE1" t="s">
+      <c r="GA1" s="3" t="s">
+        <v>295</v>
+      </c>
+      <c r="GB1" t="s">
         <v>151</v>
       </c>
-      <c r="FF1" t="s">
+      <c r="GC1" t="s">
         <v>152</v>
       </c>
-      <c r="FG1" t="s">
+      <c r="GD1" t="s">
         <v>153</v>
       </c>
-      <c r="FH1" t="s">
+      <c r="GE1" t="s">
         <v>154</v>
       </c>
-      <c r="FI1" t="s">
+      <c r="GF1" s="3" t="s">
+        <v>296</v>
+      </c>
+      <c r="GG1" t="s">
         <v>155</v>
       </c>
-      <c r="FJ1" t="s">
+      <c r="GH1" t="s">
         <v>156</v>
       </c>
-      <c r="FK1" t="s">
+      <c r="GI1" s="3" t="s">
+        <v>297</v>
+      </c>
+      <c r="GJ1" t="s">
         <v>157</v>
       </c>
-      <c r="FL1" t="s">
+      <c r="GK1" t="s">
         <v>158</v>
       </c>
-      <c r="FM1" t="s">
+      <c r="GL1" t="s">
         <v>159</v>
       </c>
-      <c r="FN1" t="s">
+      <c r="GM1" s="3" t="s">
+        <v>298</v>
+      </c>
+      <c r="GN1" t="s">
         <v>160</v>
       </c>
-      <c r="FO1" t="s">
+      <c r="GO1" t="s">
         <v>161</v>
       </c>
-      <c r="FP1" t="s">
+      <c r="GP1" t="s">
         <v>162</v>
       </c>
-      <c r="FQ1" t="s">
+      <c r="GQ1" t="s">
         <v>163</v>
       </c>
-      <c r="FR1" t="s">
+      <c r="GR1" s="3" t="s">
+        <v>299</v>
+      </c>
+      <c r="GS1" t="s">
         <v>164</v>
       </c>
-      <c r="FS1" t="s">
+      <c r="GT1" t="s">
         <v>165</v>
       </c>
-      <c r="FT1" t="s">
+      <c r="GU1" s="3" t="s">
+        <v>300</v>
+      </c>
+      <c r="GV1" t="s">
         <v>166</v>
       </c>
-      <c r="FU1" t="s">
+      <c r="GW1" t="s">
         <v>167</v>
       </c>
-      <c r="FV1" t="s">
+      <c r="GX1" s="3" t="s">
+        <v>266</v>
+      </c>
+      <c r="GY1" t="s">
         <v>168</v>
       </c>
-      <c r="FW1" t="s">
+      <c r="GZ1" t="s">
         <v>169</v>
       </c>
-      <c r="FX1" t="s">
+      <c r="HA1" t="s">
         <v>170</v>
       </c>
-      <c r="FY1" t="s">
+      <c r="HB1" s="3" t="s">
+        <v>270</v>
+      </c>
+      <c r="HC1" t="s">
         <v>171</v>
       </c>
-      <c r="FZ1" t="s">
+      <c r="HD1" t="s">
         <v>172</v>
       </c>
-      <c r="GA1" t="s">
+      <c r="HE1" t="s">
         <v>173</v>
       </c>
-      <c r="GB1" t="s">
+      <c r="HF1" t="s">
         <v>174</v>
       </c>
-      <c r="GC1" t="s">
+      <c r="HG1" t="s">
         <v>175</v>
       </c>
-      <c r="GD1" t="s">
+      <c r="HH1" t="s">
         <v>176</v>
       </c>
-      <c r="GE1" t="s">
+      <c r="HI1" t="s">
         <v>177</v>
       </c>
-      <c r="GF1" t="s">
+      <c r="HJ1" t="s">
         <v>178</v>
       </c>
-      <c r="GG1" t="s">
+      <c r="HK1" t="s">
         <v>179</v>
       </c>
-      <c r="GH1" t="s">
+    </row>
+    <row r="2" spans="1:219" x14ac:dyDescent="0.2">
+      <c r="A2" s="1" t="s">
         <v>180</v>
       </c>
-    </row>
-    <row r="2" spans="1:190" x14ac:dyDescent="0.2">
-      <c r="A2" s="1" t="s">
+      <c r="B2" s="1" t="s">
         <v>181</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="C2" t="s">
         <v>182</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" s="2" t="s">
+        <v>185</v>
+      </c>
+      <c r="E2" t="s">
         <v>183</v>
       </c>
-      <c r="D2" s="2" t="s">
-        <v>186</v>
-      </c>
-      <c r="E2" t="s">
+      <c r="F2" t="s">
         <v>184</v>
       </c>
-      <c r="F2" t="s">
-        <v>185</v>
-      </c>
       <c r="G2" s="2" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="H2" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="I2" t="s">
+        <v>186</v>
+      </c>
+      <c r="J2" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="K2" t="s">
         <v>187</v>
       </c>
-      <c r="J2" s="3" t="s">
-        <v>186</v>
-      </c>
-      <c r="K2" t="s">
+      <c r="L2" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="M2" t="s">
+        <v>186</v>
+      </c>
+      <c r="N2" t="s">
+        <v>186</v>
+      </c>
+      <c r="O2" t="s">
+        <v>186</v>
+      </c>
+      <c r="P2" t="s">
+        <v>186</v>
+      </c>
+      <c r="Q2" t="s">
+        <v>186</v>
+      </c>
+      <c r="R2" t="s">
+        <v>186</v>
+      </c>
+      <c r="S2" t="s">
+        <v>186</v>
+      </c>
+      <c r="T2" t="s">
+        <v>186</v>
+      </c>
+      <c r="U2" t="s">
+        <v>186</v>
+      </c>
+      <c r="V2" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="W2" t="s">
         <v>188</v>
       </c>
-      <c r="L2" s="3" t="s">
-        <v>186</v>
-      </c>
-      <c r="M2" t="s">
-        <v>187</v>
-      </c>
-      <c r="N2" t="s">
-        <v>187</v>
-      </c>
-      <c r="O2" t="s">
-        <v>187</v>
-      </c>
-      <c r="P2" t="s">
-        <v>187</v>
-      </c>
-      <c r="Q2" t="s">
-        <v>187</v>
-      </c>
-      <c r="R2" t="s">
-        <v>187</v>
-      </c>
-      <c r="S2" t="s">
-        <v>187</v>
-      </c>
-      <c r="T2" t="s">
-        <v>187</v>
-      </c>
-      <c r="U2" t="s">
-        <v>187</v>
-      </c>
-      <c r="V2" s="3" t="s">
-        <v>186</v>
-      </c>
-      <c r="W2" t="s">
+      <c r="X2" t="s">
+        <v>188</v>
+      </c>
+      <c r="Y2" t="s">
+        <v>188</v>
+      </c>
+      <c r="Z2" t="s">
+        <v>188</v>
+      </c>
+      <c r="AA2" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="AB2" t="s">
+        <v>185</v>
+      </c>
+      <c r="AC2" t="s">
+        <v>186</v>
+      </c>
+      <c r="AD2" t="s">
+        <v>186</v>
+      </c>
+      <c r="AE2" t="s">
+        <v>186</v>
+      </c>
+      <c r="AF2" t="s">
+        <v>186</v>
+      </c>
+      <c r="AG2" t="s">
+        <v>186</v>
+      </c>
+      <c r="AH2" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="AI2" t="s">
+        <v>185</v>
+      </c>
+      <c r="AJ2" t="s">
         <v>189</v>
-      </c>
-      <c r="X2" t="s">
-        <v>189</v>
-      </c>
-      <c r="Y2" t="s">
-        <v>189</v>
-      </c>
-      <c r="Z2" t="s">
-        <v>189</v>
-      </c>
-      <c r="AA2" s="3" t="s">
-        <v>186</v>
-      </c>
-      <c r="AB2" t="s">
-        <v>186</v>
-      </c>
-      <c r="AC2" t="s">
-        <v>187</v>
-      </c>
-      <c r="AD2" t="s">
-        <v>187</v>
-      </c>
-      <c r="AE2" t="s">
-        <v>187</v>
-      </c>
-      <c r="AF2" t="s">
-        <v>187</v>
-      </c>
-      <c r="AG2" t="s">
-        <v>187</v>
-      </c>
-      <c r="AH2" s="3" t="s">
-        <v>186</v>
-      </c>
-      <c r="AI2" t="s">
-        <v>186</v>
-      </c>
-      <c r="AJ2" t="s">
-        <v>190</v>
       </c>
       <c r="AK2">
         <v>3</v>
@@ -2621,22 +2821,22 @@
         <v>15</v>
       </c>
       <c r="AM2" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="AN2">
         <v>3</v>
       </c>
       <c r="AO2" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="AP2" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="AQ2" s="3" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="AR2" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="AS2">
         <v>5</v>
@@ -2645,7 +2845,7 @@
         <v>60</v>
       </c>
       <c r="AU2" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="AV2">
         <v>6</v>
@@ -2654,7 +2854,7 @@
         <v>30</v>
       </c>
       <c r="AX2" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="AY2">
         <v>3</v>
@@ -2663,7 +2863,7 @@
         <v>120</v>
       </c>
       <c r="BA2" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="BB2">
         <v>2</v>
@@ -2672,7 +2872,7 @@
         <v>100</v>
       </c>
       <c r="BD2" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="BE2">
         <v>1</v>
@@ -2681,7 +2881,7 @@
         <v>20</v>
       </c>
       <c r="BG2" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="BH2">
         <v>1</v>
@@ -2689,499 +2889,589 @@
       <c r="BI2">
         <v>20</v>
       </c>
+      <c r="BJ2" s="3" t="s">
+        <v>185</v>
+      </c>
       <c r="BK2" t="s">
+        <v>191</v>
+      </c>
+      <c r="BL2" t="s">
         <v>192</v>
       </c>
-      <c r="BL2" t="s">
+      <c r="BM2" t="s">
         <v>193</v>
       </c>
-      <c r="BM2" t="s">
+      <c r="BN2" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="BO2" t="s">
+        <v>185</v>
+      </c>
+      <c r="BP2" t="s">
         <v>194</v>
       </c>
-      <c r="BN2" t="s">
+      <c r="BQ2" t="s">
         <v>195</v>
-      </c>
-      <c r="BO2" t="s">
-        <v>186</v>
-      </c>
-      <c r="BP2" t="s">
-        <v>196</v>
-      </c>
-      <c r="BQ2" t="s">
-        <v>197</v>
       </c>
       <c r="BR2">
         <v>100</v>
       </c>
       <c r="BS2" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="BT2">
         <v>90</v>
       </c>
-      <c r="BU2" t="s">
+      <c r="BU2" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="BV2" t="s">
+        <v>186</v>
+      </c>
+      <c r="BW2" t="s">
+        <v>194</v>
+      </c>
+      <c r="BX2" t="s">
+        <v>196</v>
+      </c>
+      <c r="BY2" t="s">
+        <v>191</v>
+      </c>
+      <c r="BZ2">
+        <v>110</v>
+      </c>
+      <c r="CA2">
+        <v>80</v>
+      </c>
+      <c r="CB2" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="CC2" t="s">
+        <v>185</v>
+      </c>
+      <c r="CD2" t="s">
+        <v>197</v>
+      </c>
+      <c r="CE2" t="s">
+        <v>185</v>
+      </c>
+      <c r="CF2" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="CG2" t="s">
+        <v>185</v>
+      </c>
+      <c r="CH2" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="CI2" t="s">
+        <v>185</v>
+      </c>
+      <c r="CJ2" t="s">
+        <v>185</v>
+      </c>
+      <c r="CK2" t="s">
+        <v>185</v>
+      </c>
+      <c r="CL2" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="CM2" t="s">
+        <v>185</v>
+      </c>
+      <c r="CN2" t="s">
+        <v>185</v>
+      </c>
+      <c r="CO2" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="CP2" t="s">
+        <v>198</v>
+      </c>
+      <c r="CQ2" t="s">
+        <v>199</v>
+      </c>
+      <c r="CR2" t="s">
+        <v>200</v>
+      </c>
+      <c r="CS2" t="s">
+        <v>200</v>
+      </c>
+      <c r="CT2" t="s">
+        <v>200</v>
+      </c>
+      <c r="CU2" t="s">
+        <v>200</v>
+      </c>
+      <c r="CV2" t="s">
+        <v>201</v>
+      </c>
+      <c r="CW2" t="s">
+        <v>202</v>
+      </c>
+      <c r="CX2" t="s">
+        <v>203</v>
+      </c>
+      <c r="CY2" t="s">
+        <v>200</v>
+      </c>
+      <c r="CZ2" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="DA2" t="s">
+        <v>204</v>
+      </c>
+      <c r="DB2" t="s">
+        <v>205</v>
+      </c>
+      <c r="DC2" t="s">
+        <v>206</v>
+      </c>
+      <c r="DD2" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="DE2" t="s">
+        <v>207</v>
+      </c>
+      <c r="DF2" t="s">
+        <v>208</v>
+      </c>
+      <c r="DG2" t="s">
+        <v>208</v>
+      </c>
+      <c r="DH2" t="s">
+        <v>208</v>
+      </c>
+      <c r="DI2" t="s">
+        <v>208</v>
+      </c>
+      <c r="DJ2" t="s">
+        <v>208</v>
+      </c>
+      <c r="DK2" t="s">
+        <v>208</v>
+      </c>
+      <c r="DL2" t="s">
+        <v>208</v>
+      </c>
+      <c r="DM2" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="DN2" t="s">
+        <v>209</v>
+      </c>
+      <c r="DO2" t="s">
+        <v>209</v>
+      </c>
+      <c r="DP2" t="s">
+        <v>209</v>
+      </c>
+      <c r="DQ2" t="s">
+        <v>210</v>
+      </c>
+      <c r="DR2" t="s">
+        <v>211</v>
+      </c>
+      <c r="DS2" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="DT2" t="s">
+        <v>212</v>
+      </c>
+      <c r="DU2" t="s">
+        <v>213</v>
+      </c>
+      <c r="DV2" t="s">
+        <v>214</v>
+      </c>
+      <c r="DW2" t="s">
+        <v>185</v>
+      </c>
+      <c r="DX2" t="s">
+        <v>215</v>
+      </c>
+      <c r="DY2" t="s">
+        <v>216</v>
+      </c>
+      <c r="DZ2" t="s">
+        <v>217</v>
+      </c>
+      <c r="EA2" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="EB2" t="s">
+        <v>185</v>
+      </c>
+      <c r="EC2" t="s">
+        <v>185</v>
+      </c>
+      <c r="ED2" t="s">
+        <v>185</v>
+      </c>
+      <c r="EE2" t="s">
+        <v>185</v>
+      </c>
+      <c r="EF2" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="EG2" t="s">
         <v>187</v>
       </c>
-      <c r="BV2" t="s">
-        <v>196</v>
-      </c>
-      <c r="BW2" t="s">
-        <v>198</v>
-      </c>
-      <c r="BX2" t="s">
-        <v>192</v>
-      </c>
-      <c r="BY2">
-        <v>110</v>
-      </c>
-      <c r="BZ2">
-        <v>80</v>
-      </c>
-      <c r="CA2" t="s">
-        <v>186</v>
-      </c>
-      <c r="CB2" t="s">
-        <v>199</v>
-      </c>
-      <c r="CC2" t="s">
-        <v>186</v>
-      </c>
-      <c r="CD2" t="s">
-        <v>186</v>
-      </c>
-      <c r="CE2" t="s">
-        <v>186</v>
-      </c>
-      <c r="CF2" t="s">
-        <v>186</v>
-      </c>
-      <c r="CG2" t="s">
-        <v>186</v>
-      </c>
-      <c r="CH2" t="s">
-        <v>186</v>
-      </c>
-      <c r="CI2" t="s">
-        <v>186</v>
-      </c>
-      <c r="CJ2" t="s">
-        <v>200</v>
-      </c>
-      <c r="CK2" t="s">
-        <v>201</v>
-      </c>
-      <c r="CL2" t="s">
-        <v>202</v>
-      </c>
-      <c r="CM2" t="s">
-        <v>202</v>
-      </c>
-      <c r="CN2" t="s">
-        <v>202</v>
-      </c>
-      <c r="CO2" t="s">
-        <v>202</v>
-      </c>
-      <c r="CP2" t="s">
-        <v>203</v>
-      </c>
-      <c r="CQ2" t="s">
-        <v>204</v>
-      </c>
-      <c r="CR2" t="s">
-        <v>205</v>
-      </c>
-      <c r="CS2" t="s">
-        <v>202</v>
-      </c>
-      <c r="CT2" t="s">
-        <v>206</v>
-      </c>
-      <c r="CU2" t="s">
-        <v>207</v>
-      </c>
-      <c r="CV2" t="s">
-        <v>208</v>
-      </c>
-      <c r="CW2" t="s">
-        <v>209</v>
-      </c>
-      <c r="CX2" t="s">
-        <v>210</v>
-      </c>
-      <c r="CY2" t="s">
-        <v>210</v>
-      </c>
-      <c r="CZ2" t="s">
-        <v>210</v>
-      </c>
-      <c r="DA2" t="s">
-        <v>210</v>
-      </c>
-      <c r="DB2" t="s">
-        <v>210</v>
-      </c>
-      <c r="DC2" t="s">
-        <v>210</v>
-      </c>
-      <c r="DD2" t="s">
-        <v>210</v>
-      </c>
-      <c r="DE2" t="s">
-        <v>211</v>
-      </c>
-      <c r="DF2" t="s">
-        <v>211</v>
-      </c>
-      <c r="DG2" t="s">
-        <v>211</v>
-      </c>
-      <c r="DH2" t="s">
-        <v>212</v>
-      </c>
-      <c r="DI2" t="s">
-        <v>213</v>
-      </c>
-      <c r="DJ2" t="s">
-        <v>214</v>
-      </c>
-      <c r="DK2" t="s">
-        <v>215</v>
-      </c>
-      <c r="DL2" t="s">
-        <v>216</v>
-      </c>
-      <c r="DM2" t="s">
-        <v>186</v>
-      </c>
-      <c r="DN2" t="s">
-        <v>217</v>
-      </c>
-      <c r="DO2" t="s">
+      <c r="EH2" t="s">
+        <v>186</v>
+      </c>
+      <c r="EI2" t="s">
+        <v>186</v>
+      </c>
+      <c r="EJ2" t="s">
+        <v>186</v>
+      </c>
+      <c r="EK2" t="s">
+        <v>186</v>
+      </c>
+      <c r="EL2" t="s">
+        <v>186</v>
+      </c>
+      <c r="EM2" t="s">
         <v>218</v>
       </c>
-      <c r="DP2" t="s">
+      <c r="EN2" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="EO2" t="s">
         <v>219</v>
       </c>
-      <c r="DQ2" t="s">
-        <v>186</v>
-      </c>
-      <c r="DR2" t="s">
-        <v>186</v>
-      </c>
-      <c r="DS2" t="s">
-        <v>186</v>
-      </c>
-      <c r="DT2" t="s">
-        <v>186</v>
-      </c>
-      <c r="DU2" t="s">
+      <c r="EP2" t="s">
+        <v>220</v>
+      </c>
+      <c r="EQ2" t="s">
+        <v>221</v>
+      </c>
+      <c r="ER2" t="s">
+        <v>222</v>
+      </c>
+      <c r="ES2" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="ET2" t="s">
+        <v>223</v>
+      </c>
+      <c r="EU2" t="s">
+        <v>224</v>
+      </c>
+      <c r="EV2" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="EW2" t="s">
+        <v>225</v>
+      </c>
+      <c r="EX2" t="s">
+        <v>226</v>
+      </c>
+      <c r="EY2" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="EZ2" t="s">
+        <v>225</v>
+      </c>
+      <c r="FA2" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="FB2" t="s">
+        <v>227</v>
+      </c>
+      <c r="FC2" t="s">
+        <v>228</v>
+      </c>
+      <c r="FD2" t="s">
+        <v>229</v>
+      </c>
+      <c r="FE2" t="s">
+        <v>230</v>
+      </c>
+      <c r="FF2" t="s">
+        <v>231</v>
+      </c>
+      <c r="FG2" t="s">
+        <v>232</v>
+      </c>
+      <c r="FH2" t="s">
+        <v>233</v>
+      </c>
+      <c r="FI2" t="s">
+        <v>234</v>
+      </c>
+      <c r="FJ2" t="s">
+        <v>218</v>
+      </c>
+      <c r="FK2" t="s">
+        <v>235</v>
+      </c>
+      <c r="FL2" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="FM2" t="s">
+        <v>185</v>
+      </c>
+      <c r="FN2" t="s">
+        <v>186</v>
+      </c>
+      <c r="FO2" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="FP2" t="s">
+        <v>186</v>
+      </c>
+      <c r="FQ2" t="s">
+        <v>186</v>
+      </c>
+      <c r="FR2" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="FS2" t="s">
+        <v>186</v>
+      </c>
+      <c r="FT2" t="s">
+        <v>236</v>
+      </c>
+      <c r="FU2" t="s">
+        <v>186</v>
+      </c>
+      <c r="FV2" t="s">
+        <v>186</v>
+      </c>
+      <c r="FW2" t="s">
+        <v>186</v>
+      </c>
+      <c r="FX2" t="s">
+        <v>186</v>
+      </c>
+      <c r="FY2" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="FZ2" t="s">
+        <v>193</v>
+      </c>
+      <c r="GA2" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="GB2" t="s">
+        <v>237</v>
+      </c>
+      <c r="GC2" t="s">
+        <v>237</v>
+      </c>
+      <c r="GD2" t="s">
+        <v>238</v>
+      </c>
+      <c r="GE2" t="s">
+        <v>239</v>
+      </c>
+      <c r="GF2" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="GG2" t="s">
+        <v>240</v>
+      </c>
+      <c r="GH2" t="s">
+        <v>241</v>
+      </c>
+      <c r="GI2" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="GJ2" t="s">
+        <v>242</v>
+      </c>
+      <c r="GK2" t="s">
+        <v>243</v>
+      </c>
+      <c r="GL2" t="s">
+        <v>244</v>
+      </c>
+      <c r="GM2" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="GN2">
+        <v>0.5</v>
+      </c>
+      <c r="GO2">
+        <v>49</v>
+      </c>
+      <c r="GP2">
+        <v>60</v>
+      </c>
+      <c r="GQ2">
+        <v>10</v>
+      </c>
+      <c r="GR2" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="GS2" t="s">
+        <v>245</v>
+      </c>
+      <c r="GT2" t="s">
+        <v>246</v>
+      </c>
+      <c r="GU2" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="GV2" t="s">
+        <v>218</v>
+      </c>
+      <c r="GW2" t="s">
+        <v>218</v>
+      </c>
+      <c r="GX2" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="GY2" t="s">
+        <v>247</v>
+      </c>
+      <c r="GZ2" t="s">
+        <v>248</v>
+      </c>
+      <c r="HA2" t="s">
+        <v>249</v>
+      </c>
+      <c r="HB2" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="HC2" t="s">
+        <v>250</v>
+      </c>
+      <c r="HD2" t="s">
+        <v>251</v>
+      </c>
+      <c r="HE2" t="s">
+        <v>252</v>
+      </c>
+      <c r="HF2" t="s">
+        <v>253</v>
+      </c>
+      <c r="HG2" t="s">
+        <v>254</v>
+      </c>
+      <c r="HH2" t="s">
+        <v>255</v>
+      </c>
+      <c r="HI2" t="s">
+        <v>256</v>
+      </c>
+      <c r="HJ2" t="s">
+        <v>218</v>
+      </c>
+      <c r="HK2" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="3" spans="1:219" x14ac:dyDescent="0.2">
+      <c r="A3" s="1" t="s">
+        <v>258</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>258</v>
+      </c>
+      <c r="C3" t="s">
+        <v>259</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>185</v>
+      </c>
+      <c r="E3" t="s">
+        <v>260</v>
+      </c>
+      <c r="F3" t="s">
+        <v>184</v>
+      </c>
+      <c r="G3" s="2" t="s">
+        <v>185</v>
+      </c>
+      <c r="H3" t="s">
+        <v>185</v>
+      </c>
+      <c r="I3" t="s">
+        <v>186</v>
+      </c>
+      <c r="J3" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="K3" t="s">
+        <v>187</v>
+      </c>
+      <c r="L3" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="M3" t="s">
+        <v>186</v>
+      </c>
+      <c r="N3" t="s">
+        <v>186</v>
+      </c>
+      <c r="O3" t="s">
+        <v>186</v>
+      </c>
+      <c r="P3" t="s">
+        <v>186</v>
+      </c>
+      <c r="Q3" t="s">
+        <v>186</v>
+      </c>
+      <c r="R3" t="s">
+        <v>186</v>
+      </c>
+      <c r="S3" t="s">
+        <v>186</v>
+      </c>
+      <c r="T3" t="s">
+        <v>186</v>
+      </c>
+      <c r="U3" t="s">
+        <v>186</v>
+      </c>
+      <c r="V3" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="W3" t="s">
         <v>188</v>
       </c>
-      <c r="DV2" t="s">
-        <v>187</v>
-      </c>
-      <c r="DW2" t="s">
-        <v>187</v>
-      </c>
-      <c r="DX2" t="s">
-        <v>187</v>
-      </c>
-      <c r="DY2" t="s">
-        <v>187</v>
-      </c>
-      <c r="DZ2" t="s">
-        <v>187</v>
-      </c>
-      <c r="EA2" t="s">
-        <v>220</v>
-      </c>
-      <c r="EB2" t="s">
-        <v>221</v>
-      </c>
-      <c r="EC2" t="s">
-        <v>222</v>
-      </c>
-      <c r="ED2" t="s">
-        <v>223</v>
-      </c>
-      <c r="EE2" t="s">
-        <v>224</v>
-      </c>
-      <c r="EF2" t="s">
-        <v>225</v>
-      </c>
-      <c r="EG2" t="s">
-        <v>226</v>
-      </c>
-      <c r="EH2" t="s">
-        <v>227</v>
-      </c>
-      <c r="EI2" t="s">
-        <v>228</v>
-      </c>
-      <c r="EJ2" t="s">
-        <v>227</v>
-      </c>
-      <c r="EK2" t="s">
-        <v>229</v>
-      </c>
-      <c r="EL2" t="s">
-        <v>230</v>
-      </c>
-      <c r="EM2" t="s">
-        <v>231</v>
-      </c>
-      <c r="EN2" t="s">
-        <v>232</v>
-      </c>
-      <c r="EO2" t="s">
-        <v>233</v>
-      </c>
-      <c r="EP2" t="s">
-        <v>234</v>
-      </c>
-      <c r="EQ2" t="s">
-        <v>235</v>
-      </c>
-      <c r="ER2" t="s">
-        <v>236</v>
-      </c>
-      <c r="ES2" t="s">
-        <v>220</v>
-      </c>
-      <c r="ET2" t="s">
-        <v>237</v>
-      </c>
-      <c r="EU2" t="s">
-        <v>186</v>
-      </c>
-      <c r="EV2" t="s">
-        <v>187</v>
-      </c>
-      <c r="EW2" t="s">
-        <v>187</v>
-      </c>
-      <c r="EX2" t="s">
-        <v>187</v>
-      </c>
-      <c r="EY2" t="s">
-        <v>187</v>
-      </c>
-      <c r="EZ2" t="s">
-        <v>238</v>
-      </c>
-      <c r="FA2" t="s">
-        <v>187</v>
-      </c>
-      <c r="FB2" t="s">
-        <v>187</v>
-      </c>
-      <c r="FC2" t="s">
-        <v>187</v>
-      </c>
-      <c r="FD2" t="s">
-        <v>187</v>
-      </c>
-      <c r="FE2" t="s">
-        <v>194</v>
-      </c>
-      <c r="FF2" t="s">
-        <v>239</v>
-      </c>
-      <c r="FG2" t="s">
-        <v>239</v>
-      </c>
-      <c r="FH2" t="s">
-        <v>240</v>
-      </c>
-      <c r="FI2" t="s">
-        <v>241</v>
-      </c>
-      <c r="FJ2" t="s">
-        <v>242</v>
-      </c>
-      <c r="FK2" t="s">
-        <v>243</v>
-      </c>
-      <c r="FL2" t="s">
-        <v>244</v>
-      </c>
-      <c r="FM2" t="s">
-        <v>245</v>
-      </c>
-      <c r="FN2" t="s">
-        <v>246</v>
-      </c>
-      <c r="FO2">
-        <v>0.5</v>
-      </c>
-      <c r="FP2">
-        <v>49</v>
-      </c>
-      <c r="FQ2">
-        <v>60</v>
-      </c>
-      <c r="FR2">
-        <v>10</v>
-      </c>
-      <c r="FS2" t="s">
-        <v>247</v>
-      </c>
-      <c r="FT2" t="s">
-        <v>248</v>
-      </c>
-      <c r="FU2" t="s">
-        <v>220</v>
-      </c>
-      <c r="FV2" t="s">
-        <v>220</v>
-      </c>
-      <c r="FW2" t="s">
-        <v>249</v>
-      </c>
-      <c r="FX2" t="s">
-        <v>250</v>
-      </c>
-      <c r="FY2" t="s">
-        <v>251</v>
-      </c>
-      <c r="FZ2" t="s">
-        <v>252</v>
-      </c>
-      <c r="GA2" t="s">
-        <v>253</v>
-      </c>
-      <c r="GB2" t="s">
-        <v>254</v>
-      </c>
-      <c r="GC2" t="s">
-        <v>255</v>
-      </c>
-      <c r="GD2" t="s">
-        <v>256</v>
-      </c>
-      <c r="GE2" t="s">
-        <v>257</v>
-      </c>
-      <c r="GF2" t="s">
-        <v>258</v>
-      </c>
-      <c r="GG2" t="s">
-        <v>220</v>
-      </c>
-      <c r="GH2" t="s">
-        <v>259</v>
-      </c>
-    </row>
-    <row r="3" spans="1:190" x14ac:dyDescent="0.2">
-      <c r="A3" s="1" t="s">
-        <v>260</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>260</v>
-      </c>
-      <c r="C3" t="s">
-        <v>261</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>186</v>
-      </c>
-      <c r="E3" t="s">
-        <v>262</v>
-      </c>
-      <c r="F3" t="s">
-        <v>185</v>
-      </c>
-      <c r="G3" s="2" t="s">
-        <v>186</v>
-      </c>
-      <c r="H3" t="s">
-        <v>186</v>
-      </c>
-      <c r="I3" t="s">
-        <v>187</v>
-      </c>
-      <c r="J3" s="3" t="s">
-        <v>186</v>
-      </c>
-      <c r="K3" t="s">
+      <c r="X3" t="s">
         <v>188</v>
       </c>
-      <c r="L3" s="3" t="s">
-        <v>186</v>
-      </c>
-      <c r="M3" t="s">
-        <v>187</v>
-      </c>
-      <c r="N3" t="s">
-        <v>187</v>
-      </c>
-      <c r="O3" t="s">
-        <v>187</v>
-      </c>
-      <c r="P3" t="s">
-        <v>187</v>
-      </c>
-      <c r="Q3" t="s">
-        <v>187</v>
-      </c>
-      <c r="R3" t="s">
-        <v>187</v>
-      </c>
-      <c r="S3" t="s">
-        <v>187</v>
-      </c>
-      <c r="T3" t="s">
-        <v>187</v>
-      </c>
-      <c r="U3" t="s">
-        <v>187</v>
-      </c>
-      <c r="V3" s="3" t="s">
-        <v>186</v>
-      </c>
-      <c r="W3" t="s">
+      <c r="Y3" t="s">
+        <v>188</v>
+      </c>
+      <c r="Z3" t="s">
+        <v>188</v>
+      </c>
+      <c r="AA3" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="AB3" t="s">
+        <v>186</v>
+      </c>
+      <c r="AC3" t="s">
+        <v>186</v>
+      </c>
+      <c r="AD3" t="s">
+        <v>186</v>
+      </c>
+      <c r="AE3" t="s">
+        <v>186</v>
+      </c>
+      <c r="AF3" t="s">
+        <v>186</v>
+      </c>
+      <c r="AG3" t="s">
+        <v>186</v>
+      </c>
+      <c r="AH3" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="AI3" t="s">
+        <v>186</v>
+      </c>
+      <c r="AJ3" t="s">
         <v>189</v>
-      </c>
-      <c r="X3" t="s">
-        <v>189</v>
-      </c>
-      <c r="Y3" t="s">
-        <v>189</v>
-      </c>
-      <c r="Z3" t="s">
-        <v>189</v>
-      </c>
-      <c r="AA3" s="3" t="s">
-        <v>186</v>
-      </c>
-      <c r="AB3" t="s">
-        <v>187</v>
-      </c>
-      <c r="AC3" t="s">
-        <v>187</v>
-      </c>
-      <c r="AD3" t="s">
-        <v>187</v>
-      </c>
-      <c r="AE3" t="s">
-        <v>187</v>
-      </c>
-      <c r="AF3" t="s">
-        <v>187</v>
-      </c>
-      <c r="AG3" t="s">
-        <v>187</v>
-      </c>
-      <c r="AH3" s="3" t="s">
-        <v>186</v>
-      </c>
-      <c r="AI3" t="s">
-        <v>187</v>
-      </c>
-      <c r="AJ3" t="s">
-        <v>190</v>
       </c>
       <c r="AK3">
         <v>3</v>
@@ -3190,22 +3480,22 @@
         <v>15</v>
       </c>
       <c r="AM3" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="AN3">
         <v>3</v>
       </c>
       <c r="AO3" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="AP3" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="AQ3" s="3" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="AR3" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="AS3">
         <v>5</v>
@@ -3214,7 +3504,7 @@
         <v>60</v>
       </c>
       <c r="AU3" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="AV3">
         <v>6</v>
@@ -3223,7 +3513,7 @@
         <v>30</v>
       </c>
       <c r="AX3" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="AY3">
         <v>3</v>
@@ -3232,7 +3522,7 @@
         <v>120</v>
       </c>
       <c r="BA3" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="BB3">
         <v>2</v>
@@ -3241,7 +3531,7 @@
         <v>100</v>
       </c>
       <c r="BD3" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="BE3">
         <v>1</v>
@@ -3250,7 +3540,7 @@
         <v>20</v>
       </c>
       <c r="BG3" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="BH3">
         <v>1</v>
@@ -3258,499 +3548,589 @@
       <c r="BI3">
         <v>20</v>
       </c>
+      <c r="BJ3" s="3" t="s">
+        <v>185</v>
+      </c>
       <c r="BK3" t="s">
+        <v>191</v>
+      </c>
+      <c r="BL3" t="s">
         <v>192</v>
       </c>
-      <c r="BL3" t="s">
+      <c r="BM3" t="s">
         <v>193</v>
       </c>
-      <c r="BM3" t="s">
+      <c r="BN3" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="BO3" t="s">
+        <v>186</v>
+      </c>
+      <c r="BP3" t="s">
         <v>194</v>
       </c>
-      <c r="BN3" t="s">
+      <c r="BQ3" t="s">
         <v>195</v>
-      </c>
-      <c r="BO3" t="s">
-        <v>187</v>
-      </c>
-      <c r="BP3" t="s">
-        <v>196</v>
-      </c>
-      <c r="BQ3" t="s">
-        <v>197</v>
       </c>
       <c r="BR3">
         <v>100</v>
       </c>
       <c r="BS3" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="BT3">
         <v>90</v>
       </c>
-      <c r="BU3" t="s">
+      <c r="BU3" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="BV3" t="s">
+        <v>186</v>
+      </c>
+      <c r="BW3" t="s">
+        <v>194</v>
+      </c>
+      <c r="BX3" t="s">
+        <v>196</v>
+      </c>
+      <c r="BY3" t="s">
+        <v>191</v>
+      </c>
+      <c r="BZ3">
+        <v>110</v>
+      </c>
+      <c r="CA3">
+        <v>80</v>
+      </c>
+      <c r="CB3" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="CC3" t="s">
+        <v>185</v>
+      </c>
+      <c r="CD3" t="s">
+        <v>197</v>
+      </c>
+      <c r="CE3" t="s">
+        <v>185</v>
+      </c>
+      <c r="CF3" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="CG3" t="s">
+        <v>185</v>
+      </c>
+      <c r="CH3" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="CI3" t="s">
+        <v>185</v>
+      </c>
+      <c r="CJ3" t="s">
+        <v>185</v>
+      </c>
+      <c r="CK3" t="s">
+        <v>185</v>
+      </c>
+      <c r="CL3" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="CM3" t="s">
+        <v>185</v>
+      </c>
+      <c r="CN3" t="s">
+        <v>185</v>
+      </c>
+      <c r="CO3" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="CP3" t="s">
+        <v>198</v>
+      </c>
+      <c r="CQ3" t="s">
+        <v>199</v>
+      </c>
+      <c r="CR3" t="s">
+        <v>200</v>
+      </c>
+      <c r="CS3" t="s">
+        <v>200</v>
+      </c>
+      <c r="CT3" t="s">
+        <v>200</v>
+      </c>
+      <c r="CU3" t="s">
+        <v>200</v>
+      </c>
+      <c r="CV3" t="s">
+        <v>201</v>
+      </c>
+      <c r="CW3" t="s">
+        <v>202</v>
+      </c>
+      <c r="CX3" t="s">
+        <v>203</v>
+      </c>
+      <c r="CY3" t="s">
+        <v>200</v>
+      </c>
+      <c r="CZ3" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="DA3" t="s">
+        <v>204</v>
+      </c>
+      <c r="DB3" t="s">
+        <v>205</v>
+      </c>
+      <c r="DC3" t="s">
+        <v>206</v>
+      </c>
+      <c r="DD3" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="DE3" t="s">
+        <v>207</v>
+      </c>
+      <c r="DF3" t="s">
+        <v>208</v>
+      </c>
+      <c r="DG3" t="s">
+        <v>208</v>
+      </c>
+      <c r="DH3" t="s">
+        <v>208</v>
+      </c>
+      <c r="DI3" t="s">
+        <v>208</v>
+      </c>
+      <c r="DJ3" t="s">
+        <v>208</v>
+      </c>
+      <c r="DK3" t="s">
+        <v>208</v>
+      </c>
+      <c r="DL3" t="s">
+        <v>208</v>
+      </c>
+      <c r="DM3" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="DN3" t="s">
+        <v>209</v>
+      </c>
+      <c r="DO3" t="s">
+        <v>209</v>
+      </c>
+      <c r="DP3" t="s">
+        <v>209</v>
+      </c>
+      <c r="DQ3" t="s">
+        <v>210</v>
+      </c>
+      <c r="DR3" t="s">
+        <v>211</v>
+      </c>
+      <c r="DS3" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="DT3" t="s">
+        <v>212</v>
+      </c>
+      <c r="DU3" t="s">
+        <v>213</v>
+      </c>
+      <c r="DV3" t="s">
+        <v>214</v>
+      </c>
+      <c r="DW3" t="s">
+        <v>185</v>
+      </c>
+      <c r="DX3" t="s">
+        <v>215</v>
+      </c>
+      <c r="DY3" t="s">
+        <v>216</v>
+      </c>
+      <c r="DZ3" t="s">
+        <v>217</v>
+      </c>
+      <c r="EA3" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="EB3" t="s">
+        <v>185</v>
+      </c>
+      <c r="EC3" t="s">
+        <v>185</v>
+      </c>
+      <c r="ED3" t="s">
+        <v>185</v>
+      </c>
+      <c r="EE3" t="s">
+        <v>185</v>
+      </c>
+      <c r="EF3" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="EG3" t="s">
         <v>187</v>
       </c>
-      <c r="BV3" t="s">
-        <v>196</v>
-      </c>
-      <c r="BW3" t="s">
-        <v>198</v>
-      </c>
-      <c r="BX3" t="s">
-        <v>192</v>
-      </c>
-      <c r="BY3">
-        <v>110</v>
-      </c>
-      <c r="BZ3">
-        <v>80</v>
-      </c>
-      <c r="CA3" t="s">
-        <v>186</v>
-      </c>
-      <c r="CB3" t="s">
-        <v>199</v>
-      </c>
-      <c r="CC3" t="s">
-        <v>186</v>
-      </c>
-      <c r="CD3" t="s">
-        <v>186</v>
-      </c>
-      <c r="CE3" t="s">
-        <v>186</v>
-      </c>
-      <c r="CF3" t="s">
-        <v>186</v>
-      </c>
-      <c r="CG3" t="s">
-        <v>186</v>
-      </c>
-      <c r="CH3" t="s">
-        <v>186</v>
-      </c>
-      <c r="CI3" t="s">
-        <v>186</v>
-      </c>
-      <c r="CJ3" t="s">
-        <v>200</v>
-      </c>
-      <c r="CK3" t="s">
-        <v>201</v>
-      </c>
-      <c r="CL3" t="s">
-        <v>202</v>
-      </c>
-      <c r="CM3" t="s">
-        <v>202</v>
-      </c>
-      <c r="CN3" t="s">
-        <v>202</v>
-      </c>
-      <c r="CO3" t="s">
-        <v>202</v>
-      </c>
-      <c r="CP3" t="s">
-        <v>203</v>
-      </c>
-      <c r="CQ3" t="s">
-        <v>204</v>
-      </c>
-      <c r="CR3" t="s">
-        <v>205</v>
-      </c>
-      <c r="CS3" t="s">
-        <v>202</v>
-      </c>
-      <c r="CT3" t="s">
-        <v>206</v>
-      </c>
-      <c r="CU3" t="s">
-        <v>207</v>
-      </c>
-      <c r="CV3" t="s">
-        <v>208</v>
-      </c>
-      <c r="CW3" t="s">
-        <v>209</v>
-      </c>
-      <c r="CX3" t="s">
-        <v>210</v>
-      </c>
-      <c r="CY3" t="s">
-        <v>210</v>
-      </c>
-      <c r="CZ3" t="s">
-        <v>210</v>
-      </c>
-      <c r="DA3" t="s">
-        <v>210</v>
-      </c>
-      <c r="DB3" t="s">
-        <v>210</v>
-      </c>
-      <c r="DC3" t="s">
-        <v>210</v>
-      </c>
-      <c r="DD3" t="s">
-        <v>210</v>
-      </c>
-      <c r="DE3" t="s">
-        <v>211</v>
-      </c>
-      <c r="DF3" t="s">
-        <v>211</v>
-      </c>
-      <c r="DG3" t="s">
-        <v>211</v>
-      </c>
-      <c r="DH3" t="s">
-        <v>212</v>
-      </c>
-      <c r="DI3" t="s">
-        <v>213</v>
-      </c>
-      <c r="DJ3" t="s">
-        <v>214</v>
-      </c>
-      <c r="DK3" t="s">
-        <v>215</v>
-      </c>
-      <c r="DL3" t="s">
-        <v>216</v>
-      </c>
-      <c r="DM3" t="s">
-        <v>186</v>
-      </c>
-      <c r="DN3" t="s">
-        <v>217</v>
-      </c>
-      <c r="DO3" t="s">
+      <c r="EH3" t="s">
+        <v>186</v>
+      </c>
+      <c r="EI3" t="s">
+        <v>186</v>
+      </c>
+      <c r="EJ3" t="s">
+        <v>186</v>
+      </c>
+      <c r="EK3" t="s">
+        <v>186</v>
+      </c>
+      <c r="EL3" t="s">
+        <v>186</v>
+      </c>
+      <c r="EM3" t="s">
         <v>218</v>
       </c>
-      <c r="DP3" t="s">
+      <c r="EN3" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="EO3" t="s">
         <v>219</v>
       </c>
-      <c r="DQ3" t="s">
-        <v>186</v>
-      </c>
-      <c r="DR3" t="s">
-        <v>186</v>
-      </c>
-      <c r="DS3" t="s">
-        <v>186</v>
-      </c>
-      <c r="DT3" t="s">
-        <v>186</v>
-      </c>
-      <c r="DU3" t="s">
+      <c r="EP3" t="s">
+        <v>220</v>
+      </c>
+      <c r="EQ3" t="s">
+        <v>221</v>
+      </c>
+      <c r="ER3" t="s">
+        <v>222</v>
+      </c>
+      <c r="ES3" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="ET3" t="s">
+        <v>223</v>
+      </c>
+      <c r="EU3" t="s">
+        <v>224</v>
+      </c>
+      <c r="EV3" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="EW3" t="s">
+        <v>225</v>
+      </c>
+      <c r="EX3" t="s">
+        <v>226</v>
+      </c>
+      <c r="EY3" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="EZ3" t="s">
+        <v>225</v>
+      </c>
+      <c r="FA3" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="FB3" t="s">
+        <v>227</v>
+      </c>
+      <c r="FC3" t="s">
+        <v>228</v>
+      </c>
+      <c r="FD3" t="s">
+        <v>229</v>
+      </c>
+      <c r="FE3" t="s">
+        <v>230</v>
+      </c>
+      <c r="FF3" t="s">
+        <v>231</v>
+      </c>
+      <c r="FG3" t="s">
+        <v>232</v>
+      </c>
+      <c r="FH3" t="s">
+        <v>233</v>
+      </c>
+      <c r="FI3" t="s">
+        <v>234</v>
+      </c>
+      <c r="FJ3" t="s">
+        <v>218</v>
+      </c>
+      <c r="FK3" t="s">
+        <v>235</v>
+      </c>
+      <c r="FL3" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="FM3" t="s">
+        <v>185</v>
+      </c>
+      <c r="FN3" t="s">
+        <v>186</v>
+      </c>
+      <c r="FO3" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="FP3" t="s">
+        <v>185</v>
+      </c>
+      <c r="FQ3" t="s">
+        <v>185</v>
+      </c>
+      <c r="FR3" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="FS3" t="s">
+        <v>261</v>
+      </c>
+      <c r="FT3" t="s">
+        <v>236</v>
+      </c>
+      <c r="FU3" t="s">
+        <v>186</v>
+      </c>
+      <c r="FV3" t="s">
+        <v>186</v>
+      </c>
+      <c r="FW3" t="s">
+        <v>186</v>
+      </c>
+      <c r="FX3" t="s">
+        <v>186</v>
+      </c>
+      <c r="FY3" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="FZ3" t="s">
+        <v>193</v>
+      </c>
+      <c r="GA3" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="GB3" t="s">
+        <v>237</v>
+      </c>
+      <c r="GC3" t="s">
+        <v>237</v>
+      </c>
+      <c r="GD3" t="s">
+        <v>238</v>
+      </c>
+      <c r="GE3" t="s">
+        <v>239</v>
+      </c>
+      <c r="GF3" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="GG3" t="s">
+        <v>240</v>
+      </c>
+      <c r="GH3" t="s">
+        <v>241</v>
+      </c>
+      <c r="GI3" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="GJ3" t="s">
+        <v>242</v>
+      </c>
+      <c r="GK3" t="s">
+        <v>243</v>
+      </c>
+      <c r="GL3" t="s">
+        <v>244</v>
+      </c>
+      <c r="GM3" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="GN3">
+        <v>0.5</v>
+      </c>
+      <c r="GO3">
+        <v>49</v>
+      </c>
+      <c r="GP3">
+        <v>60</v>
+      </c>
+      <c r="GQ3">
+        <v>10</v>
+      </c>
+      <c r="GR3" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="GS3" t="s">
+        <v>245</v>
+      </c>
+      <c r="GT3" t="s">
+        <v>246</v>
+      </c>
+      <c r="GU3" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="GV3" t="s">
+        <v>218</v>
+      </c>
+      <c r="GW3" t="s">
+        <v>218</v>
+      </c>
+      <c r="GX3" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="GY3" t="s">
+        <v>247</v>
+      </c>
+      <c r="GZ3" t="s">
+        <v>248</v>
+      </c>
+      <c r="HA3" t="s">
+        <v>249</v>
+      </c>
+      <c r="HB3" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="HC3" t="s">
+        <v>250</v>
+      </c>
+      <c r="HD3" t="s">
+        <v>251</v>
+      </c>
+      <c r="HE3" t="s">
+        <v>252</v>
+      </c>
+      <c r="HF3" t="s">
+        <v>253</v>
+      </c>
+      <c r="HG3" t="s">
+        <v>254</v>
+      </c>
+      <c r="HH3" t="s">
+        <v>255</v>
+      </c>
+      <c r="HI3" t="s">
+        <v>256</v>
+      </c>
+      <c r="HJ3" t="s">
+        <v>218</v>
+      </c>
+      <c r="HK3" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="4" spans="1:219" x14ac:dyDescent="0.2">
+      <c r="A4" s="1" t="s">
+        <v>263</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>264</v>
+      </c>
+      <c r="C4" t="s">
+        <v>262</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>186</v>
+      </c>
+      <c r="E4" t="s">
+        <v>260</v>
+      </c>
+      <c r="F4" t="s">
+        <v>184</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>185</v>
+      </c>
+      <c r="H4" t="s">
+        <v>185</v>
+      </c>
+      <c r="I4" t="s">
+        <v>186</v>
+      </c>
+      <c r="J4" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="K4" t="s">
+        <v>187</v>
+      </c>
+      <c r="L4" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="M4" t="s">
+        <v>186</v>
+      </c>
+      <c r="N4" t="s">
+        <v>186</v>
+      </c>
+      <c r="O4" t="s">
+        <v>186</v>
+      </c>
+      <c r="P4" t="s">
+        <v>186</v>
+      </c>
+      <c r="Q4" t="s">
+        <v>186</v>
+      </c>
+      <c r="R4" t="s">
+        <v>186</v>
+      </c>
+      <c r="S4" t="s">
+        <v>186</v>
+      </c>
+      <c r="T4" t="s">
+        <v>186</v>
+      </c>
+      <c r="U4" t="s">
+        <v>186</v>
+      </c>
+      <c r="V4" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="W4" t="s">
         <v>188</v>
       </c>
-      <c r="DV3" t="s">
-        <v>187</v>
-      </c>
-      <c r="DW3" t="s">
-        <v>187</v>
-      </c>
-      <c r="DX3" t="s">
-        <v>187</v>
-      </c>
-      <c r="DY3" t="s">
-        <v>187</v>
-      </c>
-      <c r="DZ3" t="s">
-        <v>187</v>
-      </c>
-      <c r="EA3" t="s">
-        <v>220</v>
-      </c>
-      <c r="EB3" t="s">
-        <v>221</v>
-      </c>
-      <c r="EC3" t="s">
-        <v>222</v>
-      </c>
-      <c r="ED3" t="s">
-        <v>223</v>
-      </c>
-      <c r="EE3" t="s">
-        <v>224</v>
-      </c>
-      <c r="EF3" t="s">
-        <v>225</v>
-      </c>
-      <c r="EG3" t="s">
-        <v>226</v>
-      </c>
-      <c r="EH3" t="s">
-        <v>227</v>
-      </c>
-      <c r="EI3" t="s">
-        <v>228</v>
-      </c>
-      <c r="EJ3" t="s">
-        <v>227</v>
-      </c>
-      <c r="EK3" t="s">
-        <v>229</v>
-      </c>
-      <c r="EL3" t="s">
-        <v>230</v>
-      </c>
-      <c r="EM3" t="s">
-        <v>231</v>
-      </c>
-      <c r="EN3" t="s">
-        <v>232</v>
-      </c>
-      <c r="EO3" t="s">
-        <v>233</v>
-      </c>
-      <c r="EP3" t="s">
-        <v>234</v>
-      </c>
-      <c r="EQ3" t="s">
-        <v>235</v>
-      </c>
-      <c r="ER3" t="s">
-        <v>236</v>
-      </c>
-      <c r="ES3" t="s">
-        <v>220</v>
-      </c>
-      <c r="ET3" t="s">
-        <v>237</v>
-      </c>
-      <c r="EU3" t="s">
-        <v>186</v>
-      </c>
-      <c r="EV3" t="s">
-        <v>187</v>
-      </c>
-      <c r="EW3" t="s">
-        <v>186</v>
-      </c>
-      <c r="EX3" t="s">
-        <v>186</v>
-      </c>
-      <c r="EY3" t="s">
-        <v>263</v>
-      </c>
-      <c r="EZ3" t="s">
-        <v>238</v>
-      </c>
-      <c r="FA3" t="s">
-        <v>187</v>
-      </c>
-      <c r="FB3" t="s">
-        <v>187</v>
-      </c>
-      <c r="FC3" t="s">
-        <v>187</v>
-      </c>
-      <c r="FD3" t="s">
-        <v>187</v>
-      </c>
-      <c r="FE3" t="s">
-        <v>194</v>
-      </c>
-      <c r="FF3" t="s">
-        <v>239</v>
-      </c>
-      <c r="FG3" t="s">
-        <v>239</v>
-      </c>
-      <c r="FH3" t="s">
-        <v>240</v>
-      </c>
-      <c r="FI3" t="s">
-        <v>241</v>
-      </c>
-      <c r="FJ3" t="s">
-        <v>242</v>
-      </c>
-      <c r="FK3" t="s">
-        <v>243</v>
-      </c>
-      <c r="FL3" t="s">
-        <v>244</v>
-      </c>
-      <c r="FM3" t="s">
-        <v>245</v>
-      </c>
-      <c r="FN3" t="s">
-        <v>246</v>
-      </c>
-      <c r="FO3">
-        <v>0.5</v>
-      </c>
-      <c r="FP3">
-        <v>49</v>
-      </c>
-      <c r="FQ3">
-        <v>60</v>
-      </c>
-      <c r="FR3">
-        <v>10</v>
-      </c>
-      <c r="FS3" t="s">
-        <v>247</v>
-      </c>
-      <c r="FT3" t="s">
-        <v>248</v>
-      </c>
-      <c r="FU3" t="s">
-        <v>220</v>
-      </c>
-      <c r="FV3" t="s">
-        <v>220</v>
-      </c>
-      <c r="FW3" t="s">
-        <v>249</v>
-      </c>
-      <c r="FX3" t="s">
-        <v>250</v>
-      </c>
-      <c r="FY3" t="s">
-        <v>251</v>
-      </c>
-      <c r="FZ3" t="s">
-        <v>252</v>
-      </c>
-      <c r="GA3" t="s">
-        <v>253</v>
-      </c>
-      <c r="GB3" t="s">
-        <v>254</v>
-      </c>
-      <c r="GC3" t="s">
-        <v>255</v>
-      </c>
-      <c r="GD3" t="s">
-        <v>256</v>
-      </c>
-      <c r="GE3" t="s">
-        <v>257</v>
-      </c>
-      <c r="GF3" t="s">
-        <v>258</v>
-      </c>
-      <c r="GG3" t="s">
-        <v>220</v>
-      </c>
-      <c r="GH3" t="s">
-        <v>259</v>
-      </c>
-    </row>
-    <row r="4" spans="1:190" x14ac:dyDescent="0.2">
-      <c r="A4" s="1" t="s">
-        <v>265</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>266</v>
-      </c>
-      <c r="C4" t="s">
-        <v>264</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>187</v>
-      </c>
-      <c r="E4" t="s">
-        <v>262</v>
-      </c>
-      <c r="F4" t="s">
-        <v>185</v>
-      </c>
-      <c r="G4" s="2" t="s">
-        <v>186</v>
-      </c>
-      <c r="H4" t="s">
-        <v>186</v>
-      </c>
-      <c r="I4" t="s">
-        <v>187</v>
-      </c>
-      <c r="J4" s="3" t="s">
-        <v>186</v>
-      </c>
-      <c r="K4" t="s">
+      <c r="X4" t="s">
         <v>188</v>
       </c>
-      <c r="L4" s="3" t="s">
-        <v>186</v>
-      </c>
-      <c r="M4" t="s">
-        <v>187</v>
-      </c>
-      <c r="N4" t="s">
-        <v>187</v>
-      </c>
-      <c r="O4" t="s">
-        <v>187</v>
-      </c>
-      <c r="P4" t="s">
-        <v>187</v>
-      </c>
-      <c r="Q4" t="s">
-        <v>187</v>
-      </c>
-      <c r="R4" t="s">
-        <v>187</v>
-      </c>
-      <c r="S4" t="s">
-        <v>187</v>
-      </c>
-      <c r="T4" t="s">
-        <v>187</v>
-      </c>
-      <c r="U4" t="s">
-        <v>187</v>
-      </c>
-      <c r="V4" s="3" t="s">
-        <v>186</v>
-      </c>
-      <c r="W4" t="s">
+      <c r="Y4" t="s">
+        <v>188</v>
+      </c>
+      <c r="Z4" t="s">
+        <v>188</v>
+      </c>
+      <c r="AA4" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="AB4" t="s">
+        <v>186</v>
+      </c>
+      <c r="AC4" t="s">
+        <v>186</v>
+      </c>
+      <c r="AD4" t="s">
+        <v>186</v>
+      </c>
+      <c r="AE4" t="s">
+        <v>186</v>
+      </c>
+      <c r="AF4" t="s">
+        <v>186</v>
+      </c>
+      <c r="AG4" t="s">
+        <v>186</v>
+      </c>
+      <c r="AH4" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="AI4" t="s">
+        <v>186</v>
+      </c>
+      <c r="AJ4" t="s">
         <v>189</v>
-      </c>
-      <c r="X4" t="s">
-        <v>189</v>
-      </c>
-      <c r="Y4" t="s">
-        <v>189</v>
-      </c>
-      <c r="Z4" t="s">
-        <v>189</v>
-      </c>
-      <c r="AA4" s="3" t="s">
-        <v>186</v>
-      </c>
-      <c r="AB4" t="s">
-        <v>187</v>
-      </c>
-      <c r="AC4" t="s">
-        <v>187</v>
-      </c>
-      <c r="AD4" t="s">
-        <v>187</v>
-      </c>
-      <c r="AE4" t="s">
-        <v>187</v>
-      </c>
-      <c r="AF4" t="s">
-        <v>187</v>
-      </c>
-      <c r="AG4" t="s">
-        <v>187</v>
-      </c>
-      <c r="AH4" s="3" t="s">
-        <v>186</v>
-      </c>
-      <c r="AI4" t="s">
-        <v>187</v>
-      </c>
-      <c r="AJ4" t="s">
-        <v>190</v>
       </c>
       <c r="AK4">
         <v>3</v>
@@ -3759,22 +4139,22 @@
         <v>15</v>
       </c>
       <c r="AM4" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="AN4">
         <v>3</v>
       </c>
       <c r="AO4" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="AP4" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="AQ4" s="3" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="AR4" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="AS4">
         <v>5</v>
@@ -3783,7 +4163,7 @@
         <v>60</v>
       </c>
       <c r="AU4" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="AV4">
         <v>6</v>
@@ -3792,7 +4172,7 @@
         <v>30</v>
       </c>
       <c r="AX4" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="AY4">
         <v>3</v>
@@ -3801,7 +4181,7 @@
         <v>120</v>
       </c>
       <c r="BA4" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="BB4">
         <v>2</v>
@@ -3810,7 +4190,7 @@
         <v>100</v>
       </c>
       <c r="BD4" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="BE4">
         <v>1</v>
@@ -3819,7 +4199,7 @@
         <v>20</v>
       </c>
       <c r="BG4" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="BH4">
         <v>1</v>
@@ -3827,389 +4207,479 @@
       <c r="BI4">
         <v>20</v>
       </c>
+      <c r="BJ4" s="3" t="s">
+        <v>185</v>
+      </c>
       <c r="BK4" t="s">
+        <v>191</v>
+      </c>
+      <c r="BL4" t="s">
         <v>192</v>
       </c>
-      <c r="BL4" t="s">
+      <c r="BM4" t="s">
         <v>193</v>
       </c>
-      <c r="BM4" t="s">
+      <c r="BN4" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="BO4" t="s">
+        <v>186</v>
+      </c>
+      <c r="BP4" t="s">
         <v>194</v>
       </c>
-      <c r="BN4" t="s">
+      <c r="BQ4" t="s">
         <v>195</v>
-      </c>
-      <c r="BO4" t="s">
-        <v>187</v>
-      </c>
-      <c r="BP4" t="s">
-        <v>196</v>
-      </c>
-      <c r="BQ4" t="s">
-        <v>197</v>
       </c>
       <c r="BR4">
         <v>100</v>
       </c>
       <c r="BS4" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="BT4">
         <v>90</v>
       </c>
-      <c r="BU4" t="s">
+      <c r="BU4" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="BV4" t="s">
+        <v>186</v>
+      </c>
+      <c r="BW4" t="s">
+        <v>194</v>
+      </c>
+      <c r="BX4" t="s">
+        <v>196</v>
+      </c>
+      <c r="BY4" t="s">
+        <v>191</v>
+      </c>
+      <c r="BZ4">
+        <v>110</v>
+      </c>
+      <c r="CA4">
+        <v>80</v>
+      </c>
+      <c r="CB4" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="CC4" t="s">
+        <v>185</v>
+      </c>
+      <c r="CD4" t="s">
+        <v>197</v>
+      </c>
+      <c r="CE4" t="s">
+        <v>185</v>
+      </c>
+      <c r="CF4" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="CG4" t="s">
+        <v>185</v>
+      </c>
+      <c r="CH4" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="CI4" t="s">
+        <v>185</v>
+      </c>
+      <c r="CJ4" t="s">
+        <v>185</v>
+      </c>
+      <c r="CK4" t="s">
+        <v>185</v>
+      </c>
+      <c r="CL4" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="CM4" t="s">
+        <v>185</v>
+      </c>
+      <c r="CN4" t="s">
+        <v>185</v>
+      </c>
+      <c r="CO4" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="CP4" t="s">
+        <v>198</v>
+      </c>
+      <c r="CQ4" t="s">
+        <v>199</v>
+      </c>
+      <c r="CR4" t="s">
+        <v>200</v>
+      </c>
+      <c r="CS4" t="s">
+        <v>200</v>
+      </c>
+      <c r="CT4" t="s">
+        <v>200</v>
+      </c>
+      <c r="CU4" t="s">
+        <v>200</v>
+      </c>
+      <c r="CV4" t="s">
+        <v>201</v>
+      </c>
+      <c r="CW4" t="s">
+        <v>202</v>
+      </c>
+      <c r="CX4" t="s">
+        <v>203</v>
+      </c>
+      <c r="CY4" t="s">
+        <v>200</v>
+      </c>
+      <c r="CZ4" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="DA4" t="s">
+        <v>204</v>
+      </c>
+      <c r="DB4" t="s">
+        <v>205</v>
+      </c>
+      <c r="DC4" t="s">
+        <v>206</v>
+      </c>
+      <c r="DD4" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="DE4" t="s">
+        <v>207</v>
+      </c>
+      <c r="DF4" t="s">
+        <v>208</v>
+      </c>
+      <c r="DG4" t="s">
+        <v>208</v>
+      </c>
+      <c r="DH4" t="s">
+        <v>208</v>
+      </c>
+      <c r="DI4" t="s">
+        <v>208</v>
+      </c>
+      <c r="DJ4" t="s">
+        <v>208</v>
+      </c>
+      <c r="DK4" t="s">
+        <v>208</v>
+      </c>
+      <c r="DL4" t="s">
+        <v>208</v>
+      </c>
+      <c r="DM4" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="DN4" t="s">
+        <v>209</v>
+      </c>
+      <c r="DO4" t="s">
+        <v>209</v>
+      </c>
+      <c r="DP4" t="s">
+        <v>209</v>
+      </c>
+      <c r="DQ4" t="s">
+        <v>210</v>
+      </c>
+      <c r="DR4" t="s">
+        <v>211</v>
+      </c>
+      <c r="DS4" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="DT4" t="s">
+        <v>212</v>
+      </c>
+      <c r="DU4" t="s">
+        <v>213</v>
+      </c>
+      <c r="DV4" t="s">
+        <v>214</v>
+      </c>
+      <c r="DW4" t="s">
+        <v>185</v>
+      </c>
+      <c r="DX4" t="s">
+        <v>215</v>
+      </c>
+      <c r="DY4" t="s">
+        <v>216</v>
+      </c>
+      <c r="DZ4" t="s">
+        <v>217</v>
+      </c>
+      <c r="EA4" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="EB4" t="s">
+        <v>185</v>
+      </c>
+      <c r="EC4" t="s">
+        <v>185</v>
+      </c>
+      <c r="ED4" t="s">
+        <v>185</v>
+      </c>
+      <c r="EE4" t="s">
+        <v>185</v>
+      </c>
+      <c r="EF4" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="EG4" t="s">
         <v>187</v>
       </c>
-      <c r="BV4" t="s">
-        <v>196</v>
-      </c>
-      <c r="BW4" t="s">
-        <v>198</v>
-      </c>
-      <c r="BX4" t="s">
-        <v>192</v>
-      </c>
-      <c r="BY4">
-        <v>110</v>
-      </c>
-      <c r="BZ4">
-        <v>80</v>
-      </c>
-      <c r="CA4" t="s">
-        <v>186</v>
-      </c>
-      <c r="CB4" t="s">
-        <v>199</v>
-      </c>
-      <c r="CC4" t="s">
-        <v>186</v>
-      </c>
-      <c r="CD4" t="s">
-        <v>186</v>
-      </c>
-      <c r="CE4" t="s">
-        <v>186</v>
-      </c>
-      <c r="CF4" t="s">
-        <v>186</v>
-      </c>
-      <c r="CG4" t="s">
-        <v>186</v>
-      </c>
-      <c r="CH4" t="s">
-        <v>186</v>
-      </c>
-      <c r="CI4" t="s">
-        <v>186</v>
-      </c>
-      <c r="CJ4" t="s">
-        <v>200</v>
-      </c>
-      <c r="CK4" t="s">
-        <v>201</v>
-      </c>
-      <c r="CL4" t="s">
-        <v>202</v>
-      </c>
-      <c r="CM4" t="s">
-        <v>202</v>
-      </c>
-      <c r="CN4" t="s">
-        <v>202</v>
-      </c>
-      <c r="CO4" t="s">
-        <v>202</v>
-      </c>
-      <c r="CP4" t="s">
-        <v>203</v>
-      </c>
-      <c r="CQ4" t="s">
-        <v>204</v>
-      </c>
-      <c r="CR4" t="s">
-        <v>205</v>
-      </c>
-      <c r="CS4" t="s">
-        <v>202</v>
-      </c>
-      <c r="CT4" t="s">
-        <v>206</v>
-      </c>
-      <c r="CU4" t="s">
-        <v>207</v>
-      </c>
-      <c r="CV4" t="s">
-        <v>208</v>
-      </c>
-      <c r="CW4" t="s">
-        <v>209</v>
-      </c>
-      <c r="CX4" t="s">
-        <v>210</v>
-      </c>
-      <c r="CY4" t="s">
-        <v>210</v>
-      </c>
-      <c r="CZ4" t="s">
-        <v>210</v>
-      </c>
-      <c r="DA4" t="s">
-        <v>210</v>
-      </c>
-      <c r="DB4" t="s">
-        <v>210</v>
-      </c>
-      <c r="DC4" t="s">
-        <v>210</v>
-      </c>
-      <c r="DD4" t="s">
-        <v>210</v>
-      </c>
-      <c r="DE4" t="s">
-        <v>211</v>
-      </c>
-      <c r="DF4" t="s">
-        <v>211</v>
-      </c>
-      <c r="DG4" t="s">
-        <v>211</v>
-      </c>
-      <c r="DH4" t="s">
-        <v>212</v>
-      </c>
-      <c r="DI4" t="s">
-        <v>213</v>
-      </c>
-      <c r="DJ4" t="s">
-        <v>214</v>
-      </c>
-      <c r="DK4" t="s">
-        <v>215</v>
-      </c>
-      <c r="DL4" t="s">
-        <v>216</v>
-      </c>
-      <c r="DM4" t="s">
-        <v>186</v>
-      </c>
-      <c r="DN4" t="s">
-        <v>217</v>
-      </c>
-      <c r="DO4" t="s">
+      <c r="EH4" t="s">
+        <v>186</v>
+      </c>
+      <c r="EI4" t="s">
+        <v>186</v>
+      </c>
+      <c r="EJ4" t="s">
+        <v>186</v>
+      </c>
+      <c r="EK4" t="s">
+        <v>186</v>
+      </c>
+      <c r="EL4" t="s">
+        <v>186</v>
+      </c>
+      <c r="EM4" t="s">
         <v>218</v>
       </c>
-      <c r="DP4" t="s">
+      <c r="EN4" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="EO4" t="s">
         <v>219</v>
       </c>
-      <c r="DQ4" t="s">
-        <v>186</v>
-      </c>
-      <c r="DR4" t="s">
-        <v>186</v>
-      </c>
-      <c r="DS4" t="s">
-        <v>186</v>
-      </c>
-      <c r="DT4" t="s">
-        <v>186</v>
-      </c>
-      <c r="DU4" t="s">
-        <v>188</v>
-      </c>
-      <c r="DV4" t="s">
-        <v>187</v>
-      </c>
-      <c r="DW4" t="s">
-        <v>187</v>
-      </c>
-      <c r="DX4" t="s">
-        <v>187</v>
-      </c>
-      <c r="DY4" t="s">
-        <v>187</v>
-      </c>
-      <c r="DZ4" t="s">
-        <v>187</v>
-      </c>
-      <c r="EA4" t="s">
+      <c r="EP4" t="s">
         <v>220</v>
       </c>
-      <c r="EB4" t="s">
+      <c r="EQ4" t="s">
         <v>221</v>
       </c>
-      <c r="EC4" t="s">
+      <c r="ER4" t="s">
         <v>222</v>
       </c>
-      <c r="ED4" t="s">
+      <c r="ES4" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="ET4" t="s">
         <v>223</v>
       </c>
-      <c r="EE4" t="s">
+      <c r="EU4" t="s">
         <v>224</v>
       </c>
-      <c r="EF4" t="s">
+      <c r="EV4" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="EW4" t="s">
         <v>225</v>
       </c>
-      <c r="EG4" t="s">
+      <c r="EX4" t="s">
         <v>226</v>
       </c>
-      <c r="EH4" t="s">
+      <c r="EY4" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="EZ4" t="s">
+        <v>225</v>
+      </c>
+      <c r="FA4" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="FB4" t="s">
         <v>227</v>
       </c>
-      <c r="EI4" t="s">
+      <c r="FC4" t="s">
         <v>228</v>
       </c>
-      <c r="EJ4" t="s">
-        <v>227</v>
-      </c>
-      <c r="EK4" t="s">
+      <c r="FD4" t="s">
         <v>229</v>
       </c>
-      <c r="EL4" t="s">
+      <c r="FE4" t="s">
         <v>230</v>
       </c>
-      <c r="EM4" t="s">
+      <c r="FF4" t="s">
         <v>231</v>
       </c>
-      <c r="EN4" t="s">
+      <c r="FG4" t="s">
         <v>232</v>
       </c>
-      <c r="EO4" t="s">
+      <c r="FH4" t="s">
         <v>233</v>
       </c>
-      <c r="EP4" t="s">
+      <c r="FI4" t="s">
         <v>234</v>
       </c>
-      <c r="EQ4" t="s">
+      <c r="FJ4" t="s">
+        <v>218</v>
+      </c>
+      <c r="FK4" t="s">
         <v>235</v>
       </c>
-      <c r="ER4" t="s">
+      <c r="FL4" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="FM4" t="s">
+        <v>185</v>
+      </c>
+      <c r="FN4" t="s">
+        <v>186</v>
+      </c>
+      <c r="FO4" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="FP4" t="s">
+        <v>185</v>
+      </c>
+      <c r="FQ4" t="s">
+        <v>185</v>
+      </c>
+      <c r="FR4" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="FS4" t="s">
+        <v>261</v>
+      </c>
+      <c r="FT4" t="s">
         <v>236</v>
       </c>
-      <c r="ES4" t="s">
-        <v>220</v>
-      </c>
-      <c r="ET4" t="s">
+      <c r="FU4" t="s">
+        <v>186</v>
+      </c>
+      <c r="FV4" t="s">
+        <v>186</v>
+      </c>
+      <c r="FW4" t="s">
+        <v>186</v>
+      </c>
+      <c r="FX4" t="s">
+        <v>186</v>
+      </c>
+      <c r="FY4" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="FZ4" t="s">
+        <v>193</v>
+      </c>
+      <c r="GA4" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="GB4" t="s">
         <v>237</v>
       </c>
-      <c r="EU4" t="s">
-        <v>186</v>
-      </c>
-      <c r="EV4" t="s">
-        <v>187</v>
-      </c>
-      <c r="EW4" t="s">
-        <v>186</v>
-      </c>
-      <c r="EX4" t="s">
-        <v>186</v>
-      </c>
-      <c r="EY4" t="s">
-        <v>263</v>
-      </c>
-      <c r="EZ4" t="s">
+      <c r="GC4" t="s">
+        <v>237</v>
+      </c>
+      <c r="GD4" t="s">
         <v>238</v>
       </c>
-      <c r="FA4" t="s">
-        <v>187</v>
-      </c>
-      <c r="FB4" t="s">
-        <v>187</v>
-      </c>
-      <c r="FC4" t="s">
-        <v>187</v>
-      </c>
-      <c r="FD4" t="s">
-        <v>187</v>
-      </c>
-      <c r="FE4" t="s">
-        <v>194</v>
-      </c>
-      <c r="FF4" t="s">
+      <c r="GE4" t="s">
         <v>239</v>
       </c>
-      <c r="FG4" t="s">
-        <v>239</v>
-      </c>
-      <c r="FH4" t="s">
+      <c r="GF4" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="GG4" t="s">
         <v>240</v>
       </c>
-      <c r="FI4" t="s">
+      <c r="GH4" t="s">
         <v>241</v>
       </c>
-      <c r="FJ4" t="s">
+      <c r="GI4" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="GJ4" t="s">
         <v>242</v>
       </c>
-      <c r="FK4" t="s">
+      <c r="GK4" t="s">
         <v>243</v>
       </c>
-      <c r="FL4" t="s">
+      <c r="GL4" t="s">
         <v>244</v>
       </c>
-      <c r="FM4" t="s">
+      <c r="GM4" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="GN4">
+        <v>0.5</v>
+      </c>
+      <c r="GO4">
+        <v>49</v>
+      </c>
+      <c r="GP4">
+        <v>60</v>
+      </c>
+      <c r="GQ4">
+        <v>10</v>
+      </c>
+      <c r="GR4" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="GS4" t="s">
         <v>245</v>
       </c>
-      <c r="FN4" t="s">
+      <c r="GT4" t="s">
         <v>246</v>
       </c>
-      <c r="FO4">
-        <v>0.5</v>
-      </c>
-      <c r="FP4">
-        <v>49</v>
-      </c>
-      <c r="FQ4">
-        <v>60</v>
-      </c>
-      <c r="FR4">
-        <v>10</v>
-      </c>
-      <c r="FS4" t="s">
+      <c r="GU4" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="GV4" t="s">
+        <v>218</v>
+      </c>
+      <c r="GW4" t="s">
+        <v>218</v>
+      </c>
+      <c r="GX4" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="GY4" t="s">
         <v>247</v>
       </c>
-      <c r="FT4" t="s">
+      <c r="GZ4" t="s">
         <v>248</v>
       </c>
-      <c r="FU4" t="s">
-        <v>220</v>
-      </c>
-      <c r="FV4" t="s">
-        <v>220</v>
-      </c>
-      <c r="FW4" t="s">
+      <c r="HA4" t="s">
         <v>249</v>
       </c>
-      <c r="FX4" t="s">
+      <c r="HB4" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="HC4" t="s">
         <v>250</v>
       </c>
-      <c r="FY4" t="s">
+      <c r="HD4" t="s">
         <v>251</v>
       </c>
-      <c r="FZ4" t="s">
+      <c r="HE4" t="s">
         <v>252</v>
       </c>
-      <c r="GA4" t="s">
+      <c r="HF4" t="s">
         <v>253</v>
       </c>
-      <c r="GB4" t="s">
+      <c r="HG4" t="s">
         <v>254</v>
       </c>
-      <c r="GC4" t="s">
+      <c r="HH4" t="s">
         <v>255</v>
       </c>
-      <c r="GD4" t="s">
+      <c r="HI4" t="s">
         <v>256</v>
       </c>
-      <c r="GE4" t="s">
-        <v>257</v>
-      </c>
-      <c r="GF4" t="s">
-        <v>258</v>
-      </c>
-      <c r="GG4" t="s">
-        <v>220</v>
+      <c r="HJ4" t="s">
+        <v>218</v>
       </c>
     </row>
-    <row r="5" spans="1:190" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:219" x14ac:dyDescent="0.2">
       <c r="D5" s="2"/>
       <c r="G5" s="2"/>
       <c r="J5" s="3"/>
@@ -4218,7 +4688,7 @@
       <c r="AH5" s="3"/>
       <c r="AQ5" s="3"/>
     </row>
-    <row r="6" spans="1:190" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:219" x14ac:dyDescent="0.2">
       <c r="D6" s="2"/>
       <c r="G6" s="2"/>
       <c r="J6" s="3"/>
@@ -4227,7 +4697,7 @@
       <c r="AH6" s="3"/>
       <c r="AQ6" s="3"/>
     </row>
-    <row r="7" spans="1:190" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:219" x14ac:dyDescent="0.2">
       <c r="D7" s="2"/>
       <c r="G7" s="2"/>
       <c r="J7" s="3"/>
@@ -4236,7 +4706,7 @@
       <c r="AH7" s="3"/>
       <c r="AQ7" s="3"/>
     </row>
-    <row r="8" spans="1:190" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:219" x14ac:dyDescent="0.2">
       <c r="D8" s="2"/>
       <c r="G8" s="2"/>
       <c r="J8" s="3"/>
@@ -4245,7 +4715,7 @@
       <c r="AH8" s="3"/>
       <c r="AQ8" s="3"/>
     </row>
-    <row r="9" spans="1:190" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:219" x14ac:dyDescent="0.2">
       <c r="D9" s="2"/>
       <c r="G9" s="2"/>
       <c r="J9" s="3"/>
@@ -4254,7 +4724,7 @@
       <c r="AH9" s="3"/>
       <c r="AQ9" s="3"/>
     </row>
-    <row r="10" spans="1:190" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:219" x14ac:dyDescent="0.2">
       <c r="D10" s="2"/>
       <c r="G10" s="2"/>
       <c r="J10" s="3"/>
@@ -4263,7 +4733,7 @@
       <c r="AH10" s="3"/>
       <c r="AQ10" s="3"/>
     </row>
-    <row r="11" spans="1:190" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:219" x14ac:dyDescent="0.2">
       <c r="D11" s="2"/>
       <c r="G11" s="2"/>
       <c r="J11" s="3"/>
@@ -4272,7 +4742,7 @@
       <c r="AH11" s="3"/>
       <c r="AQ11" s="3"/>
     </row>
-    <row r="12" spans="1:190" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:219" x14ac:dyDescent="0.2">
       <c r="D12" s="2"/>
       <c r="G12" s="2"/>
       <c r="J12" s="3"/>
@@ -4281,7 +4751,7 @@
       <c r="AH12" s="3"/>
       <c r="AQ12" s="3"/>
     </row>
-    <row r="13" spans="1:190" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:219" x14ac:dyDescent="0.2">
       <c r="D13" s="2"/>
       <c r="G13" s="2"/>
       <c r="J13" s="3"/>
@@ -4290,7 +4760,7 @@
       <c r="AH13" s="3"/>
       <c r="AQ13" s="3"/>
     </row>
-    <row r="14" spans="1:190" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:219" x14ac:dyDescent="0.2">
       <c r="D14" s="2"/>
       <c r="G14" s="2"/>
       <c r="J14" s="3"/>
@@ -4299,10 +4769,10 @@
       <c r="AH14" s="3"/>
       <c r="AQ14" s="3"/>
     </row>
-    <row r="15" spans="1:190" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:219" x14ac:dyDescent="0.2">
       <c r="J15" s="3"/>
     </row>
-    <row r="16" spans="1:190" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:219" x14ac:dyDescent="0.2">
       <c r="J16" s="3"/>
     </row>
     <row r="17" spans="10:10" x14ac:dyDescent="0.2">
@@ -4315,11 +4785,11 @@
       <c r="J19" s="3"/>
     </row>
   </sheetData>
-  <dataValidations count="64">
+  <dataValidations count="63">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E2:E4" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"Belum Menikah,Menikah,Cerai Mati,Cerai Hidup"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G2:G14 L2:L14 AA2:AA14 AM2:AM4 AH2:AH19 AU2:AU4 AX2:AX4 BA2:BA4 BD2:BD4 BG2:BG4 BO2:BO4 BU2:BU4 CA2:CA4 CC2:CI4 DM2:DM4 DQ2:DT4 DV2:DZ4 EU2:EX4 FA2:FD4 D2:D14 H2:I4 J2:J19 M2:U4 V2:V19 AB2:AG4 AI2:AI4 AP2:AP4 AR2:AR4 AQ2:AQ14" xr:uid="{00000000-0002-0000-0000-000001000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G2:G14 L2:L14 AA2:AA14 AM2:AM4 AH2:AH19 AU2:AU4 AX2:AX4 BA2:BA4 BD2:BD4 BG2:BG4 CB2:CC4 DW2:DW4 EH2:EL4 FA2:FA4 FL2:FR4 D2:D14 H2:I4 J2:J19 M2:U4 V2:V19 AB2:AG4 AI2:AI4 AP2:AP4 AR2:AR4 AQ2:AQ14 BJ2:BJ4 BN2:BO4 BU2:BV4 CE2:CO4 CZ2:CZ4 DD2:DD4 DM2:DM4 DS2:DS4 EA2:EF4 EN2:EN4 ES2:ES4 EV2:EV4 EY2:EY4 FU2:FY4 GA2:GA4 GF2:GF4 GI2:GI4 GM2:GM4 GR2:GR4 GU2:GU4 GX2:GX4 HB2:HB4" xr:uid="{00000000-0002-0000-0000-000001000000}">
       <formula1>"Ya,Tidak"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F2:F4 G15:G19" xr:uid="{00000000-0002-0000-0000-000002000000}">
@@ -4331,178 +4801,175 @@
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AO2:AO4" xr:uid="{00000000-0002-0000-0000-000004000000}">
       <formula1>"1 s.d &lt;10 tahun lalu,10 s.d &lt;15 tahun lalu,15 tahun lalu atau lebih"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BN2:BN4" xr:uid="{00000000-0002-0000-0000-000005000000}">
-      <formula1>"True,False"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="EA2:EA4" xr:uid="{00000000-0002-0000-0000-000006000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="EM2:EM4" xr:uid="{00000000-0002-0000-0000-000006000000}">
       <formula1>"Normal,Abnormal TBC,Abnormal non TBC"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="EB2:EB4" xr:uid="{00000000-0002-0000-0000-000007000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="EO2:EO4" xr:uid="{00000000-0002-0000-0000-000007000000}">
       <formula1>"Riwayat kontak serumah,Riwayat kontak erat,Tidak ada,Tidak diketahui"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="EC2:EC4" xr:uid="{00000000-0002-0000-0000-000008000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="EP2:EP4" xr:uid="{00000000-0002-0000-0000-000008000000}">
       <formula1>"Bakteriologis,Klinis"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="ED2:ED4" xr:uid="{00000000-0002-0000-0000-000009000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="EQ2:EQ4" xr:uid="{00000000-0002-0000-0000-000009000000}">
       <formula1>"TCM,BTA,NPOC,Tidak dilakukan"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="EF2:EF4" xr:uid="{00000000-0002-0000-0000-00000A000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="ET2:ET4" xr:uid="{00000000-0002-0000-0000-00000A000000}">
       <formula1>"Suspek frambusia,Bukan frambusia,Tidak Ada"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="EG2:EG4" xr:uid="{00000000-0002-0000-0000-00000B000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="EU2:EU4" xr:uid="{00000000-0002-0000-0000-00000B000000}">
       <formula1>"Reaktif,Non Reaktif"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="EH2:EH4" xr:uid="{00000000-0002-0000-0000-00000C000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="EW2:EW4" xr:uid="{00000000-0002-0000-0000-00000C000000}">
       <formula1>"Kusta,Bukan kusta,Meragukan,Tidak Ada"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="EI2:EI4" xr:uid="{00000000-0002-0000-0000-00000D000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="EX2:EX4" xr:uid="{00000000-0002-0000-0000-00000D000000}">
       <formula1>"Kusta,Bukan kusta,Meragukan"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="EJ2:EJ4" xr:uid="{00000000-0002-0000-0000-00000E000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="EZ2:EZ4" xr:uid="{00000000-0002-0000-0000-00000E000000}">
       <formula1>"Skabies,Bukan Skabies,Meragukan,Tidak Ada"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="EK2:EK4" xr:uid="{00000000-0002-0000-0000-00000F000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="FB2:FB4" xr:uid="{00000000-0002-0000-0000-00000F000000}">
       <formula1>"Tidak ada serumen impaksi,Ada serumen impaksi"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="EL2:EL4" xr:uid="{00000000-0002-0000-0000-000010000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="FC2:FC4" xr:uid="{00000000-0002-0000-0000-000010000000}">
       <formula1>"Tidak ada infeksi telinga,Ada infeksi telinga"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="EM2:EM4" xr:uid="{00000000-0002-0000-0000-000011000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="FD2:FD4" xr:uid="{00000000-0002-0000-0000-000011000000}">
       <formula1>"Normal,Curiga gangguan pendengaran"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="EN2:EN4" xr:uid="{00000000-0002-0000-0000-000012000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="FE2:FE4" xr:uid="{00000000-0002-0000-0000-000012000000}">
       <formula1>"Normal,Gangguan Pendengaran"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="EO2:EO4" xr:uid="{00000000-0002-0000-0000-000013000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="FF2:FF4" xr:uid="{00000000-0002-0000-0000-000013000000}">
       <formula1>"Normal (visus 6/6 - 6/12),Curiga gangguan penglihatan (visus &lt;6/12)"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="EP2:EP4" xr:uid="{00000000-0002-0000-0000-000014000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="FG2:FG4" xr:uid="{00000000-0002-0000-0000-000014000000}">
       <formula1>"Normal (visus 6/6 - 6/12),Gangguan penglihatan ringan (visus &lt;6/12 - 6/18),Gangguan penglihatan sedang (&lt;6/18 - 6/60),Gangguan penglihatan berat (&lt;6/60 - 3/60),Buta (&lt;3/60)"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="EQ2:EQ4" xr:uid="{00000000-0002-0000-0000-000015000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="FH2:FH4" xr:uid="{00000000-0002-0000-0000-000015000000}">
       <formula1>"Visus membaik,Visus tidak membaik (visus tetap)"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="ER2:ER4" xr:uid="{00000000-0002-0000-0000-000016000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="FI2:FI4" xr:uid="{00000000-0002-0000-0000-000016000000}">
       <formula1>"Kelainan refraksi ringan (0.50 - 3.00 Dioptri),Kelainan refraksi sedang (3.00 - 6.00 Dioptri),Kelainan refraksi berat (&gt;6.00 Dioptri)"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="ES2:ES4" xr:uid="{00000000-0002-0000-0000-000017000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="FJ2:FJ4" xr:uid="{00000000-0002-0000-0000-000017000000}">
       <formula1>"Normal,Curiga kelainan mata"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="ET2:ET4" xr:uid="{00000000-0002-0000-0000-000018000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="FK2:FK4" xr:uid="{00000000-0002-0000-0000-000018000000}">
       <formula1>"Curiga katarak,Normal"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="EY2:EY4" xr:uid="{00000000-0002-0000-0000-000019000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="FS2:FS4" xr:uid="{00000000-0002-0000-0000-000019000000}">
       <formula1>"Iya,Tidak"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="EZ2:EZ4" xr:uid="{00000000-0002-0000-0000-00001A000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="FT2:FT4" xr:uid="{00000000-0002-0000-0000-00001A000000}">
       <formula1>"&lt;20 bungkus per tahun,20-30 bungkus per tahun,&gt;30 bungkus per tahun"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="FL2:FL4" xr:uid="{00000000-0002-0000-0000-00001B000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="GJ2:GJ4" xr:uid="{00000000-0002-0000-0000-00001B000000}">
       <formula1>"HBsAg Non Reaktif,HBsAg Reaktif"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="FM2:FM4" xr:uid="{00000000-0002-0000-0000-00001C000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="GK2:GK4" xr:uid="{00000000-0002-0000-0000-00001C000000}">
       <formula1>"Anti HCV Non Reaktif,Anti HCV Reaktif"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="FN2:FN4" xr:uid="{00000000-0002-0000-0000-00001D000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="GL2:GL4" xr:uid="{00000000-0002-0000-0000-00001D000000}">
       <formula1>"VL HCV RNA Negatif,VL HCV RNA Positif"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="FU2:FU4" xr:uid="{00000000-0002-0000-0000-00001E000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="GV2:GV4" xr:uid="{00000000-0002-0000-0000-00001E000000}">
       <formula1>"Normal,Abnormal"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="FV2:FV4" xr:uid="{00000000-0002-0000-0000-00001F000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="GW2:GW4" xr:uid="{00000000-0002-0000-0000-00001F000000}">
       <formula1>"Normal,Abnormal ST Depresi,Abnormal T Inversi,Abnormal Hipertrofi Ventrikel Kiri,Abnormal Atrial Fibrilasi,Abnormal Q-Patologis,Abnormal ST Elevasi,Abnormal Gambaran Abnormal Lainnya"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="FW2:FW4" xr:uid="{00000000-0002-0000-0000-000020000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="GY2:GY4" xr:uid="{00000000-0002-0000-0000-000020000000}">
       <formula1>"Bersedia,Menolak,Tidak tahu"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="FX2:FX4" xr:uid="{00000000-0002-0000-0000-000021000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="GZ2:GZ4" xr:uid="{00000000-0002-0000-0000-000021000000}">
       <formula1>"Ditemukan benjolan,Tidak ditemukan benjolan"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="FY2:FY4" xr:uid="{00000000-0002-0000-0000-000022000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="HA2:HA4" xr:uid="{00000000-0002-0000-0000-000022000000}">
       <formula1>"Negatif,Positif"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="FZ2:FZ4" xr:uid="{00000000-0002-0000-0000-000023000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="HC2:HC4" xr:uid="{00000000-0002-0000-0000-000023000000}">
       <formula1>"Memiliki diagnosis kanker &gt;5 tahun yang lalu,Memiliki diagnosis kanker &lt;5 tahun yang lalu,Tidak pernah didiagnosis menderita kanker"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="GA2:GA4" xr:uid="{00000000-0002-0000-0000-000024000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="HD2:HD4" xr:uid="{00000000-0002-0000-0000-000024000000}">
       <formula1>"Memiliki keluarga yang terdiagnosis kanker paru,Memiliki keluarga yang terdiagnosis kanker lain,Tidak ada keluarga yang terdiagnosis kanker"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="GB2:GB4" xr:uid="{00000000-0002-0000-0000-000025000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="HE2:HE4" xr:uid="{00000000-0002-0000-0000-000025000000}">
       <formula1>"Perokok aktif (dalam 1 tahun ini masih merokok),Perokok/bekas perokok berhenti &lt;10 tahun lalu,Perokok pasif dari lingkungan rumah/tempat kerja,Tidak pernah merokok"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="GD2:GD4" xr:uid="{00000000-0002-0000-0000-000026000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="HG2:HG4" xr:uid="{00000000-0002-0000-0000-000026000000}">
       <formula1>"Memiliki tempat tinggal berpotensi tinggi,Tidak yakin memiliki tempat tinggal berpotensi tinggi,Tidak memiliki tempat tinggal berpotensi tinggi"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="GE2:GE4" xr:uid="{00000000-0002-0000-0000-000027000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="HH2:HH4" xr:uid="{00000000-0002-0000-0000-000027000000}">
       <formula1>"Memiliki lingkungan dalam rumah yang tidak sehat,Tidak yakin memiliki lingkungan dalam rumah yang tidak sehat,Memiliki lingkungan dalam rumah yang sehat"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="GG2:GG4" xr:uid="{00000000-0002-0000-0000-000028000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="HJ2:HJ4" xr:uid="{00000000-0002-0000-0000-000028000000}">
       <formula1>"Normal,Tidak Normal"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CB2:CB4" xr:uid="{00000000-0002-0000-0000-000029000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CD2:CD4" xr:uid="{00000000-0002-0000-0000-000029000000}">
       <formula1>"Benar semua,Salah satu/Dua,Tidak Tahu"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CJ2:CJ4" xr:uid="{00000000-0002-0000-0000-00002A000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CP2:CP4" xr:uid="{00000000-0002-0000-0000-00002A000000}">
       <formula1>"Tidak terkendali/tak teratur (perlu pencahar),Kadang-kadang tak terkendali (1 x / minggu),Terkendali teratur"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CK2:CK4" xr:uid="{00000000-0002-0000-0000-00002B000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CQ2:CQ4" xr:uid="{00000000-0002-0000-0000-00002B000000}">
       <formula1>"Tak terkendali atau pakai kateter,Kadang-kadang tak terkendali (hanya 1 x / 24 jam),Mandiri"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CL2:CL4" xr:uid="{00000000-0002-0000-0000-00002C000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CR2:CR4" xr:uid="{00000000-0002-0000-0000-00002C000000}">
       <formula1>"Mandiri,Butuh pertolongan orang lain"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CM2:CM4" xr:uid="{00000000-0002-0000-0000-00002D000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CS2:CS4" xr:uid="{00000000-0002-0000-0000-00002D000000}">
       <formula1>"Tergantung pertolongan orang lain,Perlu pertolongan pada beberapa kegiatan tetapi dapat mengerjakan sendiri beberapa kegiatan yang lain,Mandiri"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CN2:CN4" xr:uid="{00000000-0002-0000-0000-00002E000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CT2:CT4" xr:uid="{00000000-0002-0000-0000-00002E000000}">
       <formula1>"Tidak mampu,Perlu ditolong memotong makanan,Mandiri"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CO2:CO4" xr:uid="{00000000-0002-0000-0000-00002F000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CU2:CU4" xr:uid="{00000000-0002-0000-0000-00002F000000}">
       <formula1>"Tidak mampu,Perlu banyak bantuan untuk bias duduk (2 orang),Bantuan minimal 1 orang,Mandiri"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CP2:CP4" xr:uid="{00000000-0002-0000-0000-000030000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CV2:CV4" xr:uid="{00000000-0002-0000-0000-000030000000}">
       <formula1>"Tidak mampu,Bisa (pindah) dengan kursi roda,Bantuan minimal 1 orang,Mandiri"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CQ2:CQ4" xr:uid="{00000000-0002-0000-0000-000031000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CW2:CW4" xr:uid="{00000000-0002-0000-0000-000031000000}">
       <formula1>"Tergantung orang lain,Sebagian dibantu (misalnya: mengancing baju),Mandiri"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CR2:CR4" xr:uid="{00000000-0002-0000-0000-000032000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CX2:CX4" xr:uid="{00000000-0002-0000-0000-000032000000}">
       <formula1>"Tidak mampu,Butuh pertolongan,Mandiri"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CS2:CS4" xr:uid="{00000000-0002-0000-0000-000033000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CY2:CY4" xr:uid="{00000000-0002-0000-0000-000033000000}">
       <formula1>"Tergantung orang lain,Mandiri"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CT2:CT4" xr:uid="{00000000-0002-0000-0000-000034000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DA2:DA4" xr:uid="{00000000-0002-0000-0000-000034000000}">
       <formula1>"SUDAH DITANYAKAN"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CU2:CU4" xr:uid="{00000000-0002-0000-0000-000035000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DB2:DB4" xr:uid="{00000000-0002-0000-0000-000035000000}">
       <formula1>"Benar,Salah"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CV2:CV4" xr:uid="{00000000-0002-0000-0000-000036000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DC2:DC4" xr:uid="{00000000-0002-0000-0000-000036000000}">
       <formula1>"Benar 1 kata,Benar 2 Kata,Benar semua kata,Tidak dapat mengingat/mengulang kata"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DE2:DF4" xr:uid="{00000000-0002-0000-0000-000037000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DN2:DO4" xr:uid="{00000000-0002-0000-0000-000037000000}">
       <formula1>"Bertahan 10 detik,Tidak bertahan 10 detik,Tidak dilakukan"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DG2:DG4" xr:uid="{00000000-0002-0000-0000-000038000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DP2:DP4" xr:uid="{00000000-0002-0000-0000-000038000000}">
       <formula1>"Bertahan 10 detik,Bertahan 3 - 9.99 detik,Bertahan &lt; 3 detik"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DJ2:DJ4" xr:uid="{00000000-0002-0000-0000-000039000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DT2:DT4" xr:uid="{00000000-0002-0000-0000-000039000000}">
       <formula1>"Nafsu Makan Yang Sangat Berkurang,Nafsu Makan Sedikit Berkurang,Nafsu Makan Biasa saja"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DK2:DK4" xr:uid="{00000000-0002-0000-0000-00003A000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DU2:DU4" xr:uid="{00000000-0002-0000-0000-00003A000000}">
       <formula1>"Penurunan BB &gt; 3 Kg,Tidak Tahu,Penurunan BB antara 1 - 3 Kg"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DN2:DN4" xr:uid="{00000000-0002-0000-0000-00003B000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DX2:DX4" xr:uid="{00000000-0002-0000-0000-00003B000000}">
       <formula1>"Dementia atau depresi berat,Demensia/kepikunan ringan,Tidak ada masalah psikologis"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DO2:DO4" xr:uid="{00000000-0002-0000-0000-00003C000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DY2:DY4" xr:uid="{00000000-0002-0000-0000-00003C000000}">
       <formula1>"IMT &lt;19,IMT 19 - &lt;21,IMT 21 - &lt;23,IMT &gt;= 23"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DP2:DP4" xr:uid="{00000000-0002-0000-0000-00003D000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DZ2:DZ4" xr:uid="{00000000-0002-0000-0000-00003D000000}">
       <formula1>"&lt;31 cm,&gt;= 31 cm"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="GF2:GF4 AJ2:AJ4 CW2:DD4 DH2:DI4 DL2:DL4 DU2:DU4 EE2:EE4 GC2:GC4 K2:K4 L15:L19" xr:uid="{00000000-0002-0000-0000-00003E000000}"/>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="HI2:HI4 AJ2:AJ4 L15:L19 DE2:DL4 DV2:DV4 EG2:EG4 DQ2:DR4 HF2:HF4 K2:K4 ER2:ER4" xr:uid="{00000000-0002-0000-0000-00003E000000}"/>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AQ15:AQ19" xr:uid="{D833678B-E8C5-404F-B459-69AFD1570727}">
       <formula1>"Pernah imunisasi tetanus minimal dua kali,Pernah imunisasi tetanus satu kali,Pernah imunisasi tetanus tetapi tidak ingat berapa kali,Tidak tahu atau tidak ingat"</formula1>
     </dataValidation>

</xml_diff>

<commit_message>
fix: stage 8 fixing skrining-filtering, doing modification for excel dewasa
</commit_message>
<xml_diff>
--- a/dataset/lansia.xlsx
+++ b/dataset/lansia.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/macbokprom12021/PycharmProjects/CKG-Helper/dataset/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E1CCC735-F43A-9D4B-B979-9FBFEDDA1110}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA1447AF-7A8E-2240-BDD7-9D3311B522ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3300" yWindow="-21000" windowWidth="38400" windowHeight="21000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="22500" yWindow="-21000" windowWidth="19200" windowHeight="21000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -1864,7 +1864,7 @@
     <col min="3" max="3" width="11.5" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="25.83203125" style="1" customWidth="1"/>
     <col min="5" max="5" width="16.6640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="10.83203125" customWidth="1"/>
+    <col min="6" max="6" width="13.1640625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="18.5" style="1" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="19.33203125" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="8.1640625" bestFit="1" customWidth="1"/>
@@ -1919,7 +1919,7 @@
     <col min="61" max="61" width="19.33203125" bestFit="1" customWidth="1"/>
     <col min="62" max="62" width="14.83203125" style="3" bestFit="1" customWidth="1"/>
     <col min="63" max="65" width="14.33203125" customWidth="1"/>
-    <col min="66" max="66" width="17.1640625" style="3" bestFit="1" customWidth="1"/>
+    <col min="66" max="66" width="24.33203125" style="3" bestFit="1" customWidth="1"/>
     <col min="67" max="67" width="14.83203125" bestFit="1" customWidth="1"/>
     <col min="68" max="68" width="18.5" bestFit="1" customWidth="1"/>
     <col min="69" max="69" width="18" bestFit="1" customWidth="1"/>

</xml_diff>

<commit_message>
feat: update dataset files for dewasa and lansia; modify screening function for cancer risk
</commit_message>
<xml_diff>
--- a/dataset/lansia.xlsx
+++ b/dataset/lansia.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/macbokprom12021/PycharmProjects/CKG-Helper/dataset/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E02BA612-D8FF-0146-8427-90F8691A1A65}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E15873A-D510-5C44-A596-EEC29857366B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="780" windowWidth="36000" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -543,7 +543,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="525" uniqueCount="302">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="525" uniqueCount="303">
   <si>
     <t>batas_awal</t>
   </si>
@@ -1449,6 +1449,9 @@
   </si>
   <si>
     <t>3512082302650001</t>
+  </si>
+  <si>
+    <t>skrining_kanker_usus_mandiri</t>
   </si>
 </sst>
 </file>
@@ -2087,7 +2090,7 @@
         <v>6</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>7</v>
+        <v>302</v>
       </c>
       <c r="K1" t="s">
         <v>8</v>

</xml_diff>